<commit_message>
📊 Dashboard aggiornata 23/04/2026 20:48
</commit_message>
<xml_diff>
--- a/docs/sarada_dati.xlsx
+++ b/docs/sarada_dati.xlsx
@@ -961,7 +961,7 @@
         <v>78.93103851222787</v>
       </c>
       <c r="J6" t="n">
-        <v>47.45383708182479</v>
+        <v>47.80188401830082</v>
       </c>
       <c r="K6" t="n">
         <v>0.9725210130735034</v>
@@ -979,13 +979,13 @@
         <v>0.3354735513319747</v>
       </c>
       <c r="P6" t="n">
-        <v>103.0021862935916</v>
+        <v>102.7255412489931</v>
       </c>
       <c r="Q6" t="n">
-        <v>3.00218629359158</v>
+        <v>2.725541248993103</v>
       </c>
       <c r="R6" t="n">
-        <v>-47.70052328027374</v>
+        <v>-61.31193457658048</v>
       </c>
       <c r="S6" t="n">
         <v>16.61777908527611</v>
@@ -1018,7 +1018,7 @@
       </c>
       <c r="Z6" t="inlineStr">
         <is>
-          <t>EMA e SMA allineate al rialzo — struttura bullish solida; trend molto direzionale (ADX 47); RSI ipercomprato (79) — attenzione estensione; breakout massimi 50g — rottura resistenza rilevante; candela di inversione bullish (engulfing); vicino alla resistenza dei 20g (79.09); favorito dal quadrante macro (Stagflazione)</t>
+          <t>EMA e SMA allineate al rialzo — struttura bullish solida; trend molto direzionale (ADX 48); RSI ipercomprato (79) — attenzione estensione; breakout massimi 50g — rottura resistenza rilevante; candela di inversione bullish (engulfing); vicino alla resistenza dei 20g (79.09); favorito dal quadrante macro (Stagflazione)</t>
         </is>
       </c>
     </row>
@@ -2019,7 +2019,7 @@
         <v>73.40000000000001</v>
       </c>
       <c r="X17" t="n">
-        <v>79.90000000000001</v>
+        <v>80</v>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
@@ -2487,7 +2487,7 @@
         <v>72.59999999999999</v>
       </c>
       <c r="X22" t="n">
-        <v>78.90000000000001</v>
+        <v>79</v>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
@@ -3441,52 +3441,52 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>6.013999938964844</v>
+        <v>6.021999835968018</v>
       </c>
       <c r="E33" t="n">
-        <v>-1.732025303535689</v>
+        <v>-1.601308029797643</v>
       </c>
       <c r="F33" t="n">
-        <v>-0.8654124509633543</v>
+        <v>-0.7335423981045031</v>
       </c>
       <c r="G33" t="n">
-        <v>10.90824879458472</v>
+        <v>11.05578031705954</v>
       </c>
       <c r="H33" t="n">
-        <v>1.742516798406624</v>
+        <v>1.877855950965879</v>
       </c>
       <c r="I33" t="n">
-        <v>58.79787118060198</v>
+        <v>59.26759223190381</v>
       </c>
       <c r="J33" t="n">
         <v>41.18504839863726</v>
       </c>
       <c r="K33" t="n">
-        <v>0.7082016218621492</v>
+        <v>0.7155185804306334</v>
       </c>
       <c r="L33" t="n">
-        <v>5.887081324860246</v>
+        <v>5.88784321981293</v>
       </c>
       <c r="M33" t="n">
-        <v>5.784705999211812</v>
+        <v>5.785019720662916</v>
       </c>
       <c r="N33" t="n">
-        <v>5.390744538828134</v>
+        <v>5.390824139793339</v>
       </c>
       <c r="O33" t="n">
-        <v>0.0307298669721969</v>
+        <v>0.0312404017097225</v>
       </c>
       <c r="P33" t="n">
-        <v>77.73178703382069</v>
+        <v>79.0562730918622</v>
       </c>
       <c r="Q33" t="n">
-        <v>-22.2682129661793</v>
+        <v>-20.94372690813781</v>
       </c>
       <c r="R33" t="n">
-        <v>72.99061488786609</v>
+        <v>73.67936242612009</v>
       </c>
       <c r="S33" t="n">
-        <v>8.771932548022443</v>
+        <v>8.916622316238509</v>
       </c>
       <c r="T33" t="inlineStr">
         <is>
@@ -3504,10 +3504,10 @@
         </is>
       </c>
       <c r="W33" t="n">
-        <v>70.59999999999999</v>
+        <v>70.7</v>
       </c>
       <c r="X33" t="n">
-        <v>77.09999999999999</v>
+        <v>77.2</v>
       </c>
       <c r="Y33" t="inlineStr">
         <is>
@@ -3523,66 +3523,66 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>AAPL</t>
+          <t>BRENT</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Apple</t>
+          <t>Brent Crude</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Azioni USA</t>
+          <t>Commodities</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>273.4299926757812</v>
+        <v>106.3099975585938</v>
       </c>
       <c r="E34" t="n">
-        <v>0.09517122497622044</v>
+        <v>4.317528935699877</v>
       </c>
       <c r="F34" t="n">
-        <v>3.807896359799701</v>
+        <v>6.962469274012317</v>
       </c>
       <c r="G34" t="n">
-        <v>8.659193029321388</v>
+        <v>1.741793216607279</v>
       </c>
       <c r="H34" t="n">
-        <v>10.23625224838607</v>
+        <v>61.36915906303897</v>
       </c>
       <c r="I34" t="n">
-        <v>62.94078408540657</v>
+        <v>56.68896901546076</v>
       </c>
       <c r="J34" t="n">
-        <v>12.76518184945696</v>
+        <v>24.05054899031809</v>
       </c>
       <c r="K34" t="n">
-        <v>0.9085562672060516</v>
+        <v>0.6258097700542922</v>
       </c>
       <c r="L34" t="n">
-        <v>263.3237552564631</v>
+        <v>99.66149848739461</v>
       </c>
       <c r="M34" t="n">
-        <v>261.302373643884</v>
+        <v>93.1982345740402</v>
       </c>
       <c r="N34" t="n">
-        <v>252.9600203919621</v>
+        <v>77.34060082017123</v>
       </c>
       <c r="O34" t="n">
-        <v>1.812859936747026</v>
+        <v>-0.4879041402273356</v>
       </c>
       <c r="P34" t="n">
-        <v>92.21816775741412</v>
+        <v>78.44123694993444</v>
       </c>
       <c r="Q34" t="n">
-        <v>-7.781832242585886</v>
+        <v>-21.55876305006557</v>
       </c>
       <c r="R34" t="n">
-        <v>131.0299973669376</v>
+        <v>26.36445346781798</v>
       </c>
       <c r="S34" t="n">
-        <v>8.237668419295252</v>
+        <v>4.001170308206037</v>
       </c>
       <c r="T34" t="inlineStr">
         <is>
@@ -3590,16 +3590,12 @@
         </is>
       </c>
       <c r="U34" t="inlineStr"/>
-      <c r="V34" t="inlineStr">
-        <is>
-          <t>Double Top, Double Bottom</t>
-        </is>
-      </c>
+      <c r="V34" t="inlineStr"/>
       <c r="W34" t="n">
         <v>70.5</v>
       </c>
       <c r="X34" t="n">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="Y34" t="inlineStr">
         <is>
@@ -3608,73 +3604,73 @@
       </c>
       <c r="Z34" t="inlineStr">
         <is>
-          <t>EMA e SMA allineate al rialzo — struttura bullish solida; mercato laterale — ATR basso (ADX 13); RSI in forza (63) — momentum positivo; pattern: Double Bottom; vicino alla resistenza dei 20g (275.77); in zona Fib Fib 23.6 — livello strutturale</t>
+          <t>EMA e SMA allineate al rialzo — struttura bullish solida; trend in sviluppo (ADX 24); favorito dal quadrante macro (Stagflazione)</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>BRENT</t>
+          <t>AAPL</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Brent Crude</t>
+          <t>Apple</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Commodities</t>
+          <t>Azioni USA</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>105.9499969482422</v>
+        <v>273.4299926757812</v>
       </c>
       <c r="E35" t="n">
-        <v>3.964275479302048</v>
+        <v>0.09517122497622044</v>
       </c>
       <c r="F35" t="n">
-        <v>6.600259179875767</v>
+        <v>3.807896359799701</v>
       </c>
       <c r="G35" t="n">
-        <v>1.397262048350467</v>
+        <v>8.659193029321388</v>
       </c>
       <c r="H35" t="n">
-        <v>60.82271002636588</v>
+        <v>10.23625224838607</v>
       </c>
       <c r="I35" t="n">
-        <v>56.43550392523061</v>
+        <v>62.94078408540657</v>
       </c>
       <c r="J35" t="n">
-        <v>24.05054899031809</v>
+        <v>12.76518184945696</v>
       </c>
       <c r="K35" t="n">
-        <v>0.6149626116446049</v>
+        <v>0.9085562672060516</v>
       </c>
       <c r="L35" t="n">
-        <v>99.62721271498017</v>
+        <v>263.3237552564631</v>
       </c>
       <c r="M35" t="n">
-        <v>93.18411690304602</v>
+        <v>261.302373643884</v>
       </c>
       <c r="N35" t="n">
-        <v>77.33701872454586</v>
+        <v>252.9600203919621</v>
       </c>
       <c r="O35" t="n">
-        <v>-0.5108785381529128</v>
+        <v>1.812859936747026</v>
       </c>
       <c r="P35" t="n">
-        <v>77.04534475306825</v>
+        <v>92.21816775741412</v>
       </c>
       <c r="Q35" t="n">
-        <v>-22.95465524693175</v>
+        <v>-7.781832242585886</v>
       </c>
       <c r="R35" t="n">
-        <v>25.36188607292824</v>
+        <v>131.0299973669376</v>
       </c>
       <c r="S35" t="n">
-        <v>3.6489881461512</v>
+        <v>8.237668419295252</v>
       </c>
       <c r="T35" t="inlineStr">
         <is>
@@ -3682,12 +3678,16 @@
         </is>
       </c>
       <c r="U35" t="inlineStr"/>
-      <c r="V35" t="inlineStr"/>
+      <c r="V35" t="inlineStr">
+        <is>
+          <t>Double Top, Double Bottom</t>
+        </is>
+      </c>
       <c r="W35" t="n">
-        <v>70.3</v>
+        <v>70.5</v>
       </c>
       <c r="X35" t="n">
-        <v>77.90000000000001</v>
+        <v>70</v>
       </c>
       <c r="Y35" t="inlineStr">
         <is>
@@ -3696,7 +3696,7 @@
       </c>
       <c r="Z35" t="inlineStr">
         <is>
-          <t>EMA e SMA allineate al rialzo — struttura bullish solida; trend in sviluppo (ADX 24); favorito dal quadrante macro (Stagflazione)</t>
+          <t>EMA e SMA allineate al rialzo — struttura bullish solida; mercato laterale — ATR basso (ADX 13); RSI in forza (63) — momentum positivo; pattern: Double Bottom; vicino alla resistenza dei 20g (275.77); in zona Fib Fib 23.6 — livello strutturale</t>
         </is>
       </c>
     </row>
@@ -5489,52 +5489,52 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>96.58000183105469</v>
+        <v>96.87999725341797</v>
       </c>
       <c r="E55" t="n">
-        <v>3.894151013590852</v>
+        <v>4.21686554168661</v>
       </c>
       <c r="F55" t="n">
-        <v>1.995986208594691</v>
+        <v>2.312804684282144</v>
       </c>
       <c r="G55" t="n">
-        <v>4.580404360395263</v>
+        <v>4.905250518836013</v>
       </c>
       <c r="H55" t="n">
-        <v>58.14639317779462</v>
+        <v>58.63762524568787</v>
       </c>
       <c r="I55" t="n">
-        <v>53.11916667753718</v>
+        <v>53.3614862947192</v>
       </c>
       <c r="J55" t="n">
         <v>18.80673059102289</v>
       </c>
       <c r="K55" t="n">
-        <v>0.4606976379621026</v>
+        <v>0.4699768105232864</v>
       </c>
       <c r="L55" t="n">
-        <v>94.2947226342537</v>
+        <v>94.32329362685974</v>
       </c>
       <c r="M55" t="n">
-        <v>87.77960142343555</v>
+        <v>87.79136594980274</v>
       </c>
       <c r="N55" t="n">
-        <v>72.76215008288928</v>
+        <v>72.76513511196752</v>
       </c>
       <c r="O55" t="n">
-        <v>-1.409990006764334</v>
+        <v>-1.390844999753115</v>
       </c>
       <c r="P55" t="n">
-        <v>43.21555005218325</v>
+        <v>44.0248174512471</v>
       </c>
       <c r="Q55" t="n">
-        <v>-56.78444994781675</v>
+        <v>-55.9751825487529</v>
       </c>
       <c r="R55" t="n">
-        <v>-19.2241759980246</v>
+        <v>-18.33464252584803</v>
       </c>
       <c r="S55" t="n">
-        <v>6.930914700378588</v>
+        <v>7.263061980468177</v>
       </c>
       <c r="T55" t="inlineStr">
         <is>
@@ -5548,10 +5548,10 @@
         </is>
       </c>
       <c r="W55" t="n">
-        <v>64.2</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="X55" t="n">
-        <v>79.2</v>
+        <v>79.3</v>
       </c>
       <c r="Y55" t="inlineStr">
         <is>
@@ -5581,52 +5581,52 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>159.7010040283203</v>
+        <v>159.7039947509766</v>
       </c>
       <c r="E56" t="n">
-        <v>0.2058083410781064</v>
+        <v>0.2076848964768452</v>
       </c>
       <c r="F56" t="n">
-        <v>0.5616799166233255</v>
+        <v>0.5635631364334204</v>
       </c>
       <c r="G56" t="n">
-        <v>0.6193385089402703</v>
+        <v>0.621222808523525</v>
       </c>
       <c r="H56" t="n">
-        <v>3.476185429248368</v>
+        <v>3.478123229038843</v>
       </c>
       <c r="I56" t="n">
-        <v>56.68743323980835</v>
+        <v>56.70762823848671</v>
       </c>
       <c r="J56" t="n">
         <v>18.64026120965874</v>
       </c>
       <c r="K56" t="n">
-        <v>0.7262490148743661</v>
+        <v>0.7276460572565669</v>
       </c>
       <c r="L56" t="n">
-        <v>159.0798210525012</v>
+        <v>159.0801058832303</v>
       </c>
       <c r="M56" t="n">
-        <v>158.2490304618226</v>
+        <v>158.249147745064</v>
       </c>
       <c r="N56" t="n">
-        <v>154.648640803066</v>
+        <v>154.6486705615004</v>
       </c>
       <c r="O56" t="n">
-        <v>-0.0602013453565261</v>
+        <v>-0.06001048442347756</v>
       </c>
       <c r="P56" t="n">
-        <v>86.93319278906296</v>
+        <v>87.05765066705612</v>
       </c>
       <c r="Q56" t="n">
-        <v>-13.06680721093705</v>
+        <v>-12.94234933294387</v>
       </c>
       <c r="R56" t="n">
-        <v>58.16167285539258</v>
+        <v>58.29725658334412</v>
       </c>
       <c r="S56" t="n">
-        <v>0.1988915684335346</v>
+        <v>0.2007679943017981</v>
       </c>
       <c r="T56" t="inlineStr">
         <is>
@@ -5769,52 +5769,52 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>1.346545696258545</v>
+        <v>1.346590995788574</v>
       </c>
       <c r="E58" t="n">
-        <v>-0.3273435791041224</v>
+        <v>-0.3239904626780032</v>
       </c>
       <c r="F58" t="n">
-        <v>-0.7974220568637724</v>
+        <v>-0.7940847544825713</v>
       </c>
       <c r="G58" t="n">
-        <v>0.3661311208964957</v>
+        <v>0.3695075667039083</v>
       </c>
       <c r="H58" t="n">
-        <v>-1.550000117662609</v>
+        <v>-1.546688132975838</v>
       </c>
       <c r="I58" t="n">
-        <v>52.77925200733311</v>
+        <v>52.81124838933329</v>
       </c>
       <c r="J58" t="n">
         <v>35.816263122645</v>
       </c>
       <c r="K58" t="n">
-        <v>0.644800549526221</v>
+        <v>0.6455824464971287</v>
       </c>
       <c r="L58" t="n">
-        <v>1.343773275324439</v>
+        <v>1.343777589565394</v>
       </c>
       <c r="M58" t="n">
-        <v>1.342366572283661</v>
+        <v>1.342368348735819</v>
       </c>
       <c r="N58" t="n">
-        <v>1.337413515777838</v>
+        <v>1.33741396651943</v>
       </c>
       <c r="O58" t="n">
-        <v>0.001537424886796145</v>
+        <v>0.001540315796974589</v>
       </c>
       <c r="P58" t="n">
-        <v>67.48436608400974</v>
+        <v>67.59499714688312</v>
       </c>
       <c r="Q58" t="n">
-        <v>-32.51563391599026</v>
+        <v>-32.40500285311688</v>
       </c>
       <c r="R58" t="n">
-        <v>46.70444653115718</v>
+        <v>46.78151109764871</v>
       </c>
       <c r="S58" t="n">
-        <v>0.7620189434283997</v>
+        <v>0.7654087074116189</v>
       </c>
       <c r="T58" t="inlineStr">
         <is>
@@ -6225,52 +6225,52 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>77984</v>
+        <v>77989.5390625</v>
       </c>
       <c r="E63" t="n">
-        <v>-0.2801699141368408</v>
+        <v>-0.2730869949311709</v>
       </c>
       <c r="F63" t="n">
-        <v>2.981515956692249</v>
+        <v>2.988830547547172</v>
       </c>
       <c r="G63" t="n">
-        <v>16.58793069677333</v>
+        <v>16.59621172666248</v>
       </c>
       <c r="H63" t="n">
-        <v>14.67320964987398</v>
+        <v>14.68135468058957</v>
       </c>
       <c r="I63" t="n">
-        <v>64.53223810986381</v>
+        <v>64.55292043013765</v>
       </c>
       <c r="J63" t="n">
         <v>45.68130131762761</v>
       </c>
       <c r="K63" t="n">
-        <v>0.8625119937210681</v>
+        <v>0.8628898686701251</v>
       </c>
       <c r="L63" t="n">
-        <v>74099.02758852454</v>
+        <v>74099.55511828644</v>
       </c>
       <c r="M63" t="n">
-        <v>72568.45906928772</v>
+        <v>72568.67628742498</v>
       </c>
       <c r="N63" t="n">
-        <v>82606.20731679273</v>
+        <v>82606.26243184248</v>
       </c>
       <c r="O63" t="n">
-        <v>416.0353225250419</v>
+        <v>416.3888125535489</v>
       </c>
       <c r="P63" t="n">
-        <v>83.37707434338166</v>
+        <v>83.43911977744153</v>
       </c>
       <c r="Q63" t="n">
-        <v>-16.62292565661834</v>
+        <v>-16.56088022255846</v>
       </c>
       <c r="R63" t="n">
-        <v>84.71425120825873</v>
+        <v>84.74492734134724</v>
       </c>
       <c r="S63" t="n">
-        <v>16.51384510260727</v>
+        <v>16.52212087033062</v>
       </c>
       <c r="T63" t="inlineStr">
         <is>
@@ -7437,52 +7437,52 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>4705.39990234375</v>
+        <v>4705.2001953125</v>
       </c>
       <c r="E76" t="n">
-        <v>-0.5726380909931272</v>
+        <v>-0.5768579965662934</v>
       </c>
       <c r="F76" t="n">
-        <v>-1.671751611831196</v>
+        <v>-1.675924868723522</v>
       </c>
       <c r="G76" t="n">
-        <v>6.957927653171025</v>
+        <v>6.953388134608596</v>
       </c>
       <c r="H76" t="n">
-        <v>-5.441909134279599</v>
+        <v>-5.445922377786927</v>
       </c>
       <c r="I76" t="n">
-        <v>46.61769538470455</v>
+        <v>46.60748835581663</v>
       </c>
       <c r="J76" t="n">
         <v>31.15818978795262</v>
       </c>
       <c r="K76" t="n">
-        <v>0.5063080781855865</v>
+        <v>0.5059182473123295</v>
       </c>
       <c r="L76" t="n">
-        <v>4751.019662703022</v>
+        <v>4751.00064298576</v>
       </c>
       <c r="M76" t="n">
-        <v>4772.904303738087</v>
+        <v>4772.896472089803</v>
       </c>
       <c r="N76" t="n">
-        <v>4293.50755042564</v>
+        <v>4293.505563291002</v>
       </c>
       <c r="O76" t="n">
-        <v>9.74483151928996</v>
+        <v>9.732086683107422</v>
       </c>
       <c r="P76" t="n">
-        <v>36.54890096802978</v>
+        <v>36.47620097194029</v>
       </c>
       <c r="Q76" t="n">
-        <v>-63.45109903197022</v>
+        <v>-63.52379902805971</v>
       </c>
       <c r="R76" t="n">
-        <v>9.001301241289806</v>
+        <v>8.974010534457566</v>
       </c>
       <c r="S76" t="n">
-        <v>3.419932839593098</v>
+        <v>3.415543480943861</v>
       </c>
       <c r="T76" t="inlineStr">
         <is>
@@ -7529,69 +7529,73 @@
         </is>
       </c>
       <c r="D77" t="n">
-        <v>2326.219970703125</v>
+        <v>2328.590087890625</v>
       </c>
       <c r="E77" t="n">
-        <v>-2.098750603264932</v>
+        <v>-1.999001896437869</v>
       </c>
       <c r="F77" t="n">
-        <v>-1.058253967660594</v>
+        <v>-0.9574451293796526</v>
       </c>
       <c r="G77" t="n">
-        <v>13.09609836023544</v>
+        <v>13.21132865227088</v>
       </c>
       <c r="H77" t="n">
-        <v>18.14086233482954</v>
+        <v>18.26123258867154</v>
       </c>
       <c r="I77" t="n">
-        <v>55.3902225703355</v>
+        <v>55.56581842199144</v>
       </c>
       <c r="J77" t="n">
         <v>47.76939751961269</v>
       </c>
       <c r="K77" t="n">
-        <v>0.6387888171610275</v>
+        <v>0.6442997088515746</v>
       </c>
       <c r="L77" t="n">
-        <v>2276.814307480008</v>
+        <v>2277.040032926436</v>
       </c>
       <c r="M77" t="n">
-        <v>2226.010301975022</v>
+        <v>2226.103247747081</v>
       </c>
       <c r="N77" t="n">
-        <v>2636.91315048008</v>
+        <v>2636.936733735677</v>
       </c>
       <c r="O77" t="n">
-        <v>0.1741131713582789</v>
+        <v>0.3253685132383737</v>
       </c>
       <c r="P77" t="n">
-        <v>51.9641954860109</v>
+        <v>52.78584408143022</v>
       </c>
       <c r="Q77" t="n">
-        <v>-48.0358045139891</v>
+        <v>-47.21415591856978</v>
       </c>
       <c r="R77" t="n">
-        <v>36.9860126584938</v>
+        <v>37.3943534897409</v>
       </c>
       <c r="S77" t="n">
-        <v>13.28706906206951</v>
+        <v>13.40249392854265</v>
       </c>
       <c r="T77" t="inlineStr">
         <is>
           <t>Range</t>
         </is>
       </c>
-      <c r="U77" t="inlineStr"/>
+      <c r="U77" t="inlineStr">
+        <is>
+          <t>Bearish Harami</t>
+        </is>
+      </c>
       <c r="V77" t="inlineStr">
         <is>
           <t>Bull Flag / Consolidation</t>
         </is>
       </c>
       <c r="W77" t="n">
-        <v>56</v>
+        <v>56.2</v>
       </c>
       <c r="X77" t="n">
-        <v>71.90000000000001</v>
+        <v>69.3</v>
       </c>
       <c r="Y77" t="inlineStr">
         <is>
@@ -7600,90 +7604,94 @@
       </c>
       <c r="Z77" t="inlineStr">
         <is>
-          <t>trend molto direzionale (ADX 48); pattern: Bull Flag / Consolidation; penalizzato dal quadrante macro (Stagflazione)</t>
+          <t>trend molto direzionale (ADX 48); pattern: Bull Flag / Consolidation; segnale candlestick: Bearish Harami; penalizzato dal quadrante macro (Stagflazione)</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>MOO</t>
+          <t>XRP</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Agribusiness</t>
+          <t>XRP</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Settoriali</t>
+          <t>Crypto</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>83.12999725341797</v>
+        <v>1.437199950218201</v>
       </c>
       <c r="E78" t="n">
-        <v>0.02406045351890373</v>
+        <v>0.5015278497465525</v>
       </c>
       <c r="F78" t="n">
-        <v>-0.7995295631743837</v>
+        <v>0.1754384069853732</v>
       </c>
       <c r="G78" t="n">
-        <v>1.119083054605063</v>
+        <v>8.986861486485886</v>
       </c>
       <c r="H78" t="n">
-        <v>4.76370365719625</v>
+        <v>0.5446928702135923</v>
       </c>
       <c r="I78" t="n">
-        <v>45.35554130370132</v>
+        <v>56.80667278161111</v>
       </c>
       <c r="J78" t="n">
-        <v>27.39858677518637</v>
+        <v>30.7101634397846</v>
       </c>
       <c r="K78" t="n">
-        <v>0.2448120791372954</v>
+        <v>0.7702375177853598</v>
       </c>
       <c r="L78" t="n">
-        <v>83.8359717804021</v>
+        <v>1.400243648871959</v>
       </c>
       <c r="M78" t="n">
-        <v>83.00361606280865</v>
+        <v>1.413822040899541</v>
       </c>
       <c r="N78" t="n">
-        <v>77.86687997661033</v>
+        <v>1.7790984048738</v>
       </c>
       <c r="O78" t="n">
-        <v>-0.2484960445130959</v>
+        <v>0.007809096669945139</v>
       </c>
       <c r="P78" t="n">
-        <v>12.88658172093755</v>
+        <v>62.03269702050819</v>
       </c>
       <c r="Q78" t="n">
-        <v>-87.11341827906246</v>
+        <v>-37.96730297949181</v>
       </c>
       <c r="R78" t="n">
-        <v>-69.47277854259958</v>
+        <v>70.80742335627504</v>
       </c>
       <c r="S78" t="n">
-        <v>0.2290750017109655</v>
+        <v>9.051699146254698</v>
       </c>
       <c r="T78" t="inlineStr">
         <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="U78" t="inlineStr"/>
+          <t>Range</t>
+        </is>
+      </c>
+      <c r="U78" t="inlineStr">
+        <is>
+          <t>Hammer, Bullish Engulfing, Piercing Pattern</t>
+        </is>
+      </c>
       <c r="V78" t="inlineStr">
         <is>
-          <t>Double Top</t>
+          <t>Double Bottom</t>
         </is>
       </c>
       <c r="W78" t="n">
         <v>55.9</v>
       </c>
       <c r="X78" t="n">
-        <v>68.90000000000001</v>
+        <v>74.90000000000001</v>
       </c>
       <c r="Y78" t="inlineStr">
         <is>
@@ -7692,94 +7700,90 @@
       </c>
       <c r="Z78" t="inlineStr">
         <is>
-          <t>trend in sviluppo (ADX 27); pattern: Double Top; sul supporto dei 20g (82.41); in zona Fib Fib 23.6 — livello strutturale; favorito dal quadrante macro (Stagflazione)</t>
+          <t>trend molto direzionale (ADX 31); pattern: Double Bottom; hammer — segnale di rimbalzo da supporto; penalizzato dal quadrante macro (Stagflazione)</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>XRP</t>
+          <t>MOO</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>XRP</t>
+          <t>Agribusiness</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Crypto</t>
+          <t>Settoriali</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>1.435400009155273</v>
+        <v>83.12999725341797</v>
       </c>
       <c r="E79" t="n">
-        <v>0.375660306516945</v>
+        <v>0.02406045351890373</v>
       </c>
       <c r="F79" t="n">
-        <v>0.04997925632361788</v>
+        <v>-0.7995295631743837</v>
       </c>
       <c r="G79" t="n">
-        <v>8.8503669595557</v>
+        <v>1.119083054605063</v>
       </c>
       <c r="H79" t="n">
-        <v>0.4187712673572763</v>
+        <v>4.76370365719625</v>
       </c>
       <c r="I79" t="n">
-        <v>56.5667712227112</v>
+        <v>45.35554130370132</v>
       </c>
       <c r="J79" t="n">
-        <v>30.7101634397846</v>
+        <v>27.39858677518637</v>
       </c>
       <c r="K79" t="n">
-        <v>0.7620851862799014</v>
+        <v>0.2448120791372954</v>
       </c>
       <c r="L79" t="n">
-        <v>1.400072225913585</v>
+        <v>83.8359717804021</v>
       </c>
       <c r="M79" t="n">
-        <v>1.413751454975504</v>
+        <v>83.00361606280865</v>
       </c>
       <c r="N79" t="n">
-        <v>1.779080495012478</v>
+        <v>77.86687997661033</v>
       </c>
       <c r="O79" t="n">
-        <v>0.007694228636299694</v>
+        <v>-0.2484960445130959</v>
       </c>
       <c r="P79" t="n">
-        <v>61.05894492454533</v>
+        <v>12.88658172093755</v>
       </c>
       <c r="Q79" t="n">
-        <v>-38.94105507545466</v>
+        <v>-87.11341827906246</v>
       </c>
       <c r="R79" t="n">
-        <v>69.98816633533384</v>
+        <v>-69.47277854259958</v>
       </c>
       <c r="S79" t="n">
-        <v>8.915123417007331</v>
+        <v>0.2290750017109655</v>
       </c>
       <c r="T79" t="inlineStr">
         <is>
-          <t>Range</t>
-        </is>
-      </c>
-      <c r="U79" t="inlineStr">
-        <is>
-          <t>Hammer, Bullish Engulfing, Piercing Pattern</t>
-        </is>
-      </c>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="U79" t="inlineStr"/>
       <c r="V79" t="inlineStr">
         <is>
-          <t>Double Bottom</t>
+          <t>Double Top</t>
         </is>
       </c>
       <c r="W79" t="n">
-        <v>55.8</v>
+        <v>55.9</v>
       </c>
       <c r="X79" t="n">
-        <v>74.8</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="Y79" t="inlineStr">
         <is>
@@ -7788,7 +7792,7 @@
       </c>
       <c r="Z79" t="inlineStr">
         <is>
-          <t>trend molto direzionale (ADX 31); pattern: Double Bottom; hammer — segnale di rimbalzo da supporto; penalizzato dal quadrante macro (Stagflazione)</t>
+          <t>trend in sviluppo (ADX 27); pattern: Double Top; sul supporto dei 20g (82.41); in zona Fib Fib 23.6 — livello strutturale; favorito dal quadrante macro (Stagflazione)</t>
         </is>
       </c>
     </row>
@@ -7809,52 +7813,52 @@
         </is>
       </c>
       <c r="D80" t="n">
-        <v>75.37999725341797</v>
+        <v>75.40000152587891</v>
       </c>
       <c r="E80" t="n">
-        <v>-3.226221305045418</v>
+        <v>-3.200539571075867</v>
       </c>
       <c r="F80" t="n">
-        <v>-4.104019335641129</v>
+        <v>-4.078570550883686</v>
       </c>
       <c r="G80" t="n">
-        <v>8.814266529014358</v>
+        <v>8.843143556270894</v>
       </c>
       <c r="H80" t="n">
-        <v>-25.31087939154135</v>
+        <v>-25.29105846327179</v>
       </c>
       <c r="I80" t="n">
-        <v>46.99941491692338</v>
+        <v>47.03071569861722</v>
       </c>
       <c r="J80" t="n">
         <v>18.16319029254958</v>
       </c>
       <c r="K80" t="n">
-        <v>0.5002428789336565</v>
+        <v>0.5015257169580563</v>
       </c>
       <c r="L80" t="n">
-        <v>76.89016410897675</v>
+        <v>76.89206927778255</v>
       </c>
       <c r="M80" t="n">
-        <v>77.42808620072778</v>
+        <v>77.42887068200076</v>
       </c>
       <c r="N80" t="n">
-        <v>64.4016033885126</v>
+        <v>64.40180243599978</v>
       </c>
       <c r="O80" t="n">
-        <v>0.4045683373287473</v>
+        <v>0.4058449632635741</v>
       </c>
       <c r="P80" t="n">
-        <v>41.9329422104666</v>
+        <v>42.08886013412985</v>
       </c>
       <c r="Q80" t="n">
-        <v>-58.0670577895334</v>
+        <v>-57.91113986587015</v>
       </c>
       <c r="R80" t="n">
-        <v>11.93355213659001</v>
+        <v>12.02627445643852</v>
       </c>
       <c r="S80" t="n">
-        <v>4.172133041052972</v>
+        <v>4.199778143309807</v>
       </c>
       <c r="T80" t="inlineStr">
         <is>
@@ -7901,52 +7905,52 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>2016.099975585938</v>
+        <v>2016.300048828125</v>
       </c>
       <c r="E81" t="n">
-        <v>-2.726050342958308</v>
+        <v>-2.716397094248457</v>
       </c>
       <c r="F81" t="n">
-        <v>-3.724756145019592</v>
+        <v>-3.715202005634788</v>
       </c>
       <c r="G81" t="n">
-        <v>6.559195326952305</v>
+        <v>6.569770022628174</v>
       </c>
       <c r="H81" t="n">
-        <v>-25.93586189861954</v>
+        <v>-25.9285119395802</v>
       </c>
       <c r="I81" t="n">
-        <v>47.51155736778559</v>
+        <v>47.52602951297266</v>
       </c>
       <c r="J81" t="n">
         <v>30.40702094970498</v>
       </c>
       <c r="K81" t="n">
-        <v>0.5145222109116466</v>
+        <v>0.5150786046652086</v>
       </c>
       <c r="L81" t="n">
-        <v>2043.503056443961</v>
+        <v>2043.522111038455</v>
       </c>
       <c r="M81" t="n">
-        <v>2060.031791023349</v>
+        <v>2060.039637032847</v>
       </c>
       <c r="N81" t="n">
-        <v>1817.275614522447</v>
+        <v>1817.277605300976</v>
       </c>
       <c r="O81" t="n">
-        <v>6.820965907734315</v>
+        <v>6.833734114643047</v>
       </c>
       <c r="P81" t="n">
-        <v>42.83604650813351</v>
+        <v>42.93455624040221</v>
       </c>
       <c r="Q81" t="n">
-        <v>-57.16395349186649</v>
+        <v>-57.06544375959778</v>
       </c>
       <c r="R81" t="n">
-        <v>22.14542942260731</v>
+        <v>22.18683528233412</v>
       </c>
       <c r="S81" t="n">
-        <v>4.72158875542934</v>
+        <v>4.731981091148341</v>
       </c>
       <c r="T81" t="inlineStr">
         <is>
@@ -8151,7 +8155,7 @@
         <v>53.4</v>
       </c>
       <c r="X83" t="n">
-        <v>63.6</v>
+        <v>63.7</v>
       </c>
       <c r="Y83" t="inlineStr">
         <is>
@@ -8369,52 +8373,52 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>98.81999969482422</v>
+        <v>98.81400299072266</v>
       </c>
       <c r="E86" t="n">
-        <v>0.2332927938706097</v>
+        <v>0.2272103267600301</v>
       </c>
       <c r="F86" t="n">
-        <v>0.6108719880514757</v>
+        <v>0.6047666082642289</v>
       </c>
       <c r="G86" t="n">
-        <v>-0.6134975444828661</v>
+        <v>-0.6195286257291266</v>
       </c>
       <c r="H86" t="n">
-        <v>1.250001270262935</v>
+        <v>1.243857106128399</v>
       </c>
       <c r="I86" t="n">
-        <v>49.89771666757966</v>
+        <v>49.8197585619892</v>
       </c>
       <c r="J86" t="n">
         <v>37.35734105194766</v>
       </c>
       <c r="K86" t="n">
-        <v>0.4286594030126377</v>
+        <v>0.426959751883883</v>
       </c>
       <c r="L86" t="n">
-        <v>98.77369101055976</v>
+        <v>98.77311989588343</v>
       </c>
       <c r="M86" t="n">
-        <v>98.79429701958396</v>
+        <v>98.79406185471723</v>
       </c>
       <c r="N86" t="n">
-        <v>99.12248579725905</v>
+        <v>99.12242612856151</v>
       </c>
       <c r="O86" t="n">
-        <v>-0.06272522445550166</v>
+        <v>-0.06310792010186431</v>
       </c>
       <c r="P86" t="n">
-        <v>44.73687229673141</v>
+        <v>44.5114326032835</v>
       </c>
       <c r="Q86" t="n">
-        <v>-55.26312770326859</v>
+        <v>-55.4885673967165</v>
       </c>
       <c r="R86" t="n">
-        <v>-26.30246620878067</v>
+        <v>-26.47163790349653</v>
       </c>
       <c r="S86" t="n">
-        <v>-0.7831313165125642</v>
+        <v>-0.7891521038553617</v>
       </c>
       <c r="T86" t="inlineStr">
         <is>
@@ -8461,52 +8465,52 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>1471.5</v>
+        <v>1471</v>
       </c>
       <c r="E87" t="n">
-        <v>-4.886560453684019</v>
+        <v>-4.918878985639951</v>
       </c>
       <c r="F87" t="n">
-        <v>-6.30372492836676</v>
+        <v>-6.335561922954469</v>
       </c>
       <c r="G87" t="n">
-        <v>4.272962791562684</v>
+        <v>4.237531951334494</v>
       </c>
       <c r="H87" t="n">
-        <v>-26.7910447761194</v>
+        <v>-26.81592039800995</v>
       </c>
       <c r="I87" t="n">
-        <v>42.32451898523097</v>
+        <v>42.28140598501045</v>
       </c>
       <c r="J87" t="n">
         <v>26.61423539958696</v>
       </c>
       <c r="K87" t="n">
-        <v>0.3693962627629984</v>
+        <v>0.3677576028937318</v>
       </c>
       <c r="L87" t="n">
-        <v>1533.80297315175</v>
+        <v>1533.755354104131</v>
       </c>
       <c r="M87" t="n">
-        <v>1573.657016385984</v>
+        <v>1573.637408542847</v>
       </c>
       <c r="N87" t="n">
-        <v>1478.459116642471</v>
+        <v>1478.454141518093</v>
       </c>
       <c r="O87" t="n">
-        <v>4.550685762144898</v>
+        <v>4.518776930235985</v>
       </c>
       <c r="P87" t="n">
-        <v>19.87870292911121</v>
+        <v>19.5417757608212</v>
       </c>
       <c r="Q87" t="n">
-        <v>-80.12129707088879</v>
+        <v>-80.4582242391788</v>
       </c>
       <c r="R87" t="n">
-        <v>-7.684417237020885</v>
+        <v>-7.821142471942546</v>
       </c>
       <c r="S87" t="n">
-        <v>3.919491525423724</v>
+        <v>3.884180790960445</v>
       </c>
       <c r="T87" t="inlineStr">
         <is>
@@ -8523,7 +8527,7 @@
         <v>49.2</v>
       </c>
       <c r="X87" t="n">
-        <v>65.8</v>
+        <v>65.7</v>
       </c>
       <c r="Y87" t="inlineStr">
         <is>
@@ -8933,52 +8937,52 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>85.80000305175781</v>
+        <v>85.84999847412109</v>
       </c>
       <c r="E92" t="n">
-        <v>-1.283795948308986</v>
+        <v>-1.226274291664209</v>
       </c>
       <c r="F92" t="n">
-        <v>-0.4671662258219134</v>
+        <v>-0.409168721316544</v>
       </c>
       <c r="G92" t="n">
-        <v>8.674568699981556</v>
+        <v>8.737893067919234</v>
       </c>
       <c r="H92" t="n">
-        <v>1.376372191737829</v>
+        <v>1.435443920934931</v>
       </c>
       <c r="I92" t="n">
-        <v>50.95389330333007</v>
+        <v>51.04767011564712</v>
       </c>
       <c r="J92" t="n">
         <v>15.81676323019232</v>
       </c>
       <c r="K92" t="n">
-        <v>0.6188843788153817</v>
+        <v>0.6236739263497695</v>
       </c>
       <c r="L92" t="n">
-        <v>85.30016193683811</v>
+        <v>85.30492340563461</v>
       </c>
       <c r="M92" t="n">
-        <v>87.07825065639238</v>
+        <v>87.08021126119094</v>
       </c>
       <c r="N92" t="n">
-        <v>116.3580650236409</v>
+        <v>116.3585624905301</v>
       </c>
       <c r="O92" t="n">
-        <v>0.2836826745723509</v>
+        <v>0.2868732656291466</v>
       </c>
       <c r="P92" t="n">
-        <v>47.42947317789923</v>
+        <v>47.96919321203016</v>
       </c>
       <c r="Q92" t="n">
-        <v>-52.57052682210077</v>
+        <v>-52.03080678796984</v>
       </c>
       <c r="R92" t="n">
-        <v>34.3603816282762</v>
+        <v>34.78491244331131</v>
       </c>
       <c r="S92" t="n">
-        <v>6.758188148811684</v>
+        <v>6.820395847149618</v>
       </c>
       <c r="T92" t="inlineStr">
         <is>
@@ -10391,7 +10395,7 @@
         <v>38.2</v>
       </c>
       <c r="X107" t="n">
-        <v>74.09999999999999</v>
+        <v>74.2</v>
       </c>
       <c r="Y107" t="inlineStr">
         <is>
@@ -10781,52 +10785,52 @@
         </is>
       </c>
       <c r="D112" t="n">
-        <v>0.2486999928951263</v>
+        <v>0.2489999979734421</v>
       </c>
       <c r="E112" t="n">
-        <v>0.05632298495155119</v>
+        <v>0.1770202341297544</v>
       </c>
       <c r="F112" t="n">
-        <v>-0.3238375465937526</v>
+        <v>-0.2035988824307999</v>
       </c>
       <c r="G112" t="n">
-        <v>3.902940432893076</v>
+        <v>4.028277830047511</v>
       </c>
       <c r="H112" t="n">
-        <v>-12.7083639952874</v>
+        <v>-12.60306469957352</v>
       </c>
       <c r="I112" t="n">
-        <v>48.41913427871974</v>
+        <v>48.60404082188705</v>
       </c>
       <c r="J112" t="n">
         <v>12.32075114472588</v>
       </c>
       <c r="K112" t="n">
-        <v>0.4640095905513412</v>
+        <v>0.4751127949939141</v>
       </c>
       <c r="L112" t="n">
-        <v>0.2498368839921969</v>
+        <v>0.2498654559044174</v>
       </c>
       <c r="M112" t="n">
-        <v>0.2593549220313111</v>
+        <v>0.2593666869363431</v>
       </c>
       <c r="N112" t="n">
-        <v>0.3851570081777929</v>
+        <v>0.3851599933029503</v>
       </c>
       <c r="O112" t="n">
-        <v>0.0006161191810473972</v>
+        <v>0.0006352648042789507</v>
       </c>
       <c r="P112" t="n">
-        <v>40.88794415938682</v>
+        <v>41.83663708549169</v>
       </c>
       <c r="Q112" t="n">
-        <v>-59.11205584061318</v>
+        <v>-58.16336291450831</v>
       </c>
       <c r="R112" t="n">
-        <v>-22.63480916647228</v>
+        <v>-21.23933115512089</v>
       </c>
       <c r="S112" t="n">
-        <v>1.028561950913609</v>
+        <v>1.150432005220314</v>
       </c>
       <c r="T112" t="inlineStr">
         <is>
@@ -10965,52 +10969,52 @@
         </is>
       </c>
       <c r="D114" t="n">
-        <v>1.235000014305115</v>
+        <v>1.235999941825867</v>
       </c>
       <c r="E114" t="n">
-        <v>-2.854958016840148</v>
+        <v>-2.776303765942656</v>
       </c>
       <c r="F114" t="n">
-        <v>-3.054523397516162</v>
+        <v>-2.976030726306123</v>
       </c>
       <c r="G114" t="n">
-        <v>-0.109754655967409</v>
+        <v>-0.0288777294757403</v>
       </c>
       <c r="H114" t="n">
-        <v>-7.928714665631476</v>
+        <v>-7.854168421898322</v>
       </c>
       <c r="I114" t="n">
-        <v>44.01954532160602</v>
+        <v>44.11286979025736</v>
       </c>
       <c r="J114" t="n">
         <v>19.33722230750936</v>
       </c>
       <c r="K114" t="n">
-        <v>0.3438322437868248</v>
+        <v>0.3489821652008541</v>
       </c>
       <c r="L114" t="n">
-        <v>1.273927837022372</v>
+        <v>1.274023068214824</v>
       </c>
       <c r="M114" t="n">
-        <v>1.345878351189991</v>
+        <v>1.345917564033942</v>
       </c>
       <c r="N114" t="n">
-        <v>2.031491962666767</v>
+        <v>2.031501912194336</v>
       </c>
       <c r="O114" t="n">
-        <v>0.006895922565655421</v>
+        <v>0.00695973560401696</v>
       </c>
       <c r="P114" t="n">
-        <v>42.08390194357455</v>
+        <v>42.57017239760088</v>
       </c>
       <c r="Q114" t="n">
-        <v>-57.91609805642546</v>
+        <v>-57.42982760239912</v>
       </c>
       <c r="R114" t="n">
-        <v>-29.53099523011899</v>
+        <v>-29.07661274092767</v>
       </c>
       <c r="S114" t="n">
-        <v>-0.1922564282250905</v>
+        <v>-0.1114462999452726</v>
       </c>
       <c r="T114" t="inlineStr">
         <is>
@@ -11020,7 +11024,7 @@
       <c r="U114" t="inlineStr"/>
       <c r="V114" t="inlineStr"/>
       <c r="W114" t="n">
-        <v>32.3</v>
+        <v>32.4</v>
       </c>
       <c r="X114" t="n">
         <v>73.5</v>
@@ -11479,52 +11483,52 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>96.58000183105469</v>
+        <v>96.87999725341797</v>
       </c>
       <c r="E2" t="n">
-        <v>15.1818766709489</v>
+        <v>15.53965297127389</v>
       </c>
       <c r="F2" t="n">
-        <v>-1.769729321776159</v>
+        <v>-1.4646078578884</v>
       </c>
       <c r="G2" t="n">
-        <v>64.9530368736917</v>
+        <v>65.46541164102284</v>
       </c>
       <c r="H2" t="n">
-        <v>36.52813789597169</v>
+        <v>36.95221964805346</v>
       </c>
       <c r="I2" t="n">
-        <v>62.61906557397396</v>
+        <v>62.75747793408465</v>
       </c>
       <c r="J2" t="n">
         <v>58.66713718370163</v>
       </c>
       <c r="K2" t="n">
-        <v>0.7793214075796742</v>
+        <v>0.7828230138208827</v>
       </c>
       <c r="L2" t="n">
-        <v>81.16944189606649</v>
+        <v>81.19801288867252</v>
       </c>
       <c r="M2" t="n">
-        <v>72.76379308687245</v>
+        <v>72.77555761323964</v>
       </c>
       <c r="N2" t="n">
-        <v>71.92678657570275</v>
+        <v>71.929771604781</v>
       </c>
       <c r="O2" t="n">
-        <v>2.370152015291222</v>
+        <v>2.38929702230244</v>
       </c>
       <c r="P2" t="n">
-        <v>62.32313170690499</v>
+        <v>62.81670756995196</v>
       </c>
       <c r="Q2" t="n">
-        <v>-37.67686829309501</v>
+        <v>-37.18329243004804</v>
       </c>
       <c r="R2" t="n">
-        <v>97.49616069605565</v>
+        <v>97.94667034221942</v>
       </c>
       <c r="S2" t="n">
-        <v>60.75232837481965</v>
+        <v>61.25165496140477</v>
       </c>
       <c r="T2" t="inlineStr">
         <is>
@@ -11575,52 +11579,52 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>105.9499969482422</v>
+        <v>106.3099975585938</v>
       </c>
       <c r="E3" t="n">
-        <v>17.22726285459739</v>
+        <v>17.62558175401288</v>
       </c>
       <c r="F3" t="n">
-        <v>-5.561997822776632</v>
+        <v>-5.241113071446335</v>
       </c>
       <c r="G3" t="n">
-        <v>67.64239821081044</v>
+        <v>68.21201942284476</v>
       </c>
       <c r="H3" t="n">
-        <v>41.7580946969786</v>
+        <v>42.23976531597933</v>
       </c>
       <c r="I3" t="n">
-        <v>66.87637536738788</v>
+        <v>67.03533199099815</v>
       </c>
       <c r="J3" t="n">
         <v>60.96010584971138</v>
       </c>
       <c r="K3" t="n">
-        <v>0.8243832754371067</v>
+        <v>0.8283145443903709</v>
       </c>
       <c r="L3" t="n">
-        <v>86.28123168917092</v>
+        <v>86.31551746158536</v>
       </c>
       <c r="M3" t="n">
-        <v>77.19915834739766</v>
+        <v>77.21327601839184</v>
       </c>
       <c r="N3" t="n">
-        <v>76.06045241872519</v>
+        <v>76.06403451435058</v>
       </c>
       <c r="O3" t="n">
-        <v>2.454738145193563</v>
+        <v>2.477712543119129</v>
       </c>
       <c r="P3" t="n">
-        <v>76.04203097623696</v>
+        <v>76.68328603466863</v>
       </c>
       <c r="Q3" t="n">
-        <v>-23.95796902376303</v>
+        <v>-23.31671396533137</v>
       </c>
       <c r="R3" t="n">
-        <v>109.5817564546903</v>
+        <v>110.0953304243817</v>
       </c>
       <c r="S3" t="n">
-        <v>66.19607364430146</v>
+        <v>66.76078048406863</v>
       </c>
       <c r="T3" t="inlineStr">
         <is>
@@ -13343,52 +13347,52 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>6.013999938964844</v>
+        <v>6.021999835968018</v>
       </c>
       <c r="E22" t="n">
-        <v>-1.466370967987651</v>
+        <v>-1.335300317571131</v>
       </c>
       <c r="F22" t="n">
-        <v>12.56901643024142</v>
+        <v>12.71875712633885</v>
       </c>
       <c r="G22" t="n">
-        <v>15.97723981961201</v>
+        <v>16.13151417656005</v>
       </c>
       <c r="H22" t="n">
-        <v>29.15279966346447</v>
+        <v>29.32460031286008</v>
       </c>
       <c r="I22" t="n">
-        <v>60.97566942831919</v>
+        <v>61.20217431761125</v>
       </c>
       <c r="J22" t="n">
         <v>48.57643889583426</v>
       </c>
       <c r="K22" t="n">
-        <v>0.7983255124047095</v>
+        <v>0.8060700836818788</v>
       </c>
       <c r="L22" t="n">
-        <v>5.667643397285032</v>
+        <v>5.668405292237716</v>
       </c>
       <c r="M22" t="n">
-        <v>5.312413917801926</v>
+        <v>5.312727639253031</v>
       </c>
       <c r="N22" t="n">
-        <v>4.525406774026774</v>
+        <v>4.52548637499198</v>
       </c>
       <c r="O22" t="n">
-        <v>-0.005522153404334346</v>
+        <v>-0.005011618666808743</v>
       </c>
       <c r="P22" t="n">
-        <v>60.16128635307183</v>
+        <v>60.80643945628248</v>
       </c>
       <c r="Q22" t="n">
-        <v>-39.83871364692817</v>
+        <v>-39.19356054371752</v>
       </c>
       <c r="R22" t="n">
-        <v>45.90320740113416</v>
+        <v>46.27821937082219</v>
       </c>
       <c r="S22" t="n">
-        <v>11.7428460250103</v>
+        <v>11.89148773902991</v>
       </c>
       <c r="T22" t="inlineStr">
         <is>
@@ -13406,10 +13410,10 @@
         </is>
       </c>
       <c r="W22" t="n">
-        <v>74.09999999999999</v>
+        <v>74.2</v>
       </c>
       <c r="X22" t="n">
-        <v>80.5</v>
+        <v>80.59999999999999</v>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
@@ -14371,52 +14375,52 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>4705.39990234375</v>
+        <v>4705.2001953125</v>
       </c>
       <c r="E33" t="n">
-        <v>-3.133238476875344</v>
+        <v>-3.137349705202819</v>
       </c>
       <c r="F33" t="n">
-        <v>2.953789665774553</v>
+        <v>2.949420091218347</v>
       </c>
       <c r="G33" t="n">
-        <v>11.54730863640774</v>
+        <v>11.54257433490009</v>
       </c>
       <c r="H33" t="n">
-        <v>63.17796306666217</v>
+        <v>63.17103745199694</v>
       </c>
       <c r="I33" t="n">
-        <v>54.59289472123281</v>
+        <v>54.5873247888562</v>
       </c>
       <c r="J33" t="n">
         <v>44.58204990747586</v>
       </c>
       <c r="K33" t="n">
-        <v>0.4708166594523198</v>
+        <v>0.4706505686999741</v>
       </c>
       <c r="L33" t="n">
-        <v>4653.993899685292</v>
+        <v>4653.974879968031</v>
       </c>
       <c r="M33" t="n">
-        <v>4170.014461147833</v>
+        <v>4170.006629499549</v>
       </c>
       <c r="N33" t="n">
-        <v>2980.280518766032</v>
+        <v>2980.278531631393</v>
       </c>
       <c r="O33" t="n">
-        <v>-63.99145816955479</v>
+        <v>-64.00420300573728</v>
       </c>
       <c r="P33" t="n">
-        <v>40.70283685611913</v>
+        <v>40.68939219618027</v>
       </c>
       <c r="Q33" t="n">
-        <v>-59.29716314388087</v>
+        <v>-59.31060780381973</v>
       </c>
       <c r="R33" t="n">
-        <v>-0.3348037936943221</v>
+        <v>-0.3446872844725172</v>
       </c>
       <c r="S33" t="n">
-        <v>11.6902848730398</v>
+        <v>11.68554450332109</v>
       </c>
       <c r="T33" t="inlineStr">
         <is>
@@ -14747,52 +14751,52 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>75.37999725341797</v>
+        <v>75.40000152587891</v>
       </c>
       <c r="E37" t="n">
-        <v>-7.778514020032368</v>
+        <v>-7.754040369203041</v>
       </c>
       <c r="F37" t="n">
-        <v>8.67934917833313</v>
+        <v>8.70819040135058</v>
       </c>
       <c r="G37" t="n">
-        <v>33.5435609158085</v>
+        <v>33.57900057984804</v>
       </c>
       <c r="H37" t="n">
-        <v>129.8100675867018</v>
+        <v>129.8710543653403</v>
       </c>
       <c r="I37" t="n">
-        <v>53.57872393323125</v>
+        <v>53.59329753150701</v>
       </c>
       <c r="J37" t="n">
         <v>55.22104530237728</v>
       </c>
       <c r="K37" t="n">
-        <v>0.4266666749979549</v>
+        <v>0.427188105239013</v>
       </c>
       <c r="L37" t="n">
-        <v>73.75112377955124</v>
+        <v>73.75302894835704</v>
       </c>
       <c r="M37" t="n">
-        <v>61.11588829125289</v>
+        <v>61.11667277252587</v>
       </c>
       <c r="N37" t="n">
-        <v>39.02584445596523</v>
+        <v>39.0260435034524</v>
       </c>
       <c r="O37" t="n">
-        <v>-1.884256430319398</v>
+        <v>-1.882979804384571</v>
       </c>
       <c r="P37" t="n">
-        <v>23.73359311202937</v>
+        <v>23.76681727993788</v>
       </c>
       <c r="Q37" t="n">
-        <v>-76.26640688797063</v>
+        <v>-76.23318272006212</v>
       </c>
       <c r="R37" t="n">
-        <v>-8.333236036402434</v>
+        <v>-8.306565081214526</v>
       </c>
       <c r="S37" t="n">
-        <v>29.02672984752115</v>
+        <v>29.06097083919878</v>
       </c>
       <c r="T37" t="inlineStr">
         <is>
@@ -15505,7 +15509,7 @@
         <v>80.95135377215732</v>
       </c>
       <c r="J45" t="n">
-        <v>24.67093203662111</v>
+        <v>24.30623998972093</v>
       </c>
       <c r="K45" t="n">
         <v>1.140966420531304</v>
@@ -15529,7 +15533,7 @@
         <v>2.285124380319148</v>
       </c>
       <c r="R45" t="n">
-        <v>214.7842957419916</v>
+        <v>205.2800019976372</v>
       </c>
       <c r="S45" t="n">
         <v>27.97360497235619</v>
@@ -15562,7 +15566,7 @@
       </c>
       <c r="Z45" t="inlineStr">
         <is>
-          <t>trend in sviluppo (ADX 25); RSI ipercomprato (81) — attenzione estensione; pattern: Double Bottom; breakout massimi 50g — rottura resistenza rilevante; hammer — segnale di rimbalzo da supporto; vicino alla resistenza dei 20g (79.09); favorito dal quadrante macro (Stagflazione)</t>
+          <t>trend in sviluppo (ADX 24); RSI ipercomprato (81) — attenzione estensione; pattern: Double Bottom; breakout massimi 50g — rottura resistenza rilevante; hammer — segnale di rimbalzo da supporto; vicino alla resistenza dei 20g (79.09); favorito dal quadrante macro (Stagflazione)</t>
         </is>
       </c>
     </row>
@@ -16051,52 +16055,52 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>159.7010040283203</v>
+        <v>159.7039947509766</v>
       </c>
       <c r="E51" t="n">
-        <v>0.3178470937037936</v>
+        <v>0.3197257472536297</v>
       </c>
       <c r="F51" t="n">
-        <v>1.125229921967841</v>
+        <v>1.127123695385768</v>
       </c>
       <c r="G51" t="n">
-        <v>2.186409050843241</v>
+        <v>2.188322696975686</v>
       </c>
       <c r="H51" t="n">
-        <v>4.387247243171877</v>
+        <v>4.38920210442808</v>
       </c>
       <c r="I51" t="n">
-        <v>59.7555905300759</v>
+        <v>59.76173602887761</v>
       </c>
       <c r="J51" t="n">
         <v>13.25914642780409</v>
       </c>
       <c r="K51" t="n">
-        <v>0.8030894705474647</v>
+        <v>0.8034032206386739</v>
       </c>
       <c r="L51" t="n">
-        <v>157.0481985107095</v>
+        <v>157.0484833414386</v>
       </c>
       <c r="M51" t="n">
-        <v>154.0784628184865</v>
+        <v>154.0785801017279</v>
       </c>
       <c r="N51" t="n">
-        <v>144.8351292100681</v>
+        <v>144.8351589685025</v>
       </c>
       <c r="O51" t="n">
-        <v>0.05160188126077347</v>
+        <v>0.05179274219382202</v>
       </c>
       <c r="P51" t="n">
-        <v>93.3358659114979</v>
+        <v>93.37347086000214</v>
       </c>
       <c r="Q51" t="n">
-        <v>-6.664134088502095</v>
+        <v>-6.626529139997851</v>
       </c>
       <c r="R51" t="n">
-        <v>53.44014287650015</v>
+        <v>53.46204122637735</v>
       </c>
       <c r="S51" t="n">
-        <v>2.938601917936423</v>
+        <v>2.940529650393908</v>
       </c>
       <c r="T51" t="inlineStr">
         <is>
@@ -16243,52 +16247,52 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>2016.099975585938</v>
+        <v>2016.300048828125</v>
       </c>
       <c r="E53" t="n">
-        <v>-5.102378179056832</v>
+        <v>-5.092960751794539</v>
       </c>
       <c r="F53" t="n">
-        <v>2.308941467761416</v>
+        <v>2.319094377771869</v>
       </c>
       <c r="G53" t="n">
-        <v>20.17047352106614</v>
+        <v>20.18239896947826</v>
       </c>
       <c r="H53" t="n">
-        <v>99.6533967080303</v>
+        <v>99.67320986356667</v>
       </c>
       <c r="I53" t="n">
-        <v>51.91982895110198</v>
+        <v>51.92575570247612</v>
       </c>
       <c r="J53" t="n">
         <v>33.03065630583864</v>
       </c>
       <c r="K53" t="n">
-        <v>0.3651829960451154</v>
+        <v>0.3654001414664626</v>
       </c>
       <c r="L53" t="n">
-        <v>2013.330759335012</v>
+        <v>2013.349813929506</v>
       </c>
       <c r="M53" t="n">
-        <v>1755.105091138624</v>
+        <v>1755.112937148122</v>
       </c>
       <c r="N53" t="n">
-        <v>1271.745849061017</v>
+        <v>1271.747839839546</v>
       </c>
       <c r="O53" t="n">
-        <v>-45.46449053423203</v>
+        <v>-45.4517223273233</v>
       </c>
       <c r="P53" t="n">
-        <v>18.79794095963702</v>
+        <v>18.81736743416452</v>
       </c>
       <c r="Q53" t="n">
-        <v>-81.20205904036297</v>
+        <v>-81.18263256583548</v>
       </c>
       <c r="R53" t="n">
-        <v>-19.47398560321286</v>
+        <v>-19.46063279094261</v>
       </c>
       <c r="S53" t="n">
-        <v>21.81872964265483</v>
+        <v>21.83081866030967</v>
       </c>
       <c r="T53" t="inlineStr">
         <is>
@@ -17179,52 +17183,52 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>1.346545696258545</v>
+        <v>1.346590995788574</v>
       </c>
       <c r="E63" t="n">
-        <v>-0.4485245541018035</v>
+        <v>-0.4451755143596303</v>
       </c>
       <c r="F63" t="n">
-        <v>0.2961119381085231</v>
+        <v>0.2994860283805467</v>
       </c>
       <c r="G63" t="n">
-        <v>1.69381903385486</v>
+        <v>1.697240144792223</v>
       </c>
       <c r="H63" t="n">
-        <v>7.179649799193122</v>
+        <v>7.183255460536886</v>
       </c>
       <c r="I63" t="n">
-        <v>51.95293536506068</v>
+        <v>51.96876117704838</v>
       </c>
       <c r="J63" t="n">
         <v>20.56534698593375</v>
       </c>
       <c r="K63" t="n">
-        <v>0.5217646219276939</v>
+        <v>0.5226699895199916</v>
       </c>
       <c r="L63" t="n">
-        <v>1.34230329201733</v>
+        <v>1.342307606258285</v>
       </c>
       <c r="M63" t="n">
-        <v>1.334202527147415</v>
+        <v>1.334204303599573</v>
       </c>
       <c r="N63" t="n">
-        <v>1.302902274338335</v>
+        <v>1.302902725079927</v>
       </c>
       <c r="O63" t="n">
-        <v>-0.0005802061342636096</v>
+        <v>-0.0005773152240851659</v>
       </c>
       <c r="P63" t="n">
-        <v>44.38117163469313</v>
+        <v>44.44724583602122</v>
       </c>
       <c r="Q63" t="n">
-        <v>-55.61882836530687</v>
+        <v>-55.55275416397878</v>
       </c>
       <c r="R63" t="n">
-        <v>18.68529636084946</v>
+        <v>18.77284236865096</v>
       </c>
       <c r="S63" t="n">
-        <v>1.078448690421929</v>
+        <v>1.081849099509036</v>
       </c>
       <c r="T63" t="inlineStr">
         <is>
@@ -18863,52 +18867,52 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>1471.5</v>
+        <v>1471</v>
       </c>
       <c r="E81" t="n">
-        <v>-7.476108060163533</v>
+        <v>-7.507546691471667</v>
       </c>
       <c r="F81" t="n">
-        <v>3.277649464588728</v>
+        <v>3.242556821209663</v>
       </c>
       <c r="G81" t="n">
-        <v>0.1974686410372239</v>
+        <v>0.1634226102383618</v>
       </c>
       <c r="H81" t="n">
-        <v>46.4179104477612</v>
+        <v>46.3681592039801</v>
       </c>
       <c r="I81" t="n">
-        <v>47.0777340603082</v>
+        <v>47.05986811946588</v>
       </c>
       <c r="J81" t="n">
         <v>27.29489222299879</v>
       </c>
       <c r="K81" t="n">
-        <v>0.2190025275188947</v>
+        <v>0.2183696702775351</v>
       </c>
       <c r="L81" t="n">
-        <v>1566.843185047831</v>
+        <v>1566.795566000211</v>
       </c>
       <c r="M81" t="n">
-        <v>1439.721111738184</v>
+        <v>1439.701503895046</v>
       </c>
       <c r="N81" t="n">
-        <v>1368.793142748639</v>
+        <v>1368.78816762426</v>
       </c>
       <c r="O81" t="n">
-        <v>-43.22375899754395</v>
+        <v>-43.25566782945285</v>
       </c>
       <c r="P81" t="n">
-        <v>15.71324815222404</v>
+        <v>15.65290539475448</v>
       </c>
       <c r="Q81" t="n">
-        <v>-84.28675184777596</v>
+        <v>-84.34709460524552</v>
       </c>
       <c r="R81" t="n">
-        <v>-49.72420026568962</v>
+        <v>-49.76995730431268</v>
       </c>
       <c r="S81" t="n">
-        <v>-0.06112635147643708</v>
+        <v>-0.09508451445588983</v>
       </c>
       <c r="T81" t="inlineStr">
         <is>
@@ -19323,52 +19327,52 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>98.81999969482422</v>
+        <v>98.81400299072266</v>
       </c>
       <c r="E86" t="n">
-        <v>0.7339462098901794</v>
+        <v>0.7278333615773791</v>
       </c>
       <c r="F86" t="n">
-        <v>-0.8329170279431808</v>
+        <v>-0.8389347941345937</v>
       </c>
       <c r="G86" t="n">
-        <v>-0.6434741559819268</v>
+        <v>-0.6495034181544179</v>
       </c>
       <c r="H86" t="n">
-        <v>-7.272215466072107</v>
+        <v>-7.277842475660856</v>
       </c>
       <c r="I86" t="n">
-        <v>49.91194831290031</v>
+        <v>49.88154856848116</v>
       </c>
       <c r="J86" t="n">
         <v>18.97345570552778</v>
       </c>
       <c r="K86" t="n">
-        <v>0.5639221123514799</v>
+        <v>0.5625210334990803</v>
       </c>
       <c r="L86" t="n">
-        <v>98.79140954764827</v>
+        <v>98.79083843297194</v>
       </c>
       <c r="M86" t="n">
-        <v>99.39048315254142</v>
+        <v>99.39024798767468</v>
       </c>
       <c r="N86" t="n">
-        <v>100.9678394482873</v>
+        <v>100.9677797795898</v>
       </c>
       <c r="O86" t="n">
-        <v>0.07549269778921093</v>
+        <v>0.07511000214284827</v>
       </c>
       <c r="P86" t="n">
-        <v>64.24359520112237</v>
+        <v>64.12578167624964</v>
       </c>
       <c r="Q86" t="n">
-        <v>-35.75640479887763</v>
+        <v>-35.87421832375037</v>
       </c>
       <c r="R86" t="n">
-        <v>7.349173803316109</v>
+        <v>7.177846743800149</v>
       </c>
       <c r="S86" t="n">
-        <v>-0.1717326726072499</v>
+        <v>-0.1777905615162001</v>
       </c>
       <c r="T86" t="inlineStr">
         <is>
@@ -20083,52 +20087,52 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>77984</v>
+        <v>77989.5390625</v>
       </c>
       <c r="E94" t="n">
-        <v>5.588752152219478</v>
+        <v>5.59625193034663</v>
       </c>
       <c r="F94" t="n">
-        <v>14.9440010907181</v>
+        <v>14.95216535526009</v>
       </c>
       <c r="G94" t="n">
-        <v>-13.72908555502317</v>
+        <v>-13.72295788797553</v>
       </c>
       <c r="H94" t="n">
-        <v>-18.91450516165026</v>
+        <v>-18.90874580558038</v>
       </c>
       <c r="I94" t="n">
-        <v>46.62357884333346</v>
+        <v>46.62941190772215</v>
       </c>
       <c r="J94" t="n">
         <v>53.35674088539724</v>
       </c>
       <c r="K94" t="n">
-        <v>0.5236082038757068</v>
+        <v>0.5237386362831515</v>
       </c>
       <c r="L94" t="n">
-        <v>77846.54053635502</v>
+        <v>77847.06806611693</v>
       </c>
       <c r="M94" t="n">
-        <v>86258.88351617246</v>
+        <v>86259.10073430972</v>
       </c>
       <c r="N94" t="n">
-        <v>68560.76792809997</v>
+        <v>68560.82304314972</v>
       </c>
       <c r="O94" t="n">
-        <v>1154.2846467864</v>
+        <v>1154.638136814884</v>
       </c>
       <c r="P94" t="n">
-        <v>53.3241934103233</v>
+        <v>53.34068528022687</v>
       </c>
       <c r="Q94" t="n">
-        <v>-46.6758065896767</v>
+        <v>-46.65931471977312</v>
       </c>
       <c r="R94" t="n">
-        <v>-2.0967491168449</v>
+        <v>-2.088931782954198</v>
       </c>
       <c r="S94" t="n">
-        <v>-13.7398955851932</v>
+        <v>-13.73376868596246</v>
       </c>
       <c r="T94" t="inlineStr">
         <is>
@@ -20827,52 +20831,52 @@
         </is>
       </c>
       <c r="D102" t="n">
-        <v>2326.219970703125</v>
+        <v>2328.590087890625</v>
       </c>
       <c r="E102" t="n">
-        <v>2.706632460574965</v>
+        <v>2.811277231031251</v>
       </c>
       <c r="F102" t="n">
-        <v>13.30565995733764</v>
+        <v>13.42110376552776</v>
       </c>
       <c r="G102" t="n">
-        <v>-22.25493083092078</v>
+        <v>-22.1757186639711</v>
       </c>
       <c r="H102" t="n">
-        <v>-12.65700193474307</v>
+        <v>-12.56801072001299</v>
       </c>
       <c r="I102" t="n">
-        <v>43.73988527897399</v>
+        <v>43.80219017260816</v>
       </c>
       <c r="J102" t="n">
         <v>39.58791687396969</v>
       </c>
       <c r="K102" t="n">
-        <v>0.4460328214542326</v>
+        <v>0.4471846191091856</v>
       </c>
       <c r="L102" t="n">
-        <v>2443.621747044112</v>
+        <v>2443.847472490541</v>
       </c>
       <c r="M102" t="n">
-        <v>2780.878046336457</v>
+        <v>2780.970992108516</v>
       </c>
       <c r="N102" t="n">
-        <v>2567.464983287915</v>
+        <v>2567.488566543513</v>
       </c>
       <c r="O102" t="n">
-        <v>31.90710717534927</v>
+        <v>32.05836251722974</v>
       </c>
       <c r="P102" t="n">
-        <v>37.65202618019774</v>
+        <v>37.80652913442218</v>
       </c>
       <c r="Q102" t="n">
-        <v>-62.34797381980226</v>
+        <v>-62.19347086557782</v>
       </c>
       <c r="R102" t="n">
-        <v>-12.37194609444037</v>
+        <v>-12.30085957334968</v>
       </c>
       <c r="S102" t="n">
-        <v>-24.01206562644249</v>
+        <v>-23.93464375251414</v>
       </c>
       <c r="T102" t="inlineStr">
         <is>
@@ -21015,52 +21019,52 @@
         </is>
       </c>
       <c r="D104" t="n">
-        <v>1.435400009155273</v>
+        <v>1.437199950218201</v>
       </c>
       <c r="E104" t="n">
-        <v>2.921662059370389</v>
+        <v>3.050722199138955</v>
       </c>
       <c r="F104" t="n">
-        <v>3.647742179059565</v>
+        <v>3.777712797728827</v>
       </c>
       <c r="G104" t="n">
-        <v>-33.57603632843922</v>
+        <v>-33.49274301715857</v>
       </c>
       <c r="H104" t="n">
-        <v>-47.37932059803902</v>
+        <v>-47.31333611914073</v>
       </c>
       <c r="I104" t="n">
-        <v>37.81141542673841</v>
+        <v>37.89762998686645</v>
       </c>
       <c r="J104" t="n">
         <v>43.71256524006639</v>
       </c>
       <c r="K104" t="n">
-        <v>0.3577127208031831</v>
+        <v>0.3591748416719711</v>
       </c>
       <c r="L104" t="n">
-        <v>1.61609089441769</v>
+        <v>1.616262317376064</v>
       </c>
       <c r="M104" t="n">
-        <v>1.890398170228543</v>
+        <v>1.890468756152579</v>
       </c>
       <c r="N104" t="n">
-        <v>1.419897481858458</v>
+        <v>1.41991539171978</v>
       </c>
       <c r="O104" t="n">
-        <v>0.01428568700100774</v>
+        <v>0.01440055503465321</v>
       </c>
       <c r="P104" t="n">
-        <v>33.84404717110214</v>
+        <v>34.04580015991653</v>
       </c>
       <c r="Q104" t="n">
-        <v>-66.15595282889785</v>
+        <v>-65.95419984008346</v>
       </c>
       <c r="R104" t="n">
-        <v>-26.82574834271536</v>
+        <v>-26.74799279635965</v>
       </c>
       <c r="S104" t="n">
-        <v>-29.75502072461781</v>
+        <v>-29.66693599432953</v>
       </c>
       <c r="T104" t="inlineStr">
         <is>
@@ -21074,7 +21078,7 @@
         </is>
       </c>
       <c r="W104" t="n">
-        <v>36.1</v>
+        <v>36.2</v>
       </c>
       <c r="X104" t="n">
         <v>71.59999999999999</v>
@@ -21107,52 +21111,52 @@
         </is>
       </c>
       <c r="D105" t="n">
-        <v>85.80000305175781</v>
+        <v>85.84999847412109</v>
       </c>
       <c r="E105" t="n">
-        <v>2.654977279121118</v>
+        <v>2.714794047934843</v>
       </c>
       <c r="F105" t="n">
-        <v>-0.3812290089082127</v>
+        <v>-0.3231814290263535</v>
       </c>
       <c r="G105" t="n">
-        <v>-35.76152501958118</v>
+        <v>-35.72409343946011</v>
       </c>
       <c r="H105" t="n">
-        <v>-54.47947382928919</v>
+        <v>-54.45294914570928</v>
       </c>
       <c r="I105" t="n">
-        <v>35.08578039780929</v>
+        <v>35.11991064863901</v>
       </c>
       <c r="J105" t="n">
         <v>61.92755203820978</v>
       </c>
       <c r="K105" t="n">
-        <v>0.3285306669973538</v>
+        <v>0.3290436211629845</v>
       </c>
       <c r="L105" t="n">
-        <v>102.8302712326047</v>
+        <v>102.8350327014012</v>
       </c>
       <c r="M105" t="n">
-        <v>130.4902289412966</v>
+        <v>130.4921895460952</v>
       </c>
       <c r="N105" t="n">
-        <v>117.4811675943665</v>
+        <v>117.4816650612557</v>
       </c>
       <c r="O105" t="n">
-        <v>1.100384845201418</v>
+        <v>1.103575436258215</v>
       </c>
       <c r="P105" t="n">
-        <v>24.68505801484667</v>
+        <v>24.75719541077144</v>
       </c>
       <c r="Q105" t="n">
-        <v>-75.31494198515333</v>
+        <v>-75.24280458922856</v>
       </c>
       <c r="R105" t="n">
-        <v>-26.85735045976111</v>
+        <v>-26.83195357575975</v>
       </c>
       <c r="S105" t="n">
-        <v>-35.04603966045982</v>
+        <v>-35.00819116901648</v>
       </c>
       <c r="T105" t="inlineStr">
         <is>
@@ -22047,52 +22051,52 @@
         </is>
       </c>
       <c r="D115" t="n">
-        <v>0.2486999928951263</v>
+        <v>0.2489999979734421</v>
       </c>
       <c r="E115" t="n">
-        <v>2.546550000583703</v>
+        <v>2.670251193357376</v>
       </c>
       <c r="F115" t="n">
-        <v>-0.756204411854422</v>
+        <v>-0.6364873088453904</v>
       </c>
       <c r="G115" t="n">
-        <v>-40.19981676536041</v>
+        <v>-40.12768021864902</v>
       </c>
       <c r="H115" t="n">
-        <v>-67.78518455894587</v>
+        <v>-67.74632405027911</v>
       </c>
       <c r="I115" t="n">
-        <v>32.36501927002818</v>
+        <v>32.42173112074623</v>
       </c>
       <c r="J115" t="n">
         <v>50.19357591898496</v>
       </c>
       <c r="K115" t="n">
-        <v>0.2855050224448236</v>
+        <v>0.2866418539301916</v>
       </c>
       <c r="L115" t="n">
-        <v>0.322255904914378</v>
+        <v>0.3222844768265986</v>
       </c>
       <c r="M115" t="n">
-        <v>0.4623867402340646</v>
+        <v>0.4623985051390966</v>
       </c>
       <c r="N115" t="n">
-        <v>0.5560564364382705</v>
+        <v>0.5560594215634279</v>
       </c>
       <c r="O115" t="n">
-        <v>0.009862853970815683</v>
+        <v>0.00988199959404723</v>
       </c>
       <c r="P115" t="n">
-        <v>15.0306790981786</v>
+        <v>15.23143063263207</v>
       </c>
       <c r="Q115" t="n">
-        <v>-84.9693209018214</v>
+        <v>-84.76856936736793</v>
       </c>
       <c r="R115" t="n">
-        <v>-22.75983354964038</v>
+        <v>-22.72259407452991</v>
       </c>
       <c r="S115" t="n">
-        <v>-40.33266894782843</v>
+        <v>-40.26069265978428</v>
       </c>
       <c r="T115" t="inlineStr">
         <is>
@@ -22139,52 +22143,52 @@
         </is>
       </c>
       <c r="D116" t="n">
-        <v>1.235000014305115</v>
+        <v>1.235999941825867</v>
       </c>
       <c r="E116" t="n">
-        <v>-0.429558970169519</v>
+        <v>-0.3489409757679862</v>
       </c>
       <c r="F116" t="n">
-        <v>-12.50492057530593</v>
+        <v>-12.43407949284947</v>
       </c>
       <c r="G116" t="n">
-        <v>-44.33371472515233</v>
+        <v>-44.28864407739557</v>
       </c>
       <c r="H116" t="n">
-        <v>-74.69680167396915</v>
+        <v>-74.67631473949452</v>
       </c>
       <c r="I116" t="n">
-        <v>30.67419795812202</v>
+        <v>30.69032533681819</v>
       </c>
       <c r="J116" t="n">
         <v>39.87769041366358</v>
       </c>
       <c r="K116" t="n">
-        <v>0.2436789550201171</v>
+        <v>0.24438021102285</v>
       </c>
       <c r="L116" t="n">
-        <v>1.672816136956734</v>
+        <v>1.672911368149187</v>
       </c>
       <c r="M116" t="n">
-        <v>2.65459090705638</v>
+        <v>2.654630119900331</v>
       </c>
       <c r="N116" t="n">
-        <v>5.831714067342209</v>
+        <v>5.831724016869779</v>
       </c>
       <c r="O116" t="n">
-        <v>0.05266346448988146</v>
+        <v>0.05272727752824302</v>
       </c>
       <c r="P116" t="n">
-        <v>11.16524766424063</v>
+        <v>11.2719017175524</v>
       </c>
       <c r="Q116" t="n">
-        <v>-88.83475233575938</v>
+        <v>-88.7280982824476</v>
       </c>
       <c r="R116" t="n">
-        <v>-27.53372905026585</v>
+        <v>-27.50810091411096</v>
       </c>
       <c r="S116" t="n">
-        <v>-40.9523458318747</v>
+        <v>-40.90453743207338</v>
       </c>
       <c r="T116" t="inlineStr">
         <is>
@@ -22473,52 +22477,52 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>4705.39990234375</v>
+        <v>4705.2001953125</v>
       </c>
       <c r="E2" t="n">
-        <v>1.24364840935105</v>
+        <v>1.239351416773093</v>
       </c>
       <c r="F2" t="n">
-        <v>11.54730863640774</v>
+        <v>11.54257433490009</v>
       </c>
       <c r="G2" t="n">
-        <v>93.91716061585618</v>
+        <v>93.90893036523799</v>
       </c>
       <c r="H2" t="n">
-        <v>172.2874815589483</v>
+        <v>172.2759251076972</v>
       </c>
       <c r="I2" t="n">
-        <v>75.55999689067148</v>
+        <v>75.55808848735455</v>
       </c>
       <c r="J2" t="n">
         <v>92.43498481484269</v>
       </c>
       <c r="K2" t="n">
-        <v>0.842485120892047</v>
+        <v>0.8424330337628082</v>
       </c>
       <c r="L2" t="n">
-        <v>3759.917043401704</v>
+        <v>3759.898023684442</v>
       </c>
       <c r="M2" t="n">
-        <v>2937.043507723088</v>
+        <v>2937.035676074803</v>
       </c>
       <c r="N2" t="n">
-        <v>2266.462439236068</v>
+        <v>2266.459054371132</v>
       </c>
       <c r="O2" t="n">
-        <v>115.2535439445708</v>
+        <v>115.2407991083879</v>
       </c>
       <c r="P2" t="n">
-        <v>67.65094027485992</v>
+        <v>67.6436056557266</v>
       </c>
       <c r="Q2" t="n">
-        <v>-32.34905972514008</v>
+        <v>-32.35639434427339</v>
       </c>
       <c r="R2" t="n">
-        <v>86.28335217775647</v>
+        <v>86.27889383030303</v>
       </c>
       <c r="S2" t="n">
-        <v>88.6839285513243</v>
+        <v>88.67592041004033</v>
       </c>
       <c r="T2" t="inlineStr">
         <is>
@@ -22569,52 +22573,52 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>2016.099975585938</v>
+        <v>2016.300048828125</v>
       </c>
       <c r="E3" t="n">
-        <v>3.389742337740387</v>
+        <v>3.400002504006405</v>
       </c>
       <c r="F3" t="n">
-        <v>20.17047352106614</v>
+        <v>20.18239896947826</v>
       </c>
       <c r="G3" t="n">
-        <v>105.2636887120072</v>
+        <v>105.2840586203458</v>
       </c>
       <c r="H3" t="n">
-        <v>70.35065277447718</v>
+        <v>70.36755799139205</v>
       </c>
       <c r="I3" t="n">
-        <v>67.17668997064877</v>
+        <v>67.18036081442389</v>
       </c>
       <c r="J3" t="n">
         <v>68.41678221756783</v>
       </c>
       <c r="K3" t="n">
-        <v>0.8217532606044605</v>
+        <v>0.8218440881550911</v>
       </c>
       <c r="L3" t="n">
-        <v>1555.135175431709</v>
+        <v>1555.154230026203</v>
       </c>
       <c r="M3" t="n">
-        <v>1260.742176672679</v>
+        <v>1260.750022682176</v>
       </c>
       <c r="N3" t="n">
-        <v>1105.768945130108</v>
+        <v>1105.77233620201</v>
       </c>
       <c r="O3" t="n">
-        <v>84.57081143445734</v>
+        <v>84.58357964136624</v>
       </c>
       <c r="P3" t="n">
-        <v>57.5029235093824</v>
+        <v>57.51309034977653</v>
       </c>
       <c r="Q3" t="n">
-        <v>-42.4970764906176</v>
+        <v>-42.48690965022347</v>
       </c>
       <c r="R3" t="n">
-        <v>116.3113828962836</v>
+        <v>116.3225062998556</v>
       </c>
       <c r="S3" t="n">
-        <v>117.2989870782165</v>
+        <v>117.320551342586</v>
       </c>
       <c r="T3" t="inlineStr">
         <is>
@@ -22665,52 +22669,52 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>75.37999725341797</v>
+        <v>75.40000152587891</v>
       </c>
       <c r="E4" t="n">
-        <v>0.9238114733668867</v>
+        <v>0.9505945391147241</v>
       </c>
       <c r="F4" t="n">
-        <v>33.5435609158085</v>
+        <v>33.57900057984804</v>
       </c>
       <c r="G4" t="n">
-        <v>161.9361928319004</v>
+        <v>162.0057052113076</v>
       </c>
       <c r="H4" t="n">
-        <v>185.508658562205</v>
+        <v>185.5844265802992</v>
       </c>
       <c r="I4" t="n">
-        <v>70.88414066502712</v>
+        <v>70.89234862618019</v>
       </c>
       <c r="J4" t="n">
         <v>61.80579865011009</v>
       </c>
       <c r="K4" t="n">
-        <v>0.8533736320181183</v>
+        <v>0.8535844692367101</v>
       </c>
       <c r="L4" t="n">
-        <v>52.94139402999487</v>
+        <v>52.94329919880068</v>
       </c>
       <c r="M4" t="n">
-        <v>38.67411272742319</v>
+        <v>38.67489720869617</v>
       </c>
       <c r="N4" t="n">
-        <v>29.25802455342868</v>
+        <v>29.25836360889413</v>
       </c>
       <c r="O4" t="n">
-        <v>4.115062306626227</v>
+        <v>4.116338932561058</v>
       </c>
       <c r="P4" t="n">
-        <v>50.6183417274925</v>
+        <v>50.63985401019983</v>
       </c>
       <c r="Q4" t="n">
-        <v>-49.3816582725075</v>
+        <v>-49.36014598980017</v>
       </c>
       <c r="R4" t="n">
-        <v>128.3147728610845</v>
+        <v>128.3401504186747</v>
       </c>
       <c r="S4" t="n">
-        <v>162.3646754078567</v>
+        <v>162.4343014975651</v>
       </c>
       <c r="T4" t="inlineStr">
         <is>
@@ -23957,52 +23961,52 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>6.013999938964844</v>
+        <v>6.021999835968018</v>
       </c>
       <c r="E18" t="n">
-        <v>7.633106690253499</v>
+        <v>7.776281578246902</v>
       </c>
       <c r="F18" t="n">
-        <v>15.97723981961201</v>
+        <v>16.13151417656005</v>
       </c>
       <c r="G18" t="n">
-        <v>44.56731152781381</v>
+        <v>44.75961675128999</v>
       </c>
       <c r="H18" t="n">
-        <v>46.87995710620116</v>
+        <v>47.07533863939128</v>
       </c>
       <c r="I18" t="n">
-        <v>65.78920953257676</v>
+        <v>65.85966854010542</v>
       </c>
       <c r="J18" t="n">
         <v>53.34789996467301</v>
       </c>
       <c r="K18" t="n">
-        <v>0.9348535121808438</v>
+        <v>0.93731346849797</v>
       </c>
       <c r="L18" t="n">
-        <v>5.057142813639588</v>
+        <v>5.057904708592272</v>
       </c>
       <c r="M18" t="n">
-        <v>4.481990182069698</v>
+        <v>4.482303903520802</v>
       </c>
       <c r="N18" t="n">
-        <v>3.807719090009125</v>
+        <v>3.807854681483755</v>
       </c>
       <c r="O18" t="n">
-        <v>0.1148640463591136</v>
+        <v>0.1153745810966392</v>
       </c>
       <c r="P18" t="n">
-        <v>79.49782390490726</v>
+        <v>79.82983870457035</v>
       </c>
       <c r="Q18" t="n">
-        <v>-20.50217609509274</v>
+        <v>-20.17016129542965</v>
       </c>
       <c r="R18" t="n">
-        <v>124.0050188627805</v>
+        <v>124.2888534542797</v>
       </c>
       <c r="S18" t="n">
-        <v>45.09046964146333</v>
+        <v>45.28347077632426</v>
       </c>
       <c r="T18" t="inlineStr">
         <is>
@@ -27427,66 +27431,66 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>BRENT</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>Brent Crude</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Azioni USA</t>
+          <t>Commodities</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>255.0800018310547</v>
+        <v>106.3099975585938</v>
       </c>
       <c r="E56" t="n">
-        <v>22.47563095901051</v>
+        <v>-10.17321594487394</v>
       </c>
       <c r="F56" t="n">
-        <v>9.373124301489376</v>
+        <v>68.21201942284476</v>
       </c>
       <c r="G56" t="n">
-        <v>36.42101169087022</v>
+        <v>31.70217536038302</v>
       </c>
       <c r="H56" t="n">
-        <v>64.94392206425452</v>
+        <v>60.75911382727157</v>
       </c>
       <c r="I56" t="n">
-        <v>62.92456550332555</v>
+        <v>65.00310752322562</v>
       </c>
       <c r="J56" t="n">
-        <v>13.65055413465318</v>
+        <v>16.10599589638658</v>
       </c>
       <c r="K56" t="n">
-        <v>0.9549815854662987</v>
+        <v>1.077703114924796</v>
       </c>
       <c r="L56" t="n">
-        <v>214.6639378795472</v>
+        <v>78.4598087451072</v>
       </c>
       <c r="M56" t="n">
-        <v>183.4627893815327</v>
+        <v>77.18588945964973</v>
       </c>
       <c r="N56" t="n">
-        <v>127.480833899757</v>
+        <v>71.44769715473507</v>
       </c>
       <c r="O56" t="n">
-        <v>-1.126357538556324</v>
+        <v>4.788295119040685</v>
       </c>
       <c r="P56" t="n">
-        <v>96.1913493744069</v>
+        <v>78.54449515006372</v>
       </c>
       <c r="Q56" t="n">
-        <v>-3.808650625593097</v>
+        <v>-21.45550484993628</v>
       </c>
       <c r="R56" t="n">
-        <v>52.41063678735669</v>
+        <v>188.8115690294602</v>
       </c>
       <c r="S56" t="n">
-        <v>42.90196181011468</v>
+        <v>34.91115918963441</v>
       </c>
       <c r="T56" t="inlineStr">
         <is>
@@ -27495,15 +27499,19 @@
       </c>
       <c r="U56" t="inlineStr">
         <is>
-          <t>Morning Star</t>
-        </is>
-      </c>
-      <c r="V56" t="inlineStr"/>
+          <t>Doji</t>
+        </is>
+      </c>
+      <c r="V56" t="inlineStr">
+        <is>
+          <t>Inside Bar</t>
+        </is>
+      </c>
       <c r="W56" t="n">
-        <v>73.40000000000001</v>
+        <v>73.59999999999999</v>
       </c>
       <c r="X56" t="n">
-        <v>76.5</v>
+        <v>84.3</v>
       </c>
       <c r="Y56" t="inlineStr">
         <is>
@@ -27512,19 +27520,19 @@
       </c>
       <c r="Z56" t="inlineStr">
         <is>
-          <t>EMA e SMA allineate al rialzo — struttura bullish solida; mercato laterale — ATR basso (ADX 14); RSI in forza (63) — momentum positivo; morning star — inversione rialzista a 3 candele; vicino alla resistenza dei 20g (258.79)</t>
+          <t>EMA allineate al rialzo (EMA20&gt;EMA50&gt;EMA200); RSI in forza (65) — momentum positivo; doji — indecisione del mercato; favorito dal quadrante macro (Stagflazione)</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>CVX</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Chevron</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -27533,65 +27541,69 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>187.6000061035156</v>
+        <v>255.0800018310547</v>
       </c>
       <c r="E57" t="n">
-        <v>-9.328172238915034</v>
+        <v>22.47563095901051</v>
       </c>
       <c r="F57" t="n">
-        <v>24.13154240879054</v>
+        <v>9.373124301489376</v>
       </c>
       <c r="G57" t="n">
-        <v>16.90658981518865</v>
+        <v>36.42101169087022</v>
       </c>
       <c r="H57" t="n">
-        <v>87.60000610351561</v>
+        <v>64.94392206425452</v>
       </c>
       <c r="I57" t="n">
-        <v>59.73765559503357</v>
+        <v>62.92456550332555</v>
       </c>
       <c r="J57" t="n">
-        <v>19.62628180651337</v>
+        <v>13.65055413465318</v>
       </c>
       <c r="K57" t="n">
-        <v>0.8930101795376867</v>
+        <v>0.9549815854662987</v>
       </c>
       <c r="L57" t="n">
-        <v>164.9002285910118</v>
+        <v>214.6639378795472</v>
       </c>
       <c r="M57" t="n">
-        <v>153.4169062027084</v>
+        <v>183.4627893815327</v>
       </c>
       <c r="N57" t="n">
-        <v>135.7044086107842</v>
+        <v>127.480833899757</v>
       </c>
       <c r="O57" t="n">
-        <v>4.859897286472398</v>
+        <v>-1.126357538556324</v>
       </c>
       <c r="P57" t="n">
-        <v>67.20697204912196</v>
+        <v>96.1913493744069</v>
       </c>
       <c r="Q57" t="n">
-        <v>-32.79302795087804</v>
+        <v>-3.808650625593097</v>
       </c>
       <c r="R57" t="n">
-        <v>209.7963547107595</v>
+        <v>52.41063678735669</v>
       </c>
       <c r="S57" t="n">
-        <v>26.79960119846729</v>
+        <v>42.90196181011468</v>
       </c>
       <c r="T57" t="inlineStr">
         <is>
           <t>Trend Bullish</t>
         </is>
       </c>
-      <c r="U57" t="inlineStr"/>
+      <c r="U57" t="inlineStr">
+        <is>
+          <t>Morning Star</t>
+        </is>
+      </c>
       <c r="V57" t="inlineStr"/>
       <c r="W57" t="n">
-        <v>73.2</v>
+        <v>73.40000000000001</v>
       </c>
       <c r="X57" t="n">
-        <v>73.7</v>
+        <v>76.5</v>
       </c>
       <c r="Y57" t="inlineStr">
         <is>
@@ -27600,73 +27612,73 @@
       </c>
       <c r="Z57" t="inlineStr">
         <is>
-          <t>EMA allineate al rialzo (EMA20&gt;EMA50&gt;EMA200)</t>
+          <t>EMA e SMA allineate al rialzo — struttura bullish solida; mercato laterale — ATR basso (ADX 14); RSI in forza (63) — momentum positivo; morning star — inversione rialzista a 3 candele; vicino alla resistenza dei 20g (258.79)</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>USDJPY</t>
+          <t>CVX</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>USD/JPY</t>
+          <t>Chevron</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>FX/Macro</t>
+          <t>Azioni USA</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>159.7010040283203</v>
+        <v>187.6000061035156</v>
       </c>
       <c r="E58" t="n">
-        <v>-0.08758665589851944</v>
+        <v>-9.328172238915034</v>
       </c>
       <c r="F58" t="n">
-        <v>2.186409050843241</v>
+        <v>24.13154240879054</v>
       </c>
       <c r="G58" t="n">
-        <v>4.60536185478595</v>
+        <v>16.90658981518865</v>
       </c>
       <c r="H58" t="n">
-        <v>50.12456154594018</v>
+        <v>87.60000610351561</v>
       </c>
       <c r="I58" t="n">
-        <v>61.40295346179372</v>
+        <v>59.73765559503357</v>
       </c>
       <c r="J58" t="n">
-        <v>19.38458414734579</v>
+        <v>19.62628180651337</v>
       </c>
       <c r="K58" t="n">
-        <v>0.8810905071628335</v>
+        <v>0.8930101795376867</v>
       </c>
       <c r="L58" t="n">
-        <v>152.2322007828246</v>
+        <v>164.9002285910118</v>
       </c>
       <c r="M58" t="n">
-        <v>144.0925966740128</v>
+        <v>153.4169062027084</v>
       </c>
       <c r="N58" t="n">
-        <v>129.4370545060583</v>
+        <v>135.7044086107842</v>
       </c>
       <c r="O58" t="n">
-        <v>0.5621404182447947</v>
+        <v>4.859897286472398</v>
       </c>
       <c r="P58" t="n">
-        <v>97.39417541864319</v>
+        <v>67.20697204912196</v>
       </c>
       <c r="Q58" t="n">
-        <v>-2.605824581356808</v>
+        <v>-32.79302795087804</v>
       </c>
       <c r="R58" t="n">
-        <v>123.7304995275291</v>
+        <v>209.7963547107595</v>
       </c>
       <c r="S58" t="n">
-        <v>10.22224080410206</v>
+        <v>26.79960119846729</v>
       </c>
       <c r="T58" t="inlineStr">
         <is>
@@ -27674,16 +27686,12 @@
         </is>
       </c>
       <c r="U58" t="inlineStr"/>
-      <c r="V58" t="inlineStr">
-        <is>
-          <t>Double Top, Inside Bar</t>
-        </is>
-      </c>
+      <c r="V58" t="inlineStr"/>
       <c r="W58" t="n">
-        <v>73.09999999999999</v>
+        <v>73.2</v>
       </c>
       <c r="X58" t="n">
-        <v>75.7</v>
+        <v>73.7</v>
       </c>
       <c r="Y58" t="inlineStr">
         <is>
@@ -27692,94 +27700,90 @@
       </c>
       <c r="Z58" t="inlineStr">
         <is>
-          <t>EMA e SMA allineate al rialzo — struttura bullish solida; RSI in forza (61) — momentum positivo; pattern: Double Top; vicino alla resistenza dei 20g (160.23)</t>
+          <t>EMA allineate al rialzo (EMA20&gt;EMA50&gt;EMA200)</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>BRENT</t>
+          <t>USDJPY</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Brent Crude</t>
+          <t>USD/JPY</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Commodities</t>
+          <t>FX/Macro</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>105.9499969482422</v>
+        <v>159.7039947509766</v>
       </c>
       <c r="E59" t="n">
-        <v>-10.47739897401887</v>
+        <v>-0.08571559491147296</v>
       </c>
       <c r="F59" t="n">
-        <v>67.64239821081044</v>
+        <v>2.188322696975686</v>
       </c>
       <c r="G59" t="n">
-        <v>31.25618848611717</v>
+        <v>4.607320800677162</v>
       </c>
       <c r="H59" t="n">
-        <v>60.21473060437197</v>
+        <v>50.12737293044089</v>
       </c>
       <c r="I59" t="n">
-        <v>64.77322890740928</v>
+        <v>61.40715268314162</v>
       </c>
       <c r="J59" t="n">
-        <v>16.10599589638658</v>
+        <v>19.38458414734579</v>
       </c>
       <c r="K59" t="n">
-        <v>1.073400729188607</v>
+        <v>0.8812043137949481</v>
       </c>
       <c r="L59" t="n">
-        <v>78.42552297269276</v>
+        <v>152.2324856135537</v>
       </c>
       <c r="M59" t="n">
-        <v>77.17177178865555</v>
+        <v>144.0927139572542</v>
       </c>
       <c r="N59" t="n">
-        <v>71.44159544947487</v>
+        <v>129.437097849865</v>
       </c>
       <c r="O59" t="n">
-        <v>4.765320721115108</v>
+        <v>0.5623312791778434</v>
       </c>
       <c r="P59" t="n">
-        <v>77.95442696821428</v>
+        <v>97.40887978951743</v>
       </c>
       <c r="Q59" t="n">
-        <v>-22.04557303178573</v>
+        <v>-2.591120210482566</v>
       </c>
       <c r="R59" t="n">
-        <v>188.1633284875432</v>
+        <v>123.7440052557841</v>
       </c>
       <c r="S59" t="n">
-        <v>34.45430564089138</v>
+        <v>10.22430493735409</v>
       </c>
       <c r="T59" t="inlineStr">
         <is>
           <t>Trend Bullish</t>
         </is>
       </c>
-      <c r="U59" t="inlineStr">
-        <is>
-          <t>Doji</t>
-        </is>
-      </c>
+      <c r="U59" t="inlineStr"/>
       <c r="V59" t="inlineStr">
         <is>
-          <t>Inside Bar</t>
+          <t>Double Top, Inside Bar</t>
         </is>
       </c>
       <c r="W59" t="n">
-        <v>72.5</v>
+        <v>73.09999999999999</v>
       </c>
       <c r="X59" t="n">
-        <v>83.3</v>
+        <v>75.7</v>
       </c>
       <c r="Y59" t="inlineStr">
         <is>
@@ -27788,7 +27792,7 @@
       </c>
       <c r="Z59" t="inlineStr">
         <is>
-          <t>EMA allineate al rialzo (EMA20&gt;EMA50&gt;EMA200); RSI in forza (65) — momentum positivo; doji — indecisione del mercato; favorito dal quadrante macro (Stagflazione)</t>
+          <t>EMA e SMA allineate al rialzo — struttura bullish solida; RSI in forza (61) — momentum positivo; pattern: Double Top; vicino alla resistenza dei 20g (160.23)</t>
         </is>
       </c>
     </row>
@@ -27897,52 +27901,52 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>96.58000183105469</v>
+        <v>96.87999725341797</v>
       </c>
       <c r="E61" t="n">
-        <v>-4.734657281914112</v>
+        <v>-4.438745434911995</v>
       </c>
       <c r="F61" t="n">
-        <v>64.9530368736917</v>
+        <v>65.46541164102284</v>
       </c>
       <c r="G61" t="n">
-        <v>23.96354420661546</v>
+        <v>24.34859799722282</v>
       </c>
       <c r="H61" t="n">
-        <v>57.04065338382875</v>
+        <v>57.52845081856582</v>
       </c>
       <c r="I61" t="n">
-        <v>65.6297415939008</v>
+        <v>65.86742985864549</v>
       </c>
       <c r="J61" t="n">
         <v>13.82316078082327</v>
       </c>
       <c r="K61" t="n">
-        <v>1.111981457028275</v>
+        <v>1.116167662605136</v>
       </c>
       <c r="L61" t="n">
-        <v>72.52435628619564</v>
+        <v>72.55292727880166</v>
       </c>
       <c r="M61" t="n">
-        <v>71.99299292062291</v>
+        <v>72.0047574469901</v>
       </c>
       <c r="N61" t="n">
-        <v>66.87676509972745</v>
+        <v>66.88184976790309</v>
       </c>
       <c r="O61" t="n">
-        <v>3.845312370648817</v>
+        <v>3.864457377660046</v>
       </c>
       <c r="P61" t="n">
-        <v>64.49612376509533</v>
+        <v>64.96123291954615</v>
       </c>
       <c r="Q61" t="n">
-        <v>-35.50387623490467</v>
+        <v>-35.03876708045385</v>
       </c>
       <c r="R61" t="n">
-        <v>202.1864011256831</v>
+        <v>202.7450756476517</v>
       </c>
       <c r="S61" t="n">
-        <v>31.31202967196405</v>
+        <v>31.71990922317518</v>
       </c>
       <c r="T61" t="inlineStr">
         <is>
@@ -28687,7 +28691,7 @@
         <v>68.3</v>
       </c>
       <c r="X69" t="n">
-        <v>87.90000000000001</v>
+        <v>88</v>
       </c>
       <c r="Y69" t="inlineStr">
         <is>
@@ -29365,52 +29369,52 @@
         </is>
       </c>
       <c r="D77" t="n">
-        <v>1471.5</v>
+        <v>1471</v>
       </c>
       <c r="E77" t="n">
-        <v>0.02039483673759168</v>
+        <v>-0.01359102627183084</v>
       </c>
       <c r="F77" t="n">
-        <v>0.1974686410372239</v>
+        <v>0.1634226102383618</v>
       </c>
       <c r="G77" t="n">
-        <v>59.49490992187157</v>
+        <v>59.4407152531927</v>
       </c>
       <c r="H77" t="n">
-        <v>-36.30146150407359</v>
+        <v>-36.32310558783027</v>
       </c>
       <c r="I77" t="n">
-        <v>55.23745339744062</v>
+        <v>55.22166244806256</v>
       </c>
       <c r="J77" t="n">
         <v>50.9561631164703</v>
       </c>
       <c r="K77" t="n">
-        <v>0.7182811051501908</v>
+        <v>0.7178797939688665</v>
       </c>
       <c r="L77" t="n">
-        <v>1336.111355483811</v>
+        <v>1336.063736436192</v>
       </c>
       <c r="M77" t="n">
-        <v>1369.827698929935</v>
+        <v>1369.808091086798</v>
       </c>
       <c r="N77" t="n">
-        <v>1349.486304279362</v>
+        <v>1349.477829703091</v>
       </c>
       <c r="O77" t="n">
-        <v>66.95836992945976</v>
+        <v>66.92646109755086</v>
       </c>
       <c r="P77" t="n">
-        <v>45.99861270427996</v>
+        <v>45.95995191186397</v>
       </c>
       <c r="Q77" t="n">
-        <v>-54.00138729572004</v>
+        <v>-54.04004808813603</v>
       </c>
       <c r="R77" t="n">
-        <v>77.83665196299293</v>
+        <v>77.79281506144999</v>
       </c>
       <c r="S77" t="n">
-        <v>53.10582014143696</v>
+        <v>53.05379641729784</v>
       </c>
       <c r="T77" t="inlineStr">
         <is>
@@ -29557,52 +29561,52 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>1.435400009155273</v>
+        <v>1.437199950218201</v>
       </c>
       <c r="E79" t="n">
-        <v>7.098706766853091</v>
+        <v>7.233004773587481</v>
       </c>
       <c r="F79" t="n">
-        <v>-33.57603632843922</v>
+        <v>-33.49274301715857</v>
       </c>
       <c r="G79" t="n">
-        <v>130.0545502709745</v>
+        <v>130.3430305754923</v>
       </c>
       <c r="H79" t="n">
-        <v>245.9187021205569</v>
+        <v>246.352471991262</v>
       </c>
       <c r="I79" t="n">
-        <v>46.39784993687425</v>
+        <v>46.42702618655936</v>
       </c>
       <c r="J79" t="n">
         <v>49.98060633402685</v>
       </c>
       <c r="K79" t="n">
-        <v>0.2990179805502031</v>
+        <v>0.2996061183408909</v>
       </c>
       <c r="L79" t="n">
-        <v>1.762918928307223</v>
+        <v>1.763090351265597</v>
       </c>
       <c r="M79" t="n">
-        <v>1.360531971261543</v>
+        <v>1.36060396890406</v>
       </c>
       <c r="N79" t="n">
-        <v>1.075428187678744</v>
+        <v>1.075464921169824</v>
       </c>
       <c r="O79" t="n">
-        <v>-0.1741466774027312</v>
+        <v>-0.1740318093690857</v>
       </c>
       <c r="P79" t="n">
-        <v>11.99721788925251</v>
+        <v>12.06873636203969</v>
       </c>
       <c r="Q79" t="n">
-        <v>-88.00278211074749</v>
+        <v>-87.93126363796031</v>
       </c>
       <c r="R79" t="n">
-        <v>-45.54876878457257</v>
+        <v>-45.50765535274312</v>
       </c>
       <c r="S79" t="n">
-        <v>153.4640626887928</v>
+        <v>153.7818976975012</v>
       </c>
       <c r="T79" t="inlineStr">
         <is>
@@ -29615,7 +29619,7 @@
         <v>61.3</v>
       </c>
       <c r="X79" t="n">
-        <v>72.8</v>
+        <v>72.90000000000001</v>
       </c>
       <c r="Y79" t="inlineStr">
         <is>
@@ -29779,7 +29783,7 @@
         <v>2.285124380319148</v>
       </c>
       <c r="R81" t="n">
-        <v>66.93150196375541</v>
+        <v>63.23428322243683</v>
       </c>
       <c r="S81" t="n">
         <v>13.927498342446</v>
@@ -30105,52 +30109,52 @@
         </is>
       </c>
       <c r="D85" t="n">
-        <v>1.346545696258545</v>
+        <v>1.346590995788574</v>
       </c>
       <c r="E85" t="n">
-        <v>2.221672003247743</v>
+        <v>2.225110871838254</v>
       </c>
       <c r="F85" t="n">
-        <v>1.69381903385486</v>
+        <v>1.697240144792223</v>
       </c>
       <c r="G85" t="n">
-        <v>4.895903136129753</v>
+        <v>4.899431969296919</v>
       </c>
       <c r="H85" t="n">
-        <v>-3.874140597010101</v>
+        <v>-3.870906799399876</v>
       </c>
       <c r="I85" t="n">
-        <v>54.87132244777467</v>
+        <v>54.87723714436931</v>
       </c>
       <c r="J85" t="n">
         <v>21.65217664783298</v>
       </c>
       <c r="K85" t="n">
-        <v>0.6622163110508387</v>
+        <v>0.6624826202997071</v>
       </c>
       <c r="L85" t="n">
-        <v>1.323290692779642</v>
+        <v>1.323295007020597</v>
       </c>
       <c r="M85" t="n">
-        <v>1.304221407834189</v>
+        <v>1.304223184286347</v>
       </c>
       <c r="N85" t="n">
-        <v>1.345124427646793</v>
+        <v>1.345125084161721</v>
       </c>
       <c r="O85" t="n">
-        <v>-6.300037372937786e-05</v>
+        <v>-6.010946355093638e-05</v>
       </c>
       <c r="P85" t="n">
-        <v>69.79203753353738</v>
+        <v>69.82792406787088</v>
       </c>
       <c r="Q85" t="n">
-        <v>-30.20796246646262</v>
+        <v>-30.17207593212912</v>
       </c>
       <c r="R85" t="n">
-        <v>41.32949905361538</v>
+        <v>41.35426252014096</v>
       </c>
       <c r="S85" t="n">
-        <v>2.27283551137758</v>
+        <v>2.276276101174335</v>
       </c>
       <c r="T85" t="inlineStr">
         <is>
@@ -30193,52 +30197,52 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>77984</v>
+        <v>77989.5390625</v>
       </c>
       <c r="E86" t="n">
-        <v>14.2902156479652</v>
+        <v>14.29833347530944</v>
       </c>
       <c r="F86" t="n">
-        <v>-13.72908555502317</v>
+        <v>-13.72295788797553</v>
       </c>
       <c r="G86" t="n">
-        <v>20.68230442167</v>
+        <v>20.69087626752091</v>
       </c>
       <c r="H86" t="n">
-        <v>72.76883818109296</v>
+        <v>72.78110963924769</v>
       </c>
       <c r="I86" t="n">
-        <v>49.38967118925057</v>
+        <v>49.39228680533802</v>
       </c>
       <c r="J86" t="n">
         <v>33.80484147146453</v>
       </c>
       <c r="K86" t="n">
-        <v>0.3053373688496108</v>
+        <v>0.3054145894168231</v>
       </c>
       <c r="L86" t="n">
-        <v>83085.3881895946</v>
+        <v>83085.9157193565</v>
       </c>
       <c r="M86" t="n">
-        <v>66675.34648353454</v>
+        <v>66675.56804603455</v>
       </c>
       <c r="N86" t="n">
-        <v>49323.88603403579</v>
+        <v>49323.99907612763</v>
       </c>
       <c r="O86" t="n">
-        <v>-5640.348204655376</v>
+        <v>-5639.994714626881</v>
       </c>
       <c r="P86" t="n">
-        <v>27.08522298645239</v>
+        <v>27.09359978402276</v>
       </c>
       <c r="Q86" t="n">
-        <v>-72.91477701354761</v>
+        <v>-72.90640021597723</v>
       </c>
       <c r="R86" t="n">
-        <v>-43.08210346123076</v>
+        <v>-43.0776726682994</v>
       </c>
       <c r="S86" t="n">
-        <v>32.24374141097146</v>
+        <v>32.25313444478493</v>
       </c>
       <c r="T86" t="inlineStr">
         <is>
@@ -31099,52 +31103,52 @@
         </is>
       </c>
       <c r="D96" t="n">
-        <v>2326.219970703125</v>
+        <v>2328.590087890625</v>
       </c>
       <c r="E96" t="n">
-        <v>10.52458071300104</v>
+        <v>10.63719096125282</v>
       </c>
       <c r="F96" t="n">
-        <v>-22.25493083092078</v>
+        <v>-22.1757186639711</v>
       </c>
       <c r="G96" t="n">
-        <v>-28.00968343426603</v>
+        <v>-27.9363346156784</v>
       </c>
       <c r="H96" t="n">
-        <v>64.27539248429757</v>
+        <v>64.4427678555496</v>
       </c>
       <c r="I96" t="n">
-        <v>46.14582702507994</v>
+        <v>46.16827413685184</v>
       </c>
       <c r="J96" t="n">
         <v>14.24892668051552</v>
       </c>
       <c r="K96" t="n">
-        <v>0.3297677937600152</v>
+        <v>0.3304671442883174</v>
       </c>
       <c r="L96" t="n">
-        <v>2760.705221208311</v>
+        <v>2760.930946654739</v>
       </c>
       <c r="M96" t="n">
-        <v>2511.34928295289</v>
+        <v>2511.444087640389</v>
       </c>
       <c r="N96" t="n">
-        <v>2059.847988951689</v>
+        <v>2059.89635869021</v>
       </c>
       <c r="O96" t="n">
-        <v>-154.4891367952573</v>
+        <v>-154.3378814533772</v>
       </c>
       <c r="P96" t="n">
-        <v>26.33692581053185</v>
+        <v>26.40337272144864</v>
       </c>
       <c r="Q96" t="n">
-        <v>-73.66307418946815</v>
+        <v>-73.59662727855137</v>
       </c>
       <c r="R96" t="n">
-        <v>-69.39449605650846</v>
+        <v>-69.31298988267595</v>
       </c>
       <c r="S96" t="n">
-        <v>-7.447055380349477</v>
+        <v>-7.352755904135078</v>
       </c>
       <c r="T96" t="inlineStr">
         <is>
@@ -31154,7 +31158,7 @@
       <c r="U96" t="inlineStr"/>
       <c r="V96" t="inlineStr"/>
       <c r="W96" t="n">
-        <v>44.9</v>
+        <v>45</v>
       </c>
       <c r="X96" t="n">
         <v>64.2</v>
@@ -31187,52 +31191,52 @@
         </is>
       </c>
       <c r="D97" t="n">
-        <v>98.81999969482422</v>
+        <v>98.81400299072266</v>
       </c>
       <c r="E97" t="n">
-        <v>-1.140455582322553</v>
+        <v>-1.146454686120557</v>
       </c>
       <c r="F97" t="n">
-        <v>-0.6434741559819268</v>
+        <v>-0.6495034181544179</v>
       </c>
       <c r="G97" t="n">
-        <v>-5.07204501122972</v>
+        <v>-5.077805533986169</v>
       </c>
       <c r="H97" t="n">
-        <v>8.677003588659771</v>
+        <v>8.670408730987456</v>
       </c>
       <c r="I97" t="n">
-        <v>45.44217860270738</v>
+        <v>45.43027834323288</v>
       </c>
       <c r="J97" t="n">
         <v>28.5699342843782</v>
       </c>
       <c r="K97" t="n">
-        <v>0.3547321343339674</v>
+        <v>0.3543708290425597</v>
       </c>
       <c r="L97" t="n">
-        <v>100.289805698223</v>
+        <v>100.2892345835467</v>
       </c>
       <c r="M97" t="n">
-        <v>100.9220092255089</v>
+        <v>100.9217740606422</v>
       </c>
       <c r="N97" t="n">
-        <v>99.52923559294915</v>
+        <v>99.52913395389658</v>
       </c>
       <c r="O97" t="n">
-        <v>-0.1954476014595103</v>
+        <v>-0.1958302971058732</v>
       </c>
       <c r="P97" t="n">
-        <v>27.22729507665608</v>
+        <v>27.17736412874308</v>
       </c>
       <c r="Q97" t="n">
-        <v>-72.77270492334392</v>
+        <v>-72.82263587125692</v>
       </c>
       <c r="R97" t="n">
-        <v>-42.06031618104782</v>
+        <v>-42.09558438194849</v>
       </c>
       <c r="S97" t="n">
-        <v>-2.831855791385796</v>
+        <v>-2.837752255772719</v>
       </c>
       <c r="T97" t="inlineStr">
         <is>
@@ -31739,52 +31743,52 @@
         </is>
       </c>
       <c r="D103" t="n">
-        <v>85.80000305175781</v>
+        <v>85.84999847412109</v>
       </c>
       <c r="E103" t="n">
-        <v>3.241074715434689</v>
+        <v>3.30123300158911</v>
       </c>
       <c r="F103" t="n">
-        <v>-35.76152501958118</v>
+        <v>-35.72409343946011</v>
       </c>
       <c r="G103" t="n">
-        <v>-50.06580794133701</v>
+        <v>-50.03671142696003</v>
       </c>
       <c r="H103" t="n">
-        <v>555.4999282335172</v>
+        <v>555.8818862126021</v>
       </c>
       <c r="I103" t="n">
-        <v>42.32490960945398</v>
+        <v>42.33417041384887</v>
       </c>
       <c r="J103" t="n">
         <v>32.80032248447666</v>
       </c>
       <c r="K103" t="n">
-        <v>0.1247279232522633</v>
+        <v>0.1249537856907138</v>
       </c>
       <c r="L103" t="n">
-        <v>132.3976653582657</v>
+        <v>132.4024268270622</v>
       </c>
       <c r="M103" t="n">
-        <v>123.8117791209574</v>
+        <v>123.8144815762203</v>
       </c>
       <c r="N103" t="n">
-        <v>96.99375715270072</v>
+        <v>96.99514591443304</v>
       </c>
       <c r="O103" t="n">
-        <v>-14.86159507593995</v>
+        <v>-14.85840448488314</v>
       </c>
       <c r="P103" t="n">
-        <v>9.2718202249198</v>
+        <v>9.298915359397753</v>
       </c>
       <c r="Q103" t="n">
-        <v>-90.72817977508021</v>
+        <v>-90.70108464060225</v>
       </c>
       <c r="R103" t="n">
-        <v>-97.80925477426443</v>
+        <v>-97.78963365577775</v>
       </c>
       <c r="S103" t="n">
-        <v>-49.05895221588102</v>
+        <v>-49.02926900948232</v>
       </c>
       <c r="T103" t="inlineStr">
         <is>
@@ -32015,52 +32019,52 @@
         </is>
       </c>
       <c r="D106" t="n">
-        <v>0.2486999928951263</v>
+        <v>0.2489999979734421</v>
       </c>
       <c r="E106" t="n">
-        <v>2.954502736687936</v>
+        <v>3.07869604002069</v>
       </c>
       <c r="F106" t="n">
-        <v>-40.19981676536041</v>
+        <v>-40.12768021864902</v>
       </c>
       <c r="G106" t="n">
-        <v>-36.02950910831589</v>
+        <v>-35.95234194837171</v>
       </c>
       <c r="H106" t="n">
-        <v>-80.98709635850267</v>
+        <v>-80.96416122457052</v>
       </c>
       <c r="I106" t="n">
-        <v>39.48447979299285</v>
+        <v>39.49800551865223</v>
       </c>
       <c r="J106" t="n">
         <v>29.80750264091312</v>
       </c>
       <c r="K106" t="n">
-        <v>0.1699735180971987</v>
+        <v>0.1702301843703743</v>
       </c>
       <c r="L106" t="n">
-        <v>0.4871927917150218</v>
+        <v>0.4872213636272424</v>
       </c>
       <c r="M106" t="n">
-        <v>0.5335897983377687</v>
+        <v>0.5336017985409013</v>
       </c>
       <c r="N106" t="n">
-        <v>0.5090743513687783</v>
+        <v>0.509080473921397</v>
       </c>
       <c r="O106" t="n">
-        <v>-0.05469933624549636</v>
+        <v>-0.05468019062226485</v>
       </c>
       <c r="P106" t="n">
-        <v>2.473706187543452</v>
+        <v>2.506745301058727</v>
       </c>
       <c r="Q106" t="n">
-        <v>-97.52629381245654</v>
+        <v>-97.49325469894127</v>
       </c>
       <c r="R106" t="n">
-        <v>-102.6004514988219</v>
+        <v>-102.5748049927999</v>
       </c>
       <c r="S106" t="n">
-        <v>-27.98651891726765</v>
+        <v>-27.89964955398172</v>
       </c>
       <c r="T106" t="inlineStr">
         <is>
@@ -32354,7 +32358,7 @@
         </is>
       </c>
       <c r="W109" t="n">
-        <v>32.1</v>
+        <v>32</v>
       </c>
       <c r="X109" t="n">
         <v>74.8</v>
@@ -33027,52 +33031,52 @@
         </is>
       </c>
       <c r="D117" t="n">
-        <v>1.235000014305115</v>
+        <v>1.235999941825867</v>
       </c>
       <c r="E117" t="n">
-        <v>-1.327882202231567</v>
+        <v>-1.247991542333571</v>
       </c>
       <c r="F117" t="n">
-        <v>-44.33371472515233</v>
+        <v>-44.28864407739557</v>
       </c>
       <c r="G117" t="n">
-        <v>-77.06732979418189</v>
+        <v>-77.04876217653209</v>
       </c>
       <c r="H117" t="n">
-        <v>-96.32519850303197</v>
+        <v>-96.32222317096108</v>
       </c>
       <c r="I117" t="n">
-        <v>35.30708939798467</v>
+        <v>35.31021235038629</v>
       </c>
       <c r="J117" t="n">
         <v>25.5772157418073</v>
       </c>
       <c r="K117" t="n">
-        <v>0.1815952279135867</v>
+        <v>0.181705723977823</v>
       </c>
       <c r="L117" t="n">
-        <v>3.425224469559719</v>
+        <v>3.425319700752172</v>
       </c>
       <c r="M117" t="n">
-        <v>4.826951096628476</v>
+        <v>4.827008235343948</v>
       </c>
       <c r="N117" t="n">
-        <v>6.781627045858009</v>
+        <v>6.781656455490972</v>
       </c>
       <c r="O117" t="n">
-        <v>-0.1105947549602722</v>
+        <v>-0.1105309419219112</v>
       </c>
       <c r="P117" t="n">
-        <v>2.471239589319516</v>
+        <v>2.494845668363295</v>
       </c>
       <c r="Q117" t="n">
-        <v>-97.52876041068049</v>
+        <v>-97.5051543316367</v>
       </c>
       <c r="R117" t="n">
-        <v>-86.44297523452234</v>
+        <v>-86.43323545322041</v>
       </c>
       <c r="S117" t="n">
-        <v>-86.22768923972298</v>
+        <v>-86.21653837948489</v>
       </c>
       <c r="T117" t="inlineStr">
         <is>
@@ -33356,7 +33360,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>23/04/2026 20:39:48</t>
+          <t>23/04/2026 20:47:08</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -33396,13 +33400,13 @@
         <v>19.30999946594238</v>
       </c>
       <c r="N2" t="n">
-        <v>98.81999969482422</v>
+        <v>98.81400299072266</v>
       </c>
       <c r="O2" t="n">
-        <v>4705.39990234375</v>
+        <v>4705.2001953125</v>
       </c>
       <c r="P2" t="n">
-        <v>96.58000183105469</v>
+        <v>96.87999725341797</v>
       </c>
       <c r="Q2" t="n">
         <v>2.787751808934846</v>
@@ -33419,7 +33423,7 @@
         <v>2.30287058551863</v>
       </c>
       <c r="U2" t="n">
-        <v>2.831622076043044</v>
+        <v>2.866040961520563</v>
       </c>
       <c r="V2" t="n">
         <v>0.008443311100047646</v>
@@ -33443,10 +33447,10 @@
         <v>-0.09933745989944809</v>
       </c>
       <c r="AC2" t="n">
-        <v>0.6619492385047592</v>
+        <v>0.6619211439920709</v>
       </c>
       <c r="AD2" t="n">
-        <v>-8.006460690483831</v>
+        <v>-8.010365089049509</v>
       </c>
       <c r="AE2" t="n">
         <v>1.215636666136732</v>
@@ -33470,7 +33474,7 @@
         <v>95</v>
       </c>
       <c r="AJ2" t="n">
-        <v>1.216706788968712</v>
+        <v>1.222443269881632</v>
       </c>
       <c r="AK2" t="inlineStr">
         <is>
@@ -33569,10 +33573,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>79.89203854716712</v>
+        <v>79.89254221614779</v>
       </c>
       <c r="C2" t="n">
-        <v>0.1991298177487536</v>
+        <v>0.1991499645079799</v>
       </c>
       <c r="D2" t="n">
         <v>69.82758620689656</v>
@@ -33754,22 +33758,22 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>DAX</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
           <t>CAC40</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>FTSEMIB</t>
-        </is>
-      </c>
       <c r="C8" t="n">
-        <v>0.946</v>
+        <v>0.944</v>
       </c>
       <c r="D8" t="n">
         <v>0.945</v>
       </c>
       <c r="E8" t="n">
-        <v>0.903</v>
+        <v>0.895</v>
       </c>
     </row>
     <row r="9">
@@ -33784,7 +33788,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.946</v>
+        <v>0.947</v>
       </c>
       <c r="D9" t="n">
         <v>0.945</v>
@@ -33796,22 +33800,22 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>DAX</t>
+          <t>CAC40</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>CAC40</t>
+          <t>FTSEMIB</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.944</v>
+        <v>0.946</v>
       </c>
       <c r="D10" t="n">
         <v>0.945</v>
       </c>
       <c r="E10" t="n">
-        <v>0.895</v>
+        <v>0.903</v>
       </c>
     </row>
     <row r="11">
@@ -33868,7 +33872,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0.918</v>
+        <v>0.919</v>
       </c>
       <c r="D13" t="n">
         <v>0.9409999999999999</v>
@@ -33955,7 +33959,7 @@
         <v>0.951</v>
       </c>
       <c r="D17" t="n">
-        <v>0.9370000000000001</v>
+        <v>0.9360000000000001</v>
       </c>
       <c r="E17" t="n">
         <v>0.952</v>
@@ -34036,7 +34040,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>0.876</v>
+        <v>0.877</v>
       </c>
       <c r="D21" t="n">
         <v>0.9340000000000001</v>
@@ -34104,7 +34108,7 @@
         <v>-0.853</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.6919999999999999</v>
+        <v>-0.6929999999999999</v>
       </c>
     </row>
     <row r="3">
@@ -34161,7 +34165,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>-0.87</v>
+        <v>-0.871</v>
       </c>
       <c r="D5" t="n">
         <v>-0.803</v>
@@ -34182,7 +34186,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>-0.9389999999999999</v>
+        <v>-0.9399999999999999</v>
       </c>
       <c r="D6" t="n">
         <v>-0.797</v>
@@ -34203,13 +34207,13 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>-0.878</v>
+        <v>-0.877</v>
       </c>
       <c r="D7" t="n">
-        <v>-0.764</v>
+        <v>-0.763</v>
       </c>
       <c r="E7" t="n">
-        <v>-0.718</v>
+        <v>-0.717</v>
       </c>
     </row>
     <row r="8">
@@ -34224,7 +34228,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>-0.83</v>
+        <v>-0.831</v>
       </c>
       <c r="D8" t="n">
         <v>-0.742</v>
@@ -34245,13 +34249,13 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>-0.91</v>
+        <v>-0.909</v>
       </c>
       <c r="D9" t="n">
         <v>-0.739</v>
       </c>
       <c r="E9" t="n">
-        <v>-0.614</v>
+        <v>-0.613</v>
       </c>
     </row>
     <row r="10">
@@ -34287,13 +34291,13 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>-0.835</v>
+        <v>-0.832</v>
       </c>
       <c r="D11" t="n">
-        <v>-0.737</v>
+        <v>-0.735</v>
       </c>
       <c r="E11" t="n">
-        <v>-0.679</v>
+        <v>-0.677</v>
       </c>
     </row>
     <row r="12">
@@ -34341,43 +34345,43 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ITA</t>
+          <t>CVX</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>CVX</t>
+          <t>ISP</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>-0.834</v>
+        <v>-0.884</v>
       </c>
       <c r="D14" t="n">
         <v>-0.716</v>
       </c>
       <c r="E14" t="n">
-        <v>-0.5</v>
+        <v>-0.442</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>ITA</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
           <t>CVX</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>ISP</t>
-        </is>
-      </c>
       <c r="C15" t="n">
-        <v>-0.884</v>
+        <v>-0.834</v>
       </c>
       <c r="D15" t="n">
         <v>-0.716</v>
       </c>
       <c r="E15" t="n">
-        <v>-0.442</v>
+        <v>-0.5</v>
       </c>
     </row>
     <row r="16">
@@ -34398,7 +34402,7 @@
         <v>-0.713</v>
       </c>
       <c r="E16" t="n">
-        <v>-0.575</v>
+        <v>-0.576</v>
       </c>
     </row>
     <row r="17">
@@ -34425,43 +34429,43 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CAC40</t>
+          <t>CVX</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>WTI</t>
+          <t>PST</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>-0.8110000000000001</v>
+        <v>-0.859</v>
       </c>
       <c r="D18" t="n">
-        <v>-0.707</v>
+        <v>-0.706</v>
       </c>
       <c r="E18" t="n">
-        <v>-0.653</v>
+        <v>-0.482</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>CVX</t>
+          <t>CAC40</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>PST</t>
+          <t>WTI</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>-0.859</v>
+        <v>-0.8090000000000001</v>
       </c>
       <c r="D19" t="n">
-        <v>-0.706</v>
+        <v>-0.705</v>
       </c>
       <c r="E19" t="n">
-        <v>-0.482</v>
+        <v>-0.652</v>
       </c>
     </row>
     <row r="20">
@@ -34476,13 +34480,13 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>-0.842</v>
+        <v>-0.843</v>
       </c>
       <c r="D20" t="n">
         <v>-0.702</v>
       </c>
       <c r="E20" t="n">
-        <v>-0.61</v>
+        <v>-0.611</v>
       </c>
     </row>
     <row r="21">

</xml_diff>

<commit_message>
📊 Dashboard aggiornata 25/05/2026 21:08
</commit_message>
<xml_diff>
--- a/docs/sarada_dati.xlsx
+++ b/docs/sarada_dati.xlsx
@@ -4029,52 +4029,52 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>158.8950042724609</v>
+        <v>158.8699951171875</v>
       </c>
       <c r="E40" t="n">
-        <v>-0.07735042226556521</v>
+        <v>-0.09307766976502929</v>
       </c>
       <c r="F40" t="n">
-        <v>0.03211335254562631</v>
+        <v>0.01636887608069681</v>
       </c>
       <c r="G40" t="n">
-        <v>-0.5333369502995455</v>
+        <v>-0.5489924281550596</v>
       </c>
       <c r="H40" t="n">
-        <v>1.725356835385705</v>
+        <v>1.709345852183364</v>
       </c>
       <c r="I40" t="n">
-        <v>54.76459884869266</v>
+        <v>54.50652682675082</v>
       </c>
       <c r="J40" t="n">
         <v>33.09448640353283</v>
       </c>
       <c r="K40" t="n">
-        <v>0.6742329447990199</v>
+        <v>0.6689404375208198</v>
       </c>
       <c r="L40" t="n">
-        <v>158.4361842426812</v>
+        <v>158.4338024183694</v>
       </c>
       <c r="M40" t="n">
-        <v>158.2621354345381</v>
+        <v>158.2611546833509</v>
       </c>
       <c r="N40" t="n">
-        <v>155.3618645600413</v>
+        <v>155.3616157127251</v>
       </c>
       <c r="O40" t="n">
-        <v>0.1802107081245447</v>
+        <v>0.1786146822609305</v>
       </c>
       <c r="P40" t="n">
-        <v>90.09624728478336</v>
+        <v>89.51068937921573</v>
       </c>
       <c r="Q40" t="n">
-        <v>-9.903752715216646</v>
+        <v>-10.48931062078427</v>
       </c>
       <c r="R40" t="n">
-        <v>52.12432931203905</v>
+        <v>51.65910227229956</v>
       </c>
       <c r="S40" t="n">
-        <v>-0.4267557393770272</v>
+        <v>-0.442427992499117</v>
       </c>
       <c r="T40" t="inlineStr">
         <is>
@@ -4091,7 +4091,7 @@
         <v>65</v>
       </c>
       <c r="X40" t="n">
-        <v>64.8</v>
+        <v>64.7</v>
       </c>
       <c r="Y40" t="inlineStr">
         <is>
@@ -4391,87 +4391,79 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>GBPUSD</t>
+          <t>RUSSELL</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>GBP/USD</t>
+          <t>Russell 2000</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>FX/Macro</t>
+          <t>Indici</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>1.350894927978516</v>
+        <v>2869.22998046875</v>
       </c>
       <c r="E44" t="n">
-        <v>0.5687233738171482</v>
+        <v>0.9066461425231154</v>
       </c>
       <c r="F44" t="n">
-        <v>1.506247194658594</v>
+        <v>2.718287699614663</v>
       </c>
       <c r="G44" t="n">
-        <v>0.316109025346889</v>
+        <v>3.391945497461468</v>
       </c>
       <c r="H44" t="n">
-        <v>-0.3620407930712166</v>
+        <v>8.177711519867925</v>
       </c>
       <c r="I44" t="n">
-        <v>52.47966055424565</v>
+        <v>60.71352792032251</v>
       </c>
       <c r="J44" t="n">
-        <v>17.35609375318657</v>
+        <v>13.05303816711215</v>
       </c>
       <c r="K44" t="n">
-        <v>0.5045191463318871</v>
+        <v>0.7840385659005626</v>
       </c>
       <c r="L44" t="n">
-        <v>1.347630609003021</v>
+        <v>2805.192564353292</v>
       </c>
       <c r="M44" t="n">
-        <v>1.346658048343221</v>
+        <v>2732.449646245859</v>
       </c>
       <c r="N44" t="n">
-        <v>1.339997511575461</v>
+        <v>2549.071487220237</v>
       </c>
       <c r="O44" t="n">
-        <v>-0.001181149147536233</v>
+        <v>-7.660916487861996</v>
       </c>
       <c r="P44" t="n">
-        <v>58.80177666888293</v>
+        <v>88.30298942258695</v>
       </c>
       <c r="Q44" t="n">
-        <v>-41.19822333111707</v>
+        <v>-11.69701057741305</v>
       </c>
       <c r="R44" t="n">
-        <v>-20.37251384402821</v>
+        <v>52.38472041406454</v>
       </c>
       <c r="S44" t="n">
-        <v>-0.04553116309100602</v>
+        <v>2.9504836910208</v>
       </c>
       <c r="T44" t="inlineStr">
         <is>
           <t>Trend Bullish</t>
         </is>
       </c>
-      <c r="U44" t="inlineStr">
-        <is>
-          <t>Morning Star</t>
-        </is>
-      </c>
-      <c r="V44" t="inlineStr">
-        <is>
-          <t>Double Top, Double Bottom, Volatility Squeeze</t>
-        </is>
-      </c>
+      <c r="U44" t="inlineStr"/>
+      <c r="V44" t="inlineStr"/>
       <c r="W44" t="n">
-        <v>64.09999999999999</v>
+        <v>63.7</v>
       </c>
       <c r="X44" t="n">
-        <v>71</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="Y44" t="inlineStr">
         <is>
@@ -4480,73 +4472,73 @@
       </c>
       <c r="Z44" t="inlineStr">
         <is>
-          <t>EMA e SMA allineate al rialzo — struttura bullish solida; pattern: Double Bottom; morning star — inversione rialzista a 3 candele; vicino alla resistenza dei 20g (1.3658); in zona Fib Fib 50.0 — livello strutturale</t>
+          <t>EMA e SMA allineate al rialzo — struttura bullish solida; mercato laterale — ATR basso (ADX 13); RSI in forza (61) — momentum positivo; vicino alla resistenza dei 20g (2,889)</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>RUSSELL</t>
+          <t>ENEL</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Russell 2000</t>
+          <t>Enel</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Indici</t>
+          <t>Azioni IT</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>2869.22998046875</v>
+        <v>9.798999786376953</v>
       </c>
       <c r="E45" t="n">
-        <v>0.9066461425231154</v>
+        <v>1.041450119922227</v>
       </c>
       <c r="F45" t="n">
-        <v>2.718287699614663</v>
+        <v>1.903074121895165</v>
       </c>
       <c r="G45" t="n">
-        <v>3.391945497461468</v>
+        <v>-0.8599761195469902</v>
       </c>
       <c r="H45" t="n">
-        <v>8.177711519867925</v>
+        <v>1.020618340809198</v>
       </c>
       <c r="I45" t="n">
-        <v>60.71352792032251</v>
+        <v>53.39541032032729</v>
       </c>
       <c r="J45" t="n">
-        <v>13.05303816711215</v>
+        <v>15.43450372025413</v>
       </c>
       <c r="K45" t="n">
-        <v>0.7840385659005626</v>
+        <v>0.660015299924777</v>
       </c>
       <c r="L45" t="n">
-        <v>2805.192564353292</v>
+        <v>9.705887222038715</v>
       </c>
       <c r="M45" t="n">
-        <v>2732.449646245859</v>
+        <v>9.647664188668227</v>
       </c>
       <c r="N45" t="n">
-        <v>2549.071487220237</v>
+        <v>9.022449951291634</v>
       </c>
       <c r="O45" t="n">
-        <v>-7.660916487861996</v>
+        <v>-4.945930047958735e-05</v>
       </c>
       <c r="P45" t="n">
-        <v>88.30298942258695</v>
+        <v>79.2421200152085</v>
       </c>
       <c r="Q45" t="n">
-        <v>-11.69701057741305</v>
+        <v>-20.7578799847915</v>
       </c>
       <c r="R45" t="n">
-        <v>52.38472041406454</v>
+        <v>64.58943997632123</v>
       </c>
       <c r="S45" t="n">
-        <v>2.9504836910208</v>
+        <v>-0.2240129577741112</v>
       </c>
       <c r="T45" t="inlineStr">
         <is>
@@ -4554,12 +4546,16 @@
         </is>
       </c>
       <c r="U45" t="inlineStr"/>
-      <c r="V45" t="inlineStr"/>
+      <c r="V45" t="inlineStr">
+        <is>
+          <t>Double Top</t>
+        </is>
+      </c>
       <c r="W45" t="n">
-        <v>63.7</v>
+        <v>63.3</v>
       </c>
       <c r="X45" t="n">
-        <v>65.40000000000001</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="Y45" t="inlineStr">
         <is>
@@ -4568,19 +4564,19 @@
       </c>
       <c r="Z45" t="inlineStr">
         <is>
-          <t>EMA e SMA allineate al rialzo — struttura bullish solida; mercato laterale — ATR basso (ADX 13); RSI in forza (61) — momentum positivo; vicino alla resistenza dei 20g (2,889)</t>
+          <t>EMA e SMA allineate al rialzo — struttura bullish solida; pattern: Double Top; in zona Fib Fib 23.6 — livello strutturale</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>ENEL</t>
+          <t>TRN</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Enel</t>
+          <t>Terna</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -4589,52 +4585,52 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>9.798999786376953</v>
+        <v>10.0600004196167</v>
       </c>
       <c r="E46" t="n">
-        <v>1.041450119922227</v>
+        <v>1.105533793569857</v>
       </c>
       <c r="F46" t="n">
-        <v>1.903074121895165</v>
+        <v>2.402280663894762</v>
       </c>
       <c r="G46" t="n">
-        <v>-0.8599761195469902</v>
+        <v>-1.613691498261938</v>
       </c>
       <c r="H46" t="n">
-        <v>1.020618340809198</v>
+        <v>0.6402573813874657</v>
       </c>
       <c r="I46" t="n">
-        <v>53.39541032032729</v>
+        <v>52.3494035573238</v>
       </c>
       <c r="J46" t="n">
-        <v>15.43450372025413</v>
+        <v>21.29316607990519</v>
       </c>
       <c r="K46" t="n">
-        <v>0.660015299924777</v>
+        <v>0.5637879203323768</v>
       </c>
       <c r="L46" t="n">
-        <v>9.705887222038715</v>
+        <v>9.994018438594653</v>
       </c>
       <c r="M46" t="n">
-        <v>9.647664188668227</v>
+        <v>9.948721105623312</v>
       </c>
       <c r="N46" t="n">
-        <v>9.022449951291634</v>
+        <v>9.382881526154984</v>
       </c>
       <c r="O46" t="n">
-        <v>-4.945930047958735e-05</v>
+        <v>0.0004422470774380835</v>
       </c>
       <c r="P46" t="n">
-        <v>79.2421200152085</v>
+        <v>66.28414822031093</v>
       </c>
       <c r="Q46" t="n">
-        <v>-20.7578799847915</v>
+        <v>-33.71585177968907</v>
       </c>
       <c r="R46" t="n">
-        <v>64.58943997632123</v>
+        <v>11.95326061216765</v>
       </c>
       <c r="S46" t="n">
-        <v>-0.2240129577741112</v>
+        <v>-1.372543061434861</v>
       </c>
       <c r="T46" t="inlineStr">
         <is>
@@ -4644,14 +4640,14 @@
       <c r="U46" t="inlineStr"/>
       <c r="V46" t="inlineStr">
         <is>
-          <t>Double Top</t>
+          <t>Double Top, Inside Bar</t>
         </is>
       </c>
       <c r="W46" t="n">
-        <v>63.3</v>
+        <v>62.8</v>
       </c>
       <c r="X46" t="n">
-        <v>69.40000000000001</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="Y46" t="inlineStr">
         <is>
@@ -4660,90 +4656,94 @@
       </c>
       <c r="Z46" t="inlineStr">
         <is>
-          <t>EMA e SMA allineate al rialzo — struttura bullish solida; pattern: Double Top; in zona Fib Fib 23.6 — livello strutturale</t>
+          <t>EMA e SMA allineate al rialzo — struttura bullish solida; trend in sviluppo (ADX 21); pattern: Double Top; in zona Fib Fib 23.6 — livello strutturale</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>TRN</t>
+          <t>CORN</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Terna</t>
+          <t>Corn</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Azioni IT</t>
+          <t>Commodities</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>10.0600004196167</v>
+        <v>463.25</v>
       </c>
       <c r="E47" t="n">
-        <v>1.105533793569857</v>
+        <v>0.2163331530557144</v>
       </c>
       <c r="F47" t="n">
-        <v>2.402280663894762</v>
+        <v>1.645639056500281</v>
       </c>
       <c r="G47" t="n">
-        <v>-1.613691498261938</v>
+        <v>1.701427003293077</v>
       </c>
       <c r="H47" t="n">
-        <v>0.6402573813874657</v>
+        <v>8.299240210403269</v>
       </c>
       <c r="I47" t="n">
-        <v>52.3494035573238</v>
+        <v>51.7640141169116</v>
       </c>
       <c r="J47" t="n">
-        <v>21.29316607990519</v>
+        <v>11.22848488519097</v>
       </c>
       <c r="K47" t="n">
-        <v>0.5637879203323768</v>
+        <v>0.4883582615914524</v>
       </c>
       <c r="L47" t="n">
-        <v>9.994018438594653</v>
+        <v>462.2647392166729</v>
       </c>
       <c r="M47" t="n">
-        <v>9.948721105623312</v>
+        <v>456.3128458033316</v>
       </c>
       <c r="N47" t="n">
-        <v>9.382881526154984</v>
+        <v>441.4133927049047</v>
       </c>
       <c r="O47" t="n">
-        <v>0.0004422470774380835</v>
+        <v>-0.1415570983329268</v>
       </c>
       <c r="P47" t="n">
-        <v>66.28414822031093</v>
+        <v>47.14285714285714</v>
       </c>
       <c r="Q47" t="n">
-        <v>-33.71585177968907</v>
+        <v>-52.85714285714285</v>
       </c>
       <c r="R47" t="n">
-        <v>11.95326061216765</v>
+        <v>1.262493424513223</v>
       </c>
       <c r="S47" t="n">
-        <v>-1.372543061434861</v>
+        <v>1.813186813186807</v>
       </c>
       <c r="T47" t="inlineStr">
         <is>
           <t>Trend Bullish</t>
         </is>
       </c>
-      <c r="U47" t="inlineStr"/>
+      <c r="U47" t="inlineStr">
+        <is>
+          <t>Doji, Bullish Harami</t>
+        </is>
+      </c>
       <c r="V47" t="inlineStr">
         <is>
-          <t>Double Top, Inside Bar</t>
+          <t>Inside Bar</t>
         </is>
       </c>
       <c r="W47" t="n">
-        <v>62.8</v>
+        <v>62.7</v>
       </c>
       <c r="X47" t="n">
-        <v>68.90000000000001</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="Y47" t="inlineStr">
         <is>
@@ -4752,94 +4752,86 @@
       </c>
       <c r="Z47" t="inlineStr">
         <is>
-          <t>EMA e SMA allineate al rialzo — struttura bullish solida; trend in sviluppo (ADX 21); pattern: Double Top; in zona Fib Fib 23.6 — livello strutturale</t>
+          <t>EMA allineate al rialzo (EMA20&gt;EMA50&gt;EMA200); mercato laterale — ATR basso (ADX 11); doji — indecisione del mercato; in zona Fib Fib 23.6 — livello strutturale; favorito dal quadrante macro (Surriscaldamento)</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>CORN</t>
+          <t>REY</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Corn</t>
+          <t>Reply</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Commodities</t>
+          <t>Azioni IT</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>463.25</v>
+        <v>105.1999969482422</v>
       </c>
       <c r="E48" t="n">
-        <v>0.2163331530557144</v>
+        <v>0.2859822859862193</v>
       </c>
       <c r="F48" t="n">
-        <v>1.645639056500281</v>
+        <v>6.316321569235805</v>
       </c>
       <c r="G48" t="n">
-        <v>1.701427003293077</v>
+        <v>14.47224722691438</v>
       </c>
       <c r="H48" t="n">
-        <v>8.299240210403269</v>
+        <v>18.73589024831612</v>
       </c>
       <c r="I48" t="n">
-        <v>51.7640141169116</v>
+        <v>69.55211064436919</v>
       </c>
       <c r="J48" t="n">
-        <v>11.22848488519097</v>
+        <v>32.07940746259378</v>
       </c>
       <c r="K48" t="n">
-        <v>0.4883582615914524</v>
+        <v>0.909898994734777</v>
       </c>
       <c r="L48" t="n">
-        <v>462.2647392166729</v>
+        <v>98.19438952999867</v>
       </c>
       <c r="M48" t="n">
-        <v>456.3128458033316</v>
+        <v>94.79156085791348</v>
       </c>
       <c r="N48" t="n">
-        <v>441.4133927049047</v>
+        <v>107.1947574065142</v>
       </c>
       <c r="O48" t="n">
-        <v>-0.1415570983329268</v>
+        <v>0.7070076473361731</v>
       </c>
       <c r="P48" t="n">
-        <v>47.14285714285714</v>
+        <v>95.49836372824642</v>
       </c>
       <c r="Q48" t="n">
-        <v>-52.85714285714285</v>
+        <v>-4.501636271753583</v>
       </c>
       <c r="R48" t="n">
-        <v>1.262493424513223</v>
+        <v>96.61357603196706</v>
       </c>
       <c r="S48" t="n">
-        <v>1.813186813186807</v>
+        <v>14.72191979201454</v>
       </c>
       <c r="T48" t="inlineStr">
         <is>
-          <t>Trend Bullish</t>
-        </is>
-      </c>
-      <c r="U48" t="inlineStr">
-        <is>
-          <t>Doji, Bullish Harami</t>
-        </is>
-      </c>
-      <c r="V48" t="inlineStr">
-        <is>
-          <t>Inside Bar</t>
-        </is>
-      </c>
+          <t>Range</t>
+        </is>
+      </c>
+      <c r="U48" t="inlineStr"/>
+      <c r="V48" t="inlineStr"/>
       <c r="W48" t="n">
-        <v>62.7</v>
+        <v>62.5</v>
       </c>
       <c r="X48" t="n">
-        <v>79.09999999999999</v>
+        <v>65.2</v>
       </c>
       <c r="Y48" t="inlineStr">
         <is>
@@ -4848,86 +4840,94 @@
       </c>
       <c r="Z48" t="inlineStr">
         <is>
-          <t>EMA allineate al rialzo (EMA20&gt;EMA50&gt;EMA200); mercato laterale — ATR basso (ADX 11); doji — indecisione del mercato; in zona Fib Fib 23.6 — livello strutturale; favorito dal quadrante macro (Surriscaldamento)</t>
+          <t>trend molto direzionale (ADX 32); RSI in forza (70) — momentum positivo; vicino alla resistenza dei 20g (105.90); in zona Fib Fib 23.6 — livello strutturale</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>REY</t>
+          <t>XLY</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Reply</t>
+          <t>Consumer Discr.</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Azioni IT</t>
+          <t>Settoriali</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>105.1999969482422</v>
+        <v>119.1800003051758</v>
       </c>
       <c r="E49" t="n">
-        <v>0.2859822859862193</v>
+        <v>0.4043836303912363</v>
       </c>
       <c r="F49" t="n">
-        <v>6.316321569235805</v>
+        <v>2.274093841619185</v>
       </c>
       <c r="G49" t="n">
-        <v>14.47224722691438</v>
+        <v>1.223035899042912</v>
       </c>
       <c r="H49" t="n">
-        <v>18.73589024831612</v>
+        <v>2.090116914558826</v>
       </c>
       <c r="I49" t="n">
-        <v>69.55211064436919</v>
+        <v>56.85244701294989</v>
       </c>
       <c r="J49" t="n">
-        <v>32.07940746259378</v>
+        <v>11.16115529921645</v>
       </c>
       <c r="K49" t="n">
-        <v>0.909898994734777</v>
+        <v>0.6940333808920923</v>
       </c>
       <c r="L49" t="n">
-        <v>98.19438952999867</v>
+        <v>117.7311802929923</v>
       </c>
       <c r="M49" t="n">
-        <v>94.79156085791348</v>
+        <v>116.6755825004548</v>
       </c>
       <c r="N49" t="n">
-        <v>107.1947574065142</v>
+        <v>115.3126143279716</v>
       </c>
       <c r="O49" t="n">
-        <v>0.7070076473361731</v>
+        <v>-0.2132384445311677</v>
       </c>
       <c r="P49" t="n">
-        <v>95.49836372824642</v>
+        <v>71.86151713751295</v>
       </c>
       <c r="Q49" t="n">
-        <v>-4.501636271753583</v>
+        <v>-28.13848286248705</v>
       </c>
       <c r="R49" t="n">
-        <v>96.61357603196706</v>
+        <v>47.6573141326727</v>
       </c>
       <c r="S49" t="n">
-        <v>14.72191979201454</v>
+        <v>0.412838363544088</v>
       </c>
       <c r="T49" t="inlineStr">
         <is>
-          <t>Range</t>
-        </is>
-      </c>
-      <c r="U49" t="inlineStr"/>
-      <c r="V49" t="inlineStr"/>
+          <t>Trend Bullish</t>
+        </is>
+      </c>
+      <c r="U49" t="inlineStr">
+        <is>
+          <t>Doji</t>
+        </is>
+      </c>
+      <c r="V49" t="inlineStr">
+        <is>
+          <t>Double Top</t>
+        </is>
+      </c>
       <c r="W49" t="n">
-        <v>62.5</v>
+        <v>62.1</v>
       </c>
       <c r="X49" t="n">
-        <v>65.2</v>
+        <v>73.90000000000001</v>
       </c>
       <c r="Y49" t="inlineStr">
         <is>
@@ -4936,73 +4936,73 @@
       </c>
       <c r="Z49" t="inlineStr">
         <is>
-          <t>trend molto direzionale (ADX 32); RSI in forza (70) — momentum positivo; vicino alla resistenza dei 20g (105.90); in zona Fib Fib 23.6 — livello strutturale</t>
+          <t>EMA allineate al rialzo (EMA20&gt;EMA50&gt;EMA200); mercato laterale — ATR basso (ADX 11); pattern: Double Top; doji — indecisione del mercato; in zona Fib Fib 23.6 — livello strutturale</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>XLY</t>
+          <t>GBPUSD</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Consumer Discr.</t>
+          <t>GBP/USD</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Settoriali</t>
+          <t>FX/Macro</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>119.1800003051758</v>
+        <v>1.350566625595093</v>
       </c>
       <c r="E50" t="n">
-        <v>0.4043836303912363</v>
+        <v>0.5442825746864388</v>
       </c>
       <c r="F50" t="n">
-        <v>2.274093841619185</v>
+        <v>1.481578553007701</v>
       </c>
       <c r="G50" t="n">
-        <v>1.223035899042912</v>
+        <v>0.291729618032055</v>
       </c>
       <c r="H50" t="n">
-        <v>2.090116914558826</v>
+        <v>-0.3862553924523615</v>
       </c>
       <c r="I50" t="n">
-        <v>56.85244701294989</v>
+        <v>52.26164993432197</v>
       </c>
       <c r="J50" t="n">
-        <v>11.16115529921645</v>
+        <v>17.3531454319541</v>
       </c>
       <c r="K50" t="n">
-        <v>0.6940333808920923</v>
+        <v>0.4951059598080276</v>
       </c>
       <c r="L50" t="n">
-        <v>117.7311802929923</v>
+        <v>1.347599342109362</v>
       </c>
       <c r="M50" t="n">
-        <v>116.6755825004548</v>
+        <v>1.346645173739949</v>
       </c>
       <c r="N50" t="n">
-        <v>115.3126143279716</v>
+        <v>1.339994244885078</v>
       </c>
       <c r="O50" t="n">
-        <v>-0.2132384445311677</v>
+        <v>-0.001202100638672023</v>
       </c>
       <c r="P50" t="n">
-        <v>71.86151713751295</v>
+        <v>57.8579213248247</v>
       </c>
       <c r="Q50" t="n">
-        <v>-28.13848286248705</v>
+        <v>-42.14207867517531</v>
       </c>
       <c r="R50" t="n">
-        <v>47.6573141326727</v>
+        <v>-21.22557768927481</v>
       </c>
       <c r="S50" t="n">
-        <v>0.412838363544088</v>
+        <v>-0.0698226824929038</v>
       </c>
       <c r="T50" t="inlineStr">
         <is>
@@ -5011,19 +5011,19 @@
       </c>
       <c r="U50" t="inlineStr">
         <is>
-          <t>Doji</t>
+          <t>Morning Star</t>
         </is>
       </c>
       <c r="V50" t="inlineStr">
         <is>
-          <t>Double Top</t>
+          <t>Double Top, Double Bottom, Bear Flag / Consolidation, Volatility Squeeze</t>
         </is>
       </c>
       <c r="W50" t="n">
-        <v>62.1</v>
+        <v>61.6</v>
       </c>
       <c r="X50" t="n">
-        <v>73.90000000000001</v>
+        <v>64.5</v>
       </c>
       <c r="Y50" t="inlineStr">
         <is>
@@ -5032,7 +5032,7 @@
       </c>
       <c r="Z50" t="inlineStr">
         <is>
-          <t>EMA allineate al rialzo (EMA20&gt;EMA50&gt;EMA200); mercato laterale — ATR basso (ADX 11); pattern: Double Top; doji — indecisione del mercato; in zona Fib Fib 23.6 — livello strutturale</t>
+          <t>EMA allineate al rialzo (EMA20&gt;EMA50&gt;EMA200); pattern: Double Bottom; morning star — inversione rialzista a 3 candele; vicino alla resistenza dei 20g (1.3658); in zona Fib Fib 50.0 — livello strutturale</t>
         </is>
       </c>
     </row>
@@ -7815,52 +7815,52 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>1.164686679840088</v>
+        <v>1.164279937744141</v>
       </c>
       <c r="E81" t="n">
-        <v>0.221284690365553</v>
+        <v>0.1862845344445807</v>
       </c>
       <c r="F81" t="n">
-        <v>0.2795276051215323</v>
+        <v>0.2445071090991124</v>
       </c>
       <c r="G81" t="n">
-        <v>-0.3167893886727002</v>
+        <v>-0.3516016336451933</v>
       </c>
       <c r="H81" t="n">
-        <v>-1.424417718885496</v>
+        <v>-1.458843148179279</v>
       </c>
       <c r="I81" t="n">
-        <v>45.97636157265175</v>
+        <v>45.47396795439307</v>
       </c>
       <c r="J81" t="n">
         <v>19.3248038386208</v>
       </c>
       <c r="K81" t="n">
-        <v>0.2706413241467881</v>
+        <v>0.253203559866135</v>
       </c>
       <c r="L81" t="n">
-        <v>1.167658239412543</v>
+        <v>1.167619502070071</v>
       </c>
       <c r="M81" t="n">
-        <v>1.168134211724731</v>
+        <v>1.168118261054302</v>
       </c>
       <c r="N81" t="n">
-        <v>1.161599668433297</v>
+        <v>1.161595621248262</v>
       </c>
       <c r="O81" t="n">
-        <v>-0.001326394412732029</v>
+        <v>-0.001352351743071416</v>
       </c>
       <c r="P81" t="n">
-        <v>31.72148789077786</v>
+        <v>29.86705943736684</v>
       </c>
       <c r="Q81" t="n">
-        <v>-68.27851210922213</v>
+        <v>-70.13294056263315</v>
       </c>
       <c r="R81" t="n">
-        <v>-86.51548647974066</v>
+        <v>-88.5001014380455</v>
       </c>
       <c r="S81" t="n">
-        <v>-0.5089672885590257</v>
+        <v>-0.5437124194800469</v>
       </c>
       <c r="T81" t="inlineStr">
         <is>
@@ -8575,52 +8575,52 @@
         </is>
       </c>
       <c r="D89" t="n">
-        <v>77280.0390625</v>
+        <v>77285.0234375</v>
       </c>
       <c r="E89" t="n">
-        <v>0.3882952639364445</v>
+        <v>0.3947700653894159</v>
       </c>
       <c r="F89" t="n">
-        <v>-0.2294597005727428</v>
+        <v>-0.2230247428160248</v>
       </c>
       <c r="G89" t="n">
-        <v>-3.191699879388987</v>
+        <v>-3.185455978935936</v>
       </c>
       <c r="H89" t="n">
-        <v>9.589315029459522</v>
+        <v>9.59638327436112</v>
       </c>
       <c r="I89" t="n">
-        <v>48.13401400670391</v>
+        <v>48.15496005944417</v>
       </c>
       <c r="J89" t="n">
         <v>33.22754798923612</v>
       </c>
       <c r="K89" t="n">
-        <v>0.3056469469887519</v>
+        <v>0.3062188210197999</v>
       </c>
       <c r="L89" t="n">
-        <v>77818.98841951831</v>
+        <v>77819.46312189927</v>
       </c>
       <c r="M89" t="n">
-        <v>76758.54317835714</v>
+        <v>76758.73864404341</v>
       </c>
       <c r="N89" t="n">
-        <v>81480.77293940274</v>
+        <v>81480.82253517388</v>
       </c>
       <c r="O89" t="n">
-        <v>-431.8786144465865</v>
+        <v>-431.5605232784949</v>
       </c>
       <c r="P89" t="n">
-        <v>39.02607920830003</v>
+        <v>39.09038769550838</v>
       </c>
       <c r="Q89" t="n">
-        <v>-60.97392079169997</v>
+        <v>-60.90961230449162</v>
       </c>
       <c r="R89" t="n">
-        <v>-49.03983820589977</v>
+        <v>-48.99259730479742</v>
       </c>
       <c r="S89" t="n">
-        <v>-4.506546839104619</v>
+        <v>-4.500387743090006</v>
       </c>
       <c r="T89" t="inlineStr">
         <is>
@@ -9511,52 +9511,52 @@
         </is>
       </c>
       <c r="D99" t="n">
-        <v>9.522000312805176</v>
+        <v>9.510000228881836</v>
       </c>
       <c r="E99" t="n">
-        <v>0.9863231834294384</v>
+        <v>0.8590553496234499</v>
       </c>
       <c r="F99" t="n">
-        <v>-1.038533610087977</v>
+        <v>-1.16324962172879</v>
       </c>
       <c r="G99" t="n">
-        <v>1.804546880625435</v>
+        <v>1.676247881863357</v>
       </c>
       <c r="H99" t="n">
-        <v>2.979211579252872</v>
+        <v>2.849432211397929</v>
       </c>
       <c r="I99" t="n">
-        <v>46.96294386571149</v>
+        <v>46.71233904314905</v>
       </c>
       <c r="J99" t="n">
         <v>33.95525235157974</v>
       </c>
       <c r="K99" t="n">
-        <v>0.2626297268640682</v>
+        <v>0.2562582788649342</v>
       </c>
       <c r="L99" t="n">
-        <v>9.684625529443531</v>
+        <v>9.683482664307975</v>
       </c>
       <c r="M99" t="n">
-        <v>9.576462542802576</v>
+        <v>9.575991951276171</v>
       </c>
       <c r="N99" t="n">
-        <v>11.23381568018078</v>
+        <v>11.23369627636065</v>
       </c>
       <c r="O99" t="n">
-        <v>-0.08543877241022103</v>
+        <v>-0.08620458973182538</v>
       </c>
       <c r="P99" t="n">
-        <v>25.09668574659035</v>
+        <v>24.38532965868136</v>
       </c>
       <c r="Q99" t="n">
-        <v>-74.90331425340965</v>
+        <v>-75.61467034131863</v>
       </c>
       <c r="R99" t="n">
-        <v>-54.38307640790317</v>
+        <v>-54.84115439304429</v>
       </c>
       <c r="S99" t="n">
-        <v>-2.498344544016473</v>
+        <v>-2.621220831529603</v>
       </c>
       <c r="T99" t="inlineStr">
         <is>
@@ -9573,7 +9573,7 @@
         <v>42.7</v>
       </c>
       <c r="X99" t="n">
-        <v>65.5</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="Y99" t="inlineStr">
         <is>
@@ -9773,83 +9773,87 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>IG</t>
+          <t>DOT</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Investment Grade Corp ETF</t>
+          <t>Polkadot</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Bond</t>
+          <t>Crypto</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>108.370002746582</v>
+        <v>1.274999976158142</v>
       </c>
       <c r="E102" t="n">
-        <v>0.1848983831213014</v>
+        <v>2.439258229041319</v>
       </c>
       <c r="F102" t="n">
-        <v>0.4728371345674942</v>
+        <v>2.210711378848695</v>
       </c>
       <c r="G102" t="n">
-        <v>-1.050030982225358</v>
+        <v>3.815947498544747</v>
       </c>
       <c r="H102" t="n">
-        <v>-2.963823020727863</v>
+        <v>-8.952116473461336</v>
       </c>
       <c r="I102" t="n">
-        <v>47.21595294956771</v>
+        <v>49.33693405077627</v>
       </c>
       <c r="J102" t="n">
-        <v>43.30556513127745</v>
+        <v>30.82866162063231</v>
       </c>
       <c r="K102" t="n">
-        <v>0.429645604460562</v>
+        <v>0.3646429768895229</v>
       </c>
       <c r="L102" t="n">
-        <v>108.4786422370491</v>
+        <v>1.278174685256816</v>
       </c>
       <c r="M102" t="n">
-        <v>109.0014902217753</v>
+        <v>1.297624518634279</v>
       </c>
       <c r="N102" t="n">
-        <v>109.7084384992036</v>
+        <v>1.824826219117784</v>
       </c>
       <c r="O102" t="n">
-        <v>-0.03662095116250719</v>
+        <v>-0.004172028199852181</v>
       </c>
       <c r="P102" t="n">
-        <v>58.53670639535785</v>
+        <v>30.78156134683335</v>
       </c>
       <c r="Q102" t="n">
-        <v>-41.46329360464215</v>
+        <v>-69.21843865316664</v>
       </c>
       <c r="R102" t="n">
-        <v>-20.25480368336319</v>
+        <v>-41.024776187779</v>
       </c>
       <c r="S102" t="n">
-        <v>-1.122258891116212</v>
+        <v>-0.3369012908570279</v>
       </c>
       <c r="T102" t="inlineStr">
         <is>
           <t>Trend Bearish</t>
         </is>
       </c>
-      <c r="U102" t="inlineStr"/>
+      <c r="U102" t="inlineStr">
+        <is>
+          <t>Piercing Pattern</t>
+        </is>
+      </c>
       <c r="V102" t="inlineStr">
         <is>
-          <t>Double Top, Double Bottom, Volatility Squeeze</t>
+          <t>Double Bottom, Inside Bar</t>
         </is>
       </c>
       <c r="W102" t="n">
-        <v>34.6</v>
+        <v>35.5</v>
       </c>
       <c r="X102" t="n">
-        <v>72.09999999999999</v>
+        <v>72.7</v>
       </c>
       <c r="Y102" t="inlineStr">
         <is>
@@ -9858,19 +9862,19 @@
       </c>
       <c r="Z102" t="inlineStr">
         <is>
-          <t>EMA e SMA allineate al ribasso — struttura bearish solida; trend molto direzionale (ADX 43); pattern: Double Bottom; sul supporto dei 20g (106.93); vicino alla resistenza dei 20g (109.59); in zona Fib Fib 78.6 — livello strutturale; penalizzato dal quadrante macro (Surriscaldamento)</t>
+          <t>EMA allineate al ribasso (EMA20&lt;EMA50&lt;EMA200); trend molto direzionale (ADX 31); pattern: Double Bottom; segnale candlestick: Piercing Pattern; in zona Fib Fib 78.6 — livello strutturale</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>US10Y</t>
+          <t>IG</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>US Treasury 7-10Y ETF</t>
+          <t>Investment Grade Corp ETF</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -9879,73 +9883,69 @@
         </is>
       </c>
       <c r="D103" t="n">
-        <v>93.87999725341797</v>
+        <v>108.370002746582</v>
       </c>
       <c r="E103" t="n">
-        <v>0.08528166210828303</v>
+        <v>0.1848983831213014</v>
       </c>
       <c r="F103" t="n">
-        <v>0.3956743757191461</v>
+        <v>0.4728371345674942</v>
       </c>
       <c r="G103" t="n">
-        <v>-1.56234187926293</v>
+        <v>-1.050030982225358</v>
       </c>
       <c r="H103" t="n">
-        <v>-3.633751777934024</v>
+        <v>-2.963823020727863</v>
       </c>
       <c r="I103" t="n">
-        <v>41.03512958474433</v>
+        <v>47.21595294956771</v>
       </c>
       <c r="J103" t="n">
-        <v>54.92695620059033</v>
+        <v>43.30556513127745</v>
       </c>
       <c r="K103" t="n">
-        <v>0.2977724724528542</v>
+        <v>0.429645604460562</v>
       </c>
       <c r="L103" t="n">
-        <v>94.29429839161831</v>
+        <v>108.4786422370491</v>
       </c>
       <c r="M103" t="n">
-        <v>94.94138304997593</v>
+        <v>109.0014902217753</v>
       </c>
       <c r="N103" t="n">
-        <v>95.62757604437337</v>
+        <v>109.7084384992036</v>
       </c>
       <c r="O103" t="n">
-        <v>-0.04903808341769722</v>
+        <v>-0.03662095116250719</v>
       </c>
       <c r="P103" t="n">
-        <v>41.70398678029772</v>
+        <v>58.53670639535785</v>
       </c>
       <c r="Q103" t="n">
-        <v>-58.29601321970228</v>
+        <v>-41.46329360464215</v>
       </c>
       <c r="R103" t="n">
-        <v>-54.48834508917206</v>
+        <v>-20.25480368336319</v>
       </c>
       <c r="S103" t="n">
-        <v>-1.758058129025875</v>
+        <v>-1.122258891116212</v>
       </c>
       <c r="T103" t="inlineStr">
         <is>
           <t>Trend Bearish</t>
         </is>
       </c>
-      <c r="U103" t="inlineStr">
-        <is>
-          <t>Hammer</t>
-        </is>
-      </c>
+      <c r="U103" t="inlineStr"/>
       <c r="V103" t="inlineStr">
         <is>
-          <t>Double Top, Double Bottom</t>
+          <t>Double Top, Double Bottom, Volatility Squeeze</t>
         </is>
       </c>
       <c r="W103" t="n">
-        <v>34.4</v>
+        <v>34.6</v>
       </c>
       <c r="X103" t="n">
-        <v>78.3</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="Y103" t="inlineStr">
         <is>
@@ -9954,19 +9954,19 @@
       </c>
       <c r="Z103" t="inlineStr">
         <is>
-          <t>EMA e SMA allineate al ribasso — struttura bearish solida; trend molto direzionale (ADX 55); pattern: Double Bottom; hammer — segnale di rimbalzo da supporto; sul supporto dei 20g (92.95); in zona Fib Fib 78.6 — livello strutturale; penalizzato dal quadrante macro (Surriscaldamento)</t>
+          <t>EMA e SMA allineate al ribasso — struttura bearish solida; trend molto direzionale (ADX 43); pattern: Double Bottom; sul supporto dei 20g (106.93); vicino alla resistenza dei 20g (109.59); in zona Fib Fib 78.6 — livello strutturale; penalizzato dal quadrante macro (Surriscaldamento)</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>US2Y</t>
+          <t>US10Y</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>US Treasury 1-3Y ETF</t>
+          <t>US Treasury 7-10Y ETF</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -9975,59 +9975,63 @@
         </is>
       </c>
       <c r="D104" t="n">
-        <v>82.12000274658203</v>
+        <v>93.87999725341797</v>
       </c>
       <c r="E104" t="n">
-        <v>-0.0243445863343017</v>
+        <v>0.08528166210828303</v>
       </c>
       <c r="F104" t="n">
-        <v>0.07312355565869399</v>
+        <v>0.3956743757191461</v>
       </c>
       <c r="G104" t="n">
-        <v>-0.4364701693738482</v>
+        <v>-1.56234187926293</v>
       </c>
       <c r="H104" t="n">
-        <v>-1.131705802602045</v>
+        <v>-3.633751777934024</v>
       </c>
       <c r="I104" t="n">
-        <v>41.74395104577886</v>
+        <v>41.03512958474433</v>
       </c>
       <c r="J104" t="n">
-        <v>41.39994093847094</v>
+        <v>54.92695620059033</v>
       </c>
       <c r="K104" t="n">
-        <v>0.3038935138985066</v>
+        <v>0.2977724724528542</v>
       </c>
       <c r="L104" t="n">
-        <v>82.22047382019801</v>
+        <v>94.29429839161831</v>
       </c>
       <c r="M104" t="n">
-        <v>82.37757725562591</v>
+        <v>94.94138304997593</v>
       </c>
       <c r="N104" t="n">
-        <v>82.60192690722243</v>
+        <v>95.62757604437337</v>
       </c>
       <c r="O104" t="n">
-        <v>-0.002411052595110319</v>
+        <v>-0.04903808341769722</v>
       </c>
       <c r="P104" t="n">
-        <v>33.3340397575552</v>
+        <v>41.70398678029772</v>
       </c>
       <c r="Q104" t="n">
-        <v>-66.6659602424448</v>
+        <v>-58.29601321970228</v>
       </c>
       <c r="R104" t="n">
-        <v>-46.24522131188951</v>
+        <v>-54.48834508917206</v>
       </c>
       <c r="S104" t="n">
-        <v>-0.5449884339413402</v>
+        <v>-1.758058129025875</v>
       </c>
       <c r="T104" t="inlineStr">
         <is>
           <t>Trend Bearish</t>
         </is>
       </c>
-      <c r="U104" t="inlineStr"/>
+      <c r="U104" t="inlineStr">
+        <is>
+          <t>Hammer</t>
+        </is>
+      </c>
       <c r="V104" t="inlineStr">
         <is>
           <t>Double Top, Double Bottom</t>
@@ -10037,7 +10041,7 @@
         <v>34.4</v>
       </c>
       <c r="X104" t="n">
-        <v>65.40000000000001</v>
+        <v>78.3</v>
       </c>
       <c r="Y104" t="inlineStr">
         <is>
@@ -10046,94 +10050,90 @@
       </c>
       <c r="Z104" t="inlineStr">
         <is>
-          <t>EMA e SMA allineate al ribasso — struttura bearish solida; trend molto direzionale (ADX 41); pattern: Double Bottom; sul supporto dei 20g (82.00); vicino alla resistenza dei 20g (82.58); in zona Fib Fib 78.6 — livello strutturale</t>
+          <t>EMA e SMA allineate al ribasso — struttura bearish solida; trend molto direzionale (ADX 55); pattern: Double Bottom; hammer — segnale di rimbalzo da supporto; sul supporto dei 20g (92.95); in zona Fib Fib 78.6 — livello strutturale; penalizzato dal quadrante macro (Surriscaldamento)</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>DOT</t>
+          <t>US2Y</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Polkadot</t>
+          <t>US Treasury 1-3Y ETF</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Crypto</t>
+          <t>Bond</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>1.269999980926514</v>
+        <v>82.12000274658203</v>
       </c>
       <c r="E105" t="n">
-        <v>2.037536023351483</v>
+        <v>-0.0243445863343017</v>
       </c>
       <c r="F105" t="n">
-        <v>1.809885434478486</v>
+        <v>0.07312355565869399</v>
       </c>
       <c r="G105" t="n">
-        <v>3.408826516453578</v>
+        <v>-0.4364701693738482</v>
       </c>
       <c r="H105" t="n">
-        <v>-9.309166663261569</v>
+        <v>-1.131705802602045</v>
       </c>
       <c r="I105" t="n">
-        <v>48.71655226240159</v>
+        <v>41.74395104577886</v>
       </c>
       <c r="J105" t="n">
-        <v>30.82866162063231</v>
+        <v>41.39994093847094</v>
       </c>
       <c r="K105" t="n">
-        <v>0.3407497842262626</v>
+        <v>0.3038935138985066</v>
       </c>
       <c r="L105" t="n">
-        <v>1.277698495234756</v>
+        <v>82.22047382019801</v>
       </c>
       <c r="M105" t="n">
-        <v>1.297428440389901</v>
+        <v>82.37757725562591</v>
       </c>
       <c r="N105" t="n">
-        <v>1.82477646792145</v>
+        <v>82.60192690722243</v>
       </c>
       <c r="O105" t="n">
-        <v>-0.004491116214634135</v>
+        <v>-0.002411052595110319</v>
       </c>
       <c r="P105" t="n">
-        <v>28.5908287261075</v>
+        <v>33.3340397575552</v>
       </c>
       <c r="Q105" t="n">
-        <v>-71.4091712738925</v>
+        <v>-66.6659602424448</v>
       </c>
       <c r="R105" t="n">
-        <v>-42.85262776591595</v>
+        <v>-46.24522131188951</v>
       </c>
       <c r="S105" t="n">
-        <v>-0.7277366066478219</v>
+        <v>-0.5449884339413402</v>
       </c>
       <c r="T105" t="inlineStr">
         <is>
           <t>Trend Bearish</t>
         </is>
       </c>
-      <c r="U105" t="inlineStr">
-        <is>
-          <t>Piercing Pattern</t>
-        </is>
-      </c>
+      <c r="U105" t="inlineStr"/>
       <c r="V105" t="inlineStr">
         <is>
-          <t>Double Bottom, Inside Bar</t>
+          <t>Double Top, Double Bottom</t>
         </is>
       </c>
       <c r="W105" t="n">
-        <v>33.9</v>
+        <v>34.4</v>
       </c>
       <c r="X105" t="n">
-        <v>72.90000000000001</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="Y105" t="inlineStr">
         <is>
@@ -10142,7 +10142,7 @@
       </c>
       <c r="Z105" t="inlineStr">
         <is>
-          <t>EMA allineate al ribasso (EMA20&lt;EMA50&lt;EMA200); trend molto direzionale (ADX 31); pattern: Double Bottom; segnale candlestick: Piercing Pattern; in zona Fib Fib 78.6 — livello strutturale</t>
+          <t>EMA e SMA allineate al ribasso — struttura bearish solida; trend molto direzionale (ADX 41); pattern: Double Bottom; sul supporto dei 20g (82.00); vicino alla resistenza dei 20g (82.58); in zona Fib Fib 78.6 — livello strutturale</t>
         </is>
       </c>
     </row>
@@ -10163,52 +10163,52 @@
         </is>
       </c>
       <c r="D106" t="n">
-        <v>85.47000122070312</v>
+        <v>85.45999908447266</v>
       </c>
       <c r="E106" t="n">
-        <v>0.2584248505975717</v>
+        <v>0.2466920974761866</v>
       </c>
       <c r="F106" t="n">
-        <v>-0.6647195183339449</v>
+        <v>-0.6763442403847075</v>
       </c>
       <c r="G106" t="n">
-        <v>1.641270693258989</v>
+        <v>1.629376112451775</v>
       </c>
       <c r="H106" t="n">
-        <v>-5.89328524529461</v>
+        <v>-5.904298093869964</v>
       </c>
       <c r="I106" t="n">
-        <v>45.89684092880506</v>
+        <v>45.87111063962005</v>
       </c>
       <c r="J106" t="n">
         <v>33.81356000471499</v>
       </c>
       <c r="K106" t="n">
-        <v>0.2911283122018055</v>
+        <v>0.2905740818640971</v>
       </c>
       <c r="L106" t="n">
-        <v>86.99136726910295</v>
+        <v>86.99041468470006</v>
       </c>
       <c r="M106" t="n">
-        <v>87.31123429969377</v>
+        <v>87.31084205905728</v>
       </c>
       <c r="N106" t="n">
-        <v>108.4240793334279</v>
+        <v>108.4239798096843</v>
       </c>
       <c r="O106" t="n">
-        <v>-0.5802308630423202</v>
+        <v>-0.5808691760097393</v>
       </c>
       <c r="P106" t="n">
-        <v>23.7235036286556</v>
+        <v>23.66070273765898</v>
       </c>
       <c r="Q106" t="n">
-        <v>-76.27649637134439</v>
+        <v>-76.33929726234102</v>
       </c>
       <c r="R106" t="n">
-        <v>-52.91165458240093</v>
+        <v>-52.95918126491046</v>
       </c>
       <c r="S106" t="n">
-        <v>-0.9837786344722987</v>
+        <v>-0.9953660185951452</v>
       </c>
       <c r="T106" t="inlineStr">
         <is>
@@ -10625,12 +10625,12 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>ADA</t>
+          <t>XRP</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Cardano</t>
+          <t>XRP</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -10639,52 +10639,52 @@
         </is>
       </c>
       <c r="D111" t="n">
-        <v>0.2449000030755997</v>
+        <v>1.354699969291687</v>
       </c>
       <c r="E111" t="n">
-        <v>1.144433362738217</v>
+        <v>0.3456896477125104</v>
       </c>
       <c r="F111" t="n">
-        <v>-1.646978661024112</v>
+        <v>-0.7813306928680652</v>
       </c>
       <c r="G111" t="n">
-        <v>-1.998443420320284</v>
+        <v>-2.676729985908566</v>
       </c>
       <c r="H111" t="n">
-        <v>-7.997702820063235</v>
+        <v>-4.290164675990615</v>
       </c>
       <c r="I111" t="n">
-        <v>42.12299840716615</v>
+        <v>42.84330468884762</v>
       </c>
       <c r="J111" t="n">
-        <v>39.60642768256695</v>
+        <v>29.15747068783356</v>
       </c>
       <c r="K111" t="n">
-        <v>0.2186157589000814</v>
+        <v>0.222002380719466</v>
       </c>
       <c r="L111" t="n">
-        <v>0.252881542207471</v>
+        <v>1.386957893098051</v>
       </c>
       <c r="M111" t="n">
-        <v>0.2563511815175361</v>
+        <v>1.401426176742333</v>
       </c>
       <c r="N111" t="n">
-        <v>0.34970750158664</v>
+        <v>1.675479009360618</v>
       </c>
       <c r="O111" t="n">
-        <v>-0.002375827773522811</v>
+        <v>-0.008537763384974322</v>
       </c>
       <c r="P111" t="n">
-        <v>17.9614334974369</v>
+        <v>19.69306552877554</v>
       </c>
       <c r="Q111" t="n">
-        <v>-82.0385665025631</v>
+        <v>-80.30693447122445</v>
       </c>
       <c r="R111" t="n">
-        <v>-74.36623753576522</v>
+        <v>-93.85040447631768</v>
       </c>
       <c r="S111" t="n">
-        <v>-6.575927717166152</v>
+        <v>-4.136084019094088</v>
       </c>
       <c r="T111" t="inlineStr">
         <is>
@@ -10693,19 +10693,19 @@
       </c>
       <c r="U111" t="inlineStr">
         <is>
-          <t>Bullish Harami</t>
+          <t>Piercing Pattern</t>
         </is>
       </c>
       <c r="V111" t="inlineStr">
         <is>
-          <t>Double Bottom</t>
+          <t>Double Top, Inside Bar</t>
         </is>
       </c>
       <c r="W111" t="n">
-        <v>32.1</v>
+        <v>32.8</v>
       </c>
       <c r="X111" t="n">
-        <v>77.3</v>
+        <v>67.3</v>
       </c>
       <c r="Y111" t="inlineStr">
         <is>
@@ -10714,19 +10714,19 @@
       </c>
       <c r="Z111" t="inlineStr">
         <is>
-          <t>EMA allineate al ribasso (EMA20&lt;EMA50&lt;EMA200); trend molto direzionale (ADX 40); pattern: Double Bottom; segnale candlestick: Bullish Harami</t>
+          <t>EMA allineate al ribasso (EMA20&lt;EMA50&lt;EMA200); trend in sviluppo (ADX 29); pattern: Double Top; segnale candlestick: Piercing Pattern; in zona Fib Fib 78.6 — livello strutturale</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>XRP</t>
+          <t>ADA</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>XRP</t>
+          <t>Cardano</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -10735,69 +10735,73 @@
         </is>
       </c>
       <c r="D112" t="n">
-        <v>1.353500008583069</v>
+        <v>0.2445999979972839</v>
       </c>
       <c r="E112" t="n">
-        <v>0.2568058449621269</v>
+        <v>1.020530368572792</v>
       </c>
       <c r="F112" t="n">
-        <v>-0.8692162080586985</v>
+        <v>-1.767462146115295</v>
       </c>
       <c r="G112" t="n">
-        <v>-2.762936601910937</v>
+        <v>-2.118496357386501</v>
       </c>
       <c r="H112" t="n">
-        <v>-4.374942150280492</v>
+        <v>-8.110406601296649</v>
       </c>
       <c r="I112" t="n">
-        <v>42.59431678630272</v>
+        <v>41.83634411301754</v>
       </c>
       <c r="J112" t="n">
-        <v>29.15747068783356</v>
+        <v>39.60642768256695</v>
       </c>
       <c r="K112" t="n">
-        <v>0.2160186219301444</v>
+        <v>0.2134253030126457</v>
       </c>
       <c r="L112" t="n">
-        <v>1.386843611125802</v>
+        <v>0.2528529702952504</v>
       </c>
       <c r="M112" t="n">
-        <v>1.401379119459643</v>
+        <v>0.2563394166125041</v>
       </c>
       <c r="N112" t="n">
-        <v>1.67546706945307</v>
+        <v>0.3497045164614827</v>
       </c>
       <c r="O112" t="n">
-        <v>-0.008614342074071284</v>
+        <v>-0.002394973396754409</v>
       </c>
       <c r="P112" t="n">
-        <v>19.19291944994862</v>
+        <v>17.29113584372839</v>
       </c>
       <c r="Q112" t="n">
-        <v>-80.80708055005138</v>
+        <v>-82.70886415627162</v>
       </c>
       <c r="R112" t="n">
-        <v>-94.48457017813621</v>
+        <v>-74.79669465470181</v>
       </c>
       <c r="S112" t="n">
-        <v>-4.22099797433061</v>
+        <v>-6.690373187847232</v>
       </c>
       <c r="T112" t="inlineStr">
         <is>
           <t>Trend Bearish</t>
         </is>
       </c>
-      <c r="U112" t="inlineStr"/>
+      <c r="U112" t="inlineStr">
+        <is>
+          <t>Bullish Harami</t>
+        </is>
+      </c>
       <c r="V112" t="inlineStr">
         <is>
-          <t>Double Top, Inside Bar</t>
+          <t>Double Bottom</t>
         </is>
       </c>
       <c r="W112" t="n">
-        <v>31.9</v>
+        <v>32</v>
       </c>
       <c r="X112" t="n">
-        <v>70.8</v>
+        <v>77.3</v>
       </c>
       <c r="Y112" t="inlineStr">
         <is>
@@ -10806,7 +10810,7 @@
       </c>
       <c r="Z112" t="inlineStr">
         <is>
-          <t>EMA allineate al ribasso (EMA20&lt;EMA50&lt;EMA200); trend in sviluppo (ADX 29); pattern: Double Top; in zona Fib Fib 78.6 — livello strutturale</t>
+          <t>EMA allineate al ribasso (EMA20&lt;EMA50&lt;EMA200); trend molto direzionale (ADX 40); pattern: Double Bottom; segnale candlestick: Bullish Harami</t>
         </is>
       </c>
     </row>
@@ -11103,52 +11107,52 @@
         </is>
       </c>
       <c r="D116" t="n">
-        <v>2114.89990234375</v>
+        <v>2110.68994140625</v>
       </c>
       <c r="E116" t="n">
-        <v>0.8058176855378241</v>
+        <v>0.6051516614585806</v>
       </c>
       <c r="F116" t="n">
-        <v>-0.568104861684704</v>
+        <v>-0.7660359287815499</v>
       </c>
       <c r="G116" t="n">
-        <v>-9.866065845219385</v>
+        <v>-10.04548821008606</v>
       </c>
       <c r="H116" t="n">
-        <v>-1.892858983223222</v>
+        <v>-2.088152968963497</v>
       </c>
       <c r="I116" t="n">
-        <v>39.6988657298682</v>
+        <v>39.1242087568104</v>
       </c>
       <c r="J116" t="n">
         <v>47.20569154547086</v>
       </c>
       <c r="K116" t="n">
-        <v>0.2612677387593735</v>
+        <v>0.2518557187328582</v>
       </c>
       <c r="L116" t="n">
-        <v>2182.200074694491</v>
+        <v>2181.799126033777</v>
       </c>
       <c r="M116" t="n">
-        <v>2221.417480681568</v>
+        <v>2221.252384174215</v>
       </c>
       <c r="N116" t="n">
-        <v>2528.748418638445</v>
+        <v>2528.706528479863</v>
       </c>
       <c r="O116" t="n">
-        <v>-12.33511493915154</v>
+        <v>-12.60378481094645</v>
       </c>
       <c r="P116" t="n">
-        <v>31.70367705553691</v>
+        <v>30.42459801618134</v>
       </c>
       <c r="Q116" t="n">
-        <v>-68.29632294446309</v>
+        <v>-69.57540198381865</v>
       </c>
       <c r="R116" t="n">
-        <v>-77.54968253549303</v>
+        <v>-78.52059058609963</v>
       </c>
       <c r="S116" t="n">
-        <v>-10.43048144819512</v>
+        <v>-10.60878027636939</v>
       </c>
       <c r="T116" t="inlineStr">
         <is>
@@ -11162,10 +11166,10 @@
       </c>
       <c r="V116" t="inlineStr"/>
       <c r="W116" t="n">
-        <v>28</v>
+        <v>27.9</v>
       </c>
       <c r="X116" t="n">
-        <v>78</v>
+        <v>78.09999999999999</v>
       </c>
       <c r="Y116" t="inlineStr">
         <is>
@@ -16689,52 +16693,52 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>158.8950042724609</v>
+        <v>158.8699951171875</v>
       </c>
       <c r="E59" t="n">
-        <v>-0.07735042226556521</v>
+        <v>-0.09307766976502929</v>
       </c>
       <c r="F59" t="n">
-        <v>-0.5333369502995455</v>
+        <v>-0.5489924281550596</v>
       </c>
       <c r="G59" t="n">
-        <v>1.380710533384377</v>
+        <v>1.364753795517948</v>
       </c>
       <c r="H59" t="n">
-        <v>6.930880853266563</v>
+        <v>6.914050550671269</v>
       </c>
       <c r="I59" t="n">
-        <v>56.462210134142</v>
+        <v>56.38290723045462</v>
       </c>
       <c r="J59" t="n">
         <v>10.58957675968701</v>
       </c>
       <c r="K59" t="n">
-        <v>0.6529190656177376</v>
+        <v>0.6500713545183054</v>
       </c>
       <c r="L59" t="n">
-        <v>157.4805174086109</v>
+        <v>157.4781355842991</v>
       </c>
       <c r="M59" t="n">
-        <v>154.8032819016445</v>
+        <v>154.8023011504573</v>
       </c>
       <c r="N59" t="n">
-        <v>145.5023379046181</v>
+        <v>145.5020890573019</v>
       </c>
       <c r="O59" t="n">
-        <v>-0.213138660418962</v>
+        <v>-0.2147346862825763</v>
       </c>
       <c r="P59" t="n">
-        <v>73.05812763053122</v>
+        <v>72.68524627459902</v>
       </c>
       <c r="Q59" t="n">
-        <v>-26.94187236946878</v>
+        <v>-27.31475372540098</v>
       </c>
       <c r="R59" t="n">
-        <v>47.11970561662537</v>
+        <v>46.84461525717781</v>
       </c>
       <c r="S59" t="n">
-        <v>1.2844207846332</v>
+        <v>1.268479202216688</v>
       </c>
       <c r="T59" t="inlineStr">
         <is>
@@ -17061,52 +17065,52 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>1.350894927978516</v>
+        <v>1.350566625595093</v>
       </c>
       <c r="E63" t="n">
-        <v>0.5687233738171482</v>
+        <v>0.5442825746864388</v>
       </c>
       <c r="F63" t="n">
-        <v>0.316109025346889</v>
+        <v>0.291729618032055</v>
       </c>
       <c r="G63" t="n">
-        <v>0.2620745999095675</v>
+        <v>0.2377083243567224</v>
       </c>
       <c r="H63" t="n">
-        <v>4.171568230457412</v>
+        <v>4.146251846905558</v>
       </c>
       <c r="I63" t="n">
-        <v>52.72294075196015</v>
+        <v>52.61350507125866</v>
       </c>
       <c r="J63" t="n">
-        <v>11.10477856791236</v>
+        <v>11.10344450471869</v>
       </c>
       <c r="K63" t="n">
-        <v>0.5789555779293744</v>
+        <v>0.5726803758139501</v>
       </c>
       <c r="L63" t="n">
-        <v>1.3450438271134</v>
+        <v>1.34501256021974</v>
       </c>
       <c r="M63" t="n">
-        <v>1.336993760279298</v>
+        <v>1.336980885676026</v>
       </c>
       <c r="N63" t="n">
-        <v>1.305115883664347</v>
+        <v>1.305112616973965</v>
       </c>
       <c r="O63" t="n">
-        <v>-1.565877062598533e-05</v>
+        <v>-3.66102617617753e-05</v>
       </c>
       <c r="P63" t="n">
-        <v>70.02066596740009</v>
+        <v>69.35964303801721</v>
       </c>
       <c r="Q63" t="n">
-        <v>-29.9793340325999</v>
+        <v>-30.64035696198278</v>
       </c>
       <c r="R63" t="n">
-        <v>7.702090583851151</v>
+        <v>7.079978873523908</v>
       </c>
       <c r="S63" t="n">
-        <v>0.5279342434799439</v>
+        <v>0.5035033571621605</v>
       </c>
       <c r="T63" t="inlineStr">
         <is>
@@ -17116,7 +17120,7 @@
       <c r="U63" t="inlineStr"/>
       <c r="V63" t="inlineStr">
         <is>
-          <t>Double Top, Double Bottom</t>
+          <t>Double Top, Double Bottom, Volatility Squeeze</t>
         </is>
       </c>
       <c r="W63" t="n">
@@ -18163,66 +18167,66 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>EURUSD</t>
+          <t>V</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>EUR/USD</t>
+          <t>Visa</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>FX/Macro</t>
+          <t>Azioni USA</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>1.164686679840088</v>
+        <v>328.8800048828125</v>
       </c>
       <c r="E75" t="n">
-        <v>0.221284690365553</v>
+        <v>0.9608610538181184</v>
       </c>
       <c r="F75" t="n">
-        <v>-0.3167893886727002</v>
+        <v>3.741094025660674</v>
       </c>
       <c r="G75" t="n">
-        <v>-0.881667313583856</v>
+        <v>-7.3577451034331</v>
       </c>
       <c r="H75" t="n">
-        <v>7.278125961458004</v>
+        <v>-0.8800431035513534</v>
       </c>
       <c r="I75" t="n">
-        <v>49.24280346298583</v>
+        <v>52.95237519130382</v>
       </c>
       <c r="J75" t="n">
-        <v>17.2833888244175</v>
+        <v>27.77548190956076</v>
       </c>
       <c r="K75" t="n">
-        <v>0.3988124283578505</v>
+        <v>0.7044218044939171</v>
       </c>
       <c r="L75" t="n">
-        <v>1.167225823633194</v>
+        <v>320.8600168106299</v>
       </c>
       <c r="M75" t="n">
-        <v>1.157431950395351</v>
+        <v>325.8391032128765</v>
       </c>
       <c r="N75" t="n">
-        <v>1.12207996859848</v>
+        <v>288.6760504158779</v>
       </c>
       <c r="O75" t="n">
-        <v>-0.001017683830873413</v>
+        <v>2.692434862859466</v>
       </c>
       <c r="P75" t="n">
-        <v>53.09168151670184</v>
+        <v>72.75939467436808</v>
       </c>
       <c r="Q75" t="n">
-        <v>-46.90831848329816</v>
+        <v>-27.24060532563191</v>
       </c>
       <c r="R75" t="n">
-        <v>-39.48952992513703</v>
+        <v>46.97949264557219</v>
       </c>
       <c r="S75" t="n">
-        <v>-0.09434188000276844</v>
+        <v>-5.079659878044196</v>
       </c>
       <c r="T75" t="inlineStr">
         <is>
@@ -18232,14 +18236,14 @@
       <c r="U75" t="inlineStr"/>
       <c r="V75" t="inlineStr">
         <is>
-          <t>Double Top, Double Bottom, Inside Bar</t>
+          <t>Double Top</t>
         </is>
       </c>
       <c r="W75" t="n">
-        <v>54.1</v>
+        <v>54</v>
       </c>
       <c r="X75" t="n">
-        <v>56.1</v>
+        <v>61.2</v>
       </c>
       <c r="Y75" t="inlineStr">
         <is>
@@ -18248,73 +18252,73 @@
       </c>
       <c r="Z75" t="inlineStr">
         <is>
-          <t>pattern: Double Bottom; in zona Fib Fib 23.6 — livello strutturale</t>
+          <t>trend in sviluppo (ADX 28); pattern: Double Top</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>EURUSD</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Visa</t>
+          <t>EUR/USD</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Azioni USA</t>
+          <t>FX/Macro</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>328.8800048828125</v>
+        <v>1.164279937744141</v>
       </c>
       <c r="E76" t="n">
-        <v>0.9608610538181184</v>
+        <v>0.1862845344445807</v>
       </c>
       <c r="F76" t="n">
-        <v>3.741094025660674</v>
+        <v>-0.3516016336451933</v>
       </c>
       <c r="G76" t="n">
-        <v>-7.3577451034331</v>
+        <v>-0.9162822869337783</v>
       </c>
       <c r="H76" t="n">
-        <v>-0.8800431035513534</v>
+        <v>7.24066135354402</v>
       </c>
       <c r="I76" t="n">
-        <v>52.95237519130382</v>
+        <v>49.04392101428784</v>
       </c>
       <c r="J76" t="n">
-        <v>27.77548190956076</v>
+        <v>17.2833888244175</v>
       </c>
       <c r="K76" t="n">
-        <v>0.7044218044939171</v>
+        <v>0.3906069218412305</v>
       </c>
       <c r="L76" t="n">
-        <v>320.8600168106299</v>
+        <v>1.167187086290723</v>
       </c>
       <c r="M76" t="n">
-        <v>325.8391032128765</v>
+        <v>1.157415999724921</v>
       </c>
       <c r="N76" t="n">
-        <v>288.6760504158779</v>
+        <v>1.122075921413446</v>
       </c>
       <c r="O76" t="n">
-        <v>2.692434862859466</v>
+        <v>-0.001043641161212978</v>
       </c>
       <c r="P76" t="n">
-        <v>72.75939467436808</v>
+        <v>52.1577032675552</v>
       </c>
       <c r="Q76" t="n">
-        <v>-27.24060532563191</v>
+        <v>-47.84229673244479</v>
       </c>
       <c r="R76" t="n">
-        <v>46.97949264557219</v>
+        <v>-40.39525437265983</v>
       </c>
       <c r="S76" t="n">
-        <v>-5.079659878044196</v>
+        <v>-0.129231810044983</v>
       </c>
       <c r="T76" t="inlineStr">
         <is>
@@ -18324,14 +18328,14 @@
       <c r="U76" t="inlineStr"/>
       <c r="V76" t="inlineStr">
         <is>
-          <t>Double Top</t>
+          <t>Double Top, Double Bottom, Inside Bar</t>
         </is>
       </c>
       <c r="W76" t="n">
         <v>54</v>
       </c>
       <c r="X76" t="n">
-        <v>61.2</v>
+        <v>56</v>
       </c>
       <c r="Y76" t="inlineStr">
         <is>
@@ -18340,7 +18344,7 @@
       </c>
       <c r="Z76" t="inlineStr">
         <is>
-          <t>trend in sviluppo (ADX 28); pattern: Double Top</t>
+          <t>pattern: Double Bottom; in zona Fib Fib 23.6 — livello strutturale</t>
         </is>
       </c>
     </row>
@@ -19097,52 +19101,52 @@
         </is>
       </c>
       <c r="D85" t="n">
-        <v>77280.0390625</v>
+        <v>77285.0234375</v>
       </c>
       <c r="E85" t="n">
-        <v>0.3882952639364445</v>
+        <v>0.3947700653894159</v>
       </c>
       <c r="F85" t="n">
-        <v>-1.751262519038976</v>
+        <v>-1.744925713871393</v>
       </c>
       <c r="G85" t="n">
-        <v>-15.46101432818101</v>
+        <v>-15.45556176873849</v>
       </c>
       <c r="H85" t="n">
-        <v>-10.19626943720177</v>
+        <v>-10.19047731448866</v>
       </c>
       <c r="I85" t="n">
-        <v>46.20191620734643</v>
+        <v>46.20812259641718</v>
       </c>
       <c r="J85" t="n">
         <v>39.73448181746351</v>
       </c>
       <c r="K85" t="n">
-        <v>0.5991465500754584</v>
+        <v>0.5993048604406241</v>
       </c>
       <c r="L85" t="n">
-        <v>78071.2954903991</v>
+        <v>78071.77019278007</v>
       </c>
       <c r="M85" t="n">
-        <v>84857.90640135838</v>
+        <v>84858.10186704465</v>
       </c>
       <c r="N85" t="n">
-        <v>69068.5217720073</v>
+        <v>69068.57136777844</v>
       </c>
       <c r="O85" t="n">
-        <v>1951.015329729778</v>
+        <v>1951.33342089787</v>
       </c>
       <c r="P85" t="n">
-        <v>72.76463515138414</v>
+        <v>72.78926269833764</v>
       </c>
       <c r="Q85" t="n">
-        <v>-27.23536484861586</v>
+        <v>-27.21073730166236</v>
       </c>
       <c r="R85" t="n">
-        <v>14.6027042580682</v>
+        <v>14.61166226488456</v>
       </c>
       <c r="S85" t="n">
-        <v>-14.91555718410121</v>
+        <v>-14.91006944399645</v>
       </c>
       <c r="T85" t="inlineStr">
         <is>
@@ -20291,87 +20295,87 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>ETH</t>
+          <t>US2Y</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Ethereum</t>
+          <t>US Treasury 1-3Y ETF</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Crypto</t>
+          <t>Bond</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>2114.89990234375</v>
+        <v>82.12000274658203</v>
       </c>
       <c r="E98" t="n">
-        <v>0.8058176855378241</v>
+        <v>0.07312355565869399</v>
       </c>
       <c r="F98" t="n">
-        <v>-10.75351236966088</v>
+        <v>-0.6292311797034489</v>
       </c>
       <c r="G98" t="n">
-        <v>-32.66173572702857</v>
+        <v>-0.8092742620318671</v>
       </c>
       <c r="H98" t="n">
-        <v>5.465553884297414</v>
+        <v>-0.3639837770298748</v>
       </c>
       <c r="I98" t="n">
-        <v>39.86694005758697</v>
+        <v>37.6045789973985</v>
       </c>
       <c r="J98" t="n">
-        <v>31.27410151462559</v>
+        <v>20.53341526844853</v>
       </c>
       <c r="K98" t="n">
-        <v>0.4173885881260038</v>
+        <v>0.1251952687362177</v>
       </c>
       <c r="L98" t="n">
-        <v>2347.365763671929</v>
+        <v>82.51472921149627</v>
       </c>
       <c r="M98" t="n">
-        <v>2677.111177215168</v>
+        <v>82.60273548624369</v>
       </c>
       <c r="N98" t="n">
-        <v>2548.92842992531</v>
+        <v>82.65215982067235</v>
       </c>
       <c r="O98" t="n">
-        <v>41.20518235627196</v>
+        <v>-0.06232869820654374</v>
       </c>
       <c r="P98" t="n">
-        <v>47.04108693551448</v>
+        <v>10.00025431379779</v>
       </c>
       <c r="Q98" t="n">
-        <v>-52.95891306448552</v>
+        <v>-89.9997456862022</v>
       </c>
       <c r="R98" t="n">
-        <v>-16.86844598964621</v>
+        <v>-136.8409919792621</v>
       </c>
       <c r="S98" t="n">
-        <v>-32.19051904218206</v>
+        <v>-0.89307006796846</v>
       </c>
       <c r="T98" t="inlineStr">
         <is>
-          <t>Range</t>
+          <t>Trend Bearish</t>
         </is>
       </c>
       <c r="U98" t="inlineStr">
         <is>
-          <t>Piercing Pattern</t>
+          <t>Doji, Bullish Harami</t>
         </is>
       </c>
       <c r="V98" t="inlineStr">
         <is>
-          <t>Inside Bar, Bull Flag / Consolidation</t>
+          <t>Double Top, Double Bottom</t>
         </is>
       </c>
       <c r="W98" t="n">
-        <v>39.3</v>
+        <v>38.9</v>
       </c>
       <c r="X98" t="n">
-        <v>73.8</v>
+        <v>70.3</v>
       </c>
       <c r="Y98" t="inlineStr">
         <is>
@@ -20380,94 +20384,94 @@
       </c>
       <c r="Z98" t="inlineStr">
         <is>
-          <t>trend molto direzionale (ADX 31); pattern: Bull Flag / Consolidation; segnale candlestick: Piercing Pattern</t>
+          <t>EMA allineate al ribasso (EMA20&lt;EMA50&lt;EMA200); trend in sviluppo (ADX 21); RSI scarico (38) — zona di interesse long; pattern: Double Bottom; doji — indecisione del mercato; sul supporto dei 20g (82.00); vicino alla resistenza dei 20g (83.20)</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>US2Y</t>
+          <t>PALLADIUM</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>US Treasury 1-3Y ETF</t>
+          <t>Palladium</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Bond</t>
+          <t>Commodities</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>82.12000274658203</v>
+        <v>1360.300048828125</v>
       </c>
       <c r="E99" t="n">
-        <v>0.07312355565869399</v>
+        <v>0.1693703113494038</v>
       </c>
       <c r="F99" t="n">
-        <v>-0.6292311797034489</v>
+        <v>-9.40392615197303</v>
       </c>
       <c r="G99" t="n">
-        <v>-0.8092742620318671</v>
+        <v>-18.44723927888939</v>
       </c>
       <c r="H99" t="n">
-        <v>-0.3639837770298748</v>
+        <v>43.00883424842219</v>
       </c>
       <c r="I99" t="n">
-        <v>37.6045789973985</v>
+        <v>42.60350580589397</v>
       </c>
       <c r="J99" t="n">
-        <v>20.53341526844853</v>
+        <v>26.53773457615651</v>
       </c>
       <c r="K99" t="n">
-        <v>0.1251952687362177</v>
+        <v>0.1727757723383724</v>
       </c>
       <c r="L99" t="n">
-        <v>82.51472921149627</v>
+        <v>1511.980699505505</v>
       </c>
       <c r="M99" t="n">
-        <v>82.60273548624369</v>
+        <v>1438.697354415907</v>
       </c>
       <c r="N99" t="n">
-        <v>82.65215982067235</v>
+        <v>1372.713817705288</v>
       </c>
       <c r="O99" t="n">
-        <v>-0.06232869820654374</v>
+        <v>-40.40031411387112</v>
       </c>
       <c r="P99" t="n">
-        <v>10.00025431379779</v>
+        <v>3.794687807644279</v>
       </c>
       <c r="Q99" t="n">
-        <v>-89.9997456862022</v>
+        <v>-96.20531219235572</v>
       </c>
       <c r="R99" t="n">
-        <v>-136.8409919792621</v>
+        <v>-80.71923537662148</v>
       </c>
       <c r="S99" t="n">
-        <v>-0.89307006796846</v>
+        <v>-26.58931198984754</v>
       </c>
       <c r="T99" t="inlineStr">
         <is>
-          <t>Trend Bearish</t>
+          <t>Range</t>
         </is>
       </c>
       <c r="U99" t="inlineStr">
         <is>
-          <t>Doji, Bullish Harami</t>
+          <t>Doji, Shooting Star</t>
         </is>
       </c>
       <c r="V99" t="inlineStr">
         <is>
-          <t>Double Top, Double Bottom</t>
+          <t>Double Top, Inside Bar</t>
         </is>
       </c>
       <c r="W99" t="n">
-        <v>38.9</v>
+        <v>38.5</v>
       </c>
       <c r="X99" t="n">
-        <v>70.3</v>
+        <v>76.2</v>
       </c>
       <c r="Y99" t="inlineStr">
         <is>
@@ -20476,94 +20480,90 @@
       </c>
       <c r="Z99" t="inlineStr">
         <is>
-          <t>EMA allineate al ribasso (EMA20&lt;EMA50&lt;EMA200); trend in sviluppo (ADX 21); RSI scarico (38) — zona di interesse long; pattern: Double Bottom; doji — indecisione del mercato; sul supporto dei 20g (82.00); vicino alla resistenza dei 20g (83.20)</t>
+          <t>trend in sviluppo (ADX 27); pattern: Double Top; doji — indecisione del mercato; sul supporto dei 20g (1,341)</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>PALLADIUM</t>
+          <t>ETH</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Palladium</t>
+          <t>Ethereum</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Commodities</t>
+          <t>Crypto</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>1360.300048828125</v>
+        <v>2110.68994140625</v>
       </c>
       <c r="E100" t="n">
-        <v>0.1693703113494038</v>
+        <v>0.6051516614585806</v>
       </c>
       <c r="F100" t="n">
-        <v>-9.40392615197303</v>
+        <v>-10.93116816619121</v>
       </c>
       <c r="G100" t="n">
-        <v>-18.44723927888939</v>
+        <v>-32.79578058743737</v>
       </c>
       <c r="H100" t="n">
-        <v>43.00883424842219</v>
+        <v>5.255612098583273</v>
       </c>
       <c r="I100" t="n">
-        <v>42.60350580589397</v>
+        <v>39.72844952803676</v>
       </c>
       <c r="J100" t="n">
-        <v>26.53773457615651</v>
+        <v>31.27410151462559</v>
       </c>
       <c r="K100" t="n">
-        <v>0.1727757723383724</v>
+        <v>0.4143139330364269</v>
       </c>
       <c r="L100" t="n">
-        <v>1511.980699505505</v>
+        <v>2346.964815011214</v>
       </c>
       <c r="M100" t="n">
-        <v>1438.697354415907</v>
+        <v>2676.946080707815</v>
       </c>
       <c r="N100" t="n">
-        <v>1372.713817705288</v>
+        <v>2548.886539766728</v>
       </c>
       <c r="O100" t="n">
-        <v>-40.40031411387112</v>
+        <v>40.93651248447742</v>
       </c>
       <c r="P100" t="n">
-        <v>3.794687807644279</v>
+        <v>46.40386075403251</v>
       </c>
       <c r="Q100" t="n">
-        <v>-96.20531219235572</v>
+        <v>-53.59613924596749</v>
       </c>
       <c r="R100" t="n">
-        <v>-80.71923537662148</v>
+        <v>-17.02875336350607</v>
       </c>
       <c r="S100" t="n">
-        <v>-26.58931198984754</v>
+        <v>-32.32550191570162</v>
       </c>
       <c r="T100" t="inlineStr">
         <is>
           <t>Range</t>
         </is>
       </c>
-      <c r="U100" t="inlineStr">
-        <is>
-          <t>Doji, Shooting Star</t>
-        </is>
-      </c>
+      <c r="U100" t="inlineStr"/>
       <c r="V100" t="inlineStr">
         <is>
-          <t>Double Top, Inside Bar</t>
+          <t>Inside Bar, Bull Flag / Consolidation</t>
         </is>
       </c>
       <c r="W100" t="n">
-        <v>38.5</v>
+        <v>37.8</v>
       </c>
       <c r="X100" t="n">
-        <v>76.2</v>
+        <v>71.3</v>
       </c>
       <c r="Y100" t="inlineStr">
         <is>
@@ -20572,7 +20572,7 @@
       </c>
       <c r="Z100" t="inlineStr">
         <is>
-          <t>trend in sviluppo (ADX 27); pattern: Double Top; doji — indecisione del mercato; sul supporto dei 20g (1,341)</t>
+          <t>trend molto direzionale (ADX 31); pattern: Bull Flag / Consolidation</t>
         </is>
       </c>
     </row>
@@ -20685,52 +20685,52 @@
         </is>
       </c>
       <c r="D102" t="n">
-        <v>85.47000122070312</v>
+        <v>85.45999908447266</v>
       </c>
       <c r="E102" t="n">
-        <v>0.2584248505975717</v>
+        <v>0.2466920974761866</v>
       </c>
       <c r="F102" t="n">
-        <v>-1.725163697470622</v>
+        <v>-1.736664320925463</v>
       </c>
       <c r="G102" t="n">
-        <v>-36.16859700213498</v>
+        <v>-36.1760668790444</v>
       </c>
       <c r="H102" t="n">
-        <v>-35.54265469079563</v>
+        <v>-35.55019781867242</v>
       </c>
       <c r="I102" t="n">
-        <v>38.48843930563677</v>
+        <v>38.48150442873197</v>
       </c>
       <c r="J102" t="n">
         <v>49.21776064464172</v>
       </c>
       <c r="K102" t="n">
-        <v>0.4129867792723947</v>
+        <v>0.4128212473515054</v>
       </c>
       <c r="L102" t="n">
-        <v>96.69322535421418</v>
+        <v>96.69227276981128</v>
       </c>
       <c r="M102" t="n">
-        <v>122.6755980011857</v>
+        <v>122.6752057605492</v>
       </c>
       <c r="N102" t="n">
-        <v>116.0167511260987</v>
+        <v>116.0166516023551</v>
       </c>
       <c r="O102" t="n">
-        <v>3.067930719815742</v>
+        <v>3.067292406848324</v>
       </c>
       <c r="P102" t="n">
-        <v>42.46980265396393</v>
+        <v>42.42483591083208</v>
       </c>
       <c r="Q102" t="n">
-        <v>-57.53019734603607</v>
+        <v>-57.57516408916792</v>
       </c>
       <c r="R102" t="n">
-        <v>-13.38881077023896</v>
+        <v>-13.39556583800539</v>
       </c>
       <c r="S102" t="n">
-        <v>-38.72699306809812</v>
+        <v>-38.73416354842841</v>
       </c>
       <c r="T102" t="inlineStr">
         <is>
@@ -21249,52 +21249,52 @@
         </is>
       </c>
       <c r="D108" t="n">
-        <v>1.353500008583069</v>
+        <v>1.354699969291687</v>
       </c>
       <c r="E108" t="n">
-        <v>0.2568058449621269</v>
+        <v>0.3456896477125104</v>
       </c>
       <c r="F108" t="n">
-        <v>-5.453778903200379</v>
+        <v>-5.369957883809873</v>
       </c>
       <c r="G108" t="n">
-        <v>-35.23988148547663</v>
+        <v>-35.18246767150538</v>
       </c>
       <c r="H108" t="n">
-        <v>-44.42603559911418</v>
+        <v>-44.37676587375007</v>
       </c>
       <c r="I108" t="n">
-        <v>36.84207667020258</v>
+        <v>36.91052007889797</v>
       </c>
       <c r="J108" t="n">
         <v>35.86970734861186</v>
       </c>
       <c r="K108" t="n">
-        <v>0.3594781022771072</v>
+        <v>0.3610998231863631</v>
       </c>
       <c r="L108" t="n">
-        <v>1.526472412542831</v>
+        <v>1.52658669451508</v>
       </c>
       <c r="M108" t="n">
-        <v>1.799815676842058</v>
+        <v>1.799862734124749</v>
       </c>
       <c r="N108" t="n">
-        <v>1.416174154987639</v>
+        <v>1.416186094895188</v>
       </c>
       <c r="O108" t="n">
-        <v>0.03372847929233208</v>
+        <v>0.03380505798142905</v>
       </c>
       <c r="P108" t="n">
-        <v>24.52398351704119</v>
+        <v>24.88886182327508</v>
       </c>
       <c r="Q108" t="n">
-        <v>-75.47601648295881</v>
+        <v>-75.11113817672492</v>
       </c>
       <c r="R108" t="n">
-        <v>-20.74973653892273</v>
+        <v>-20.68467407429605</v>
       </c>
       <c r="S108" t="n">
-        <v>-34.6471481151133</v>
+        <v>-34.58920880668279</v>
       </c>
       <c r="T108" t="inlineStr">
         <is>
@@ -21311,7 +21311,7 @@
         <v>32.4</v>
       </c>
       <c r="X108" t="n">
-        <v>68.7</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="Y108" t="inlineStr">
         <is>
@@ -21529,52 +21529,52 @@
         </is>
       </c>
       <c r="D111" t="n">
-        <v>9.522000312805176</v>
+        <v>9.510000228881836</v>
       </c>
       <c r="E111" t="n">
-        <v>0.9863231834294384</v>
+        <v>0.8590553496234499</v>
       </c>
       <c r="F111" t="n">
-        <v>0.2940956959148089</v>
+        <v>0.1677002405662265</v>
       </c>
       <c r="G111" t="n">
-        <v>-28.93371905200555</v>
+        <v>-29.02328020591023</v>
       </c>
       <c r="H111" t="n">
-        <v>-34.0384812813282</v>
+        <v>-34.12160916773151</v>
       </c>
       <c r="I111" t="n">
-        <v>42.46136072720428</v>
+        <v>42.38996238298512</v>
       </c>
       <c r="J111" t="n">
         <v>45.80678007727939</v>
       </c>
       <c r="K111" t="n">
-        <v>0.5176955316408393</v>
+        <v>0.5152884432440258</v>
       </c>
       <c r="L111" t="n">
-        <v>10.20190474299847</v>
+        <v>10.20076187786291</v>
       </c>
       <c r="M111" t="n">
-        <v>12.53264962158528</v>
+        <v>12.53217903005887</v>
       </c>
       <c r="N111" t="n">
-        <v>13.46313319260038</v>
+        <v>13.46301378878025</v>
       </c>
       <c r="O111" t="n">
-        <v>0.3763527669167934</v>
+        <v>0.3755869495951889</v>
       </c>
       <c r="P111" t="n">
-        <v>52.02165528038958</v>
+        <v>51.58943588894541</v>
       </c>
       <c r="Q111" t="n">
-        <v>-47.97834471961042</v>
+        <v>-48.41056411105459</v>
       </c>
       <c r="R111" t="n">
-        <v>-1.422273755328402</v>
+        <v>-1.518817741909937</v>
       </c>
       <c r="S111" t="n">
-        <v>-27.72222835121503</v>
+        <v>-27.81331628411617</v>
       </c>
       <c r="T111" t="inlineStr">
         <is>
@@ -21809,52 +21809,52 @@
         </is>
       </c>
       <c r="D114" t="n">
-        <v>0.2449000030755997</v>
+        <v>0.2445999979972839</v>
       </c>
       <c r="E114" t="n">
-        <v>1.144433362738217</v>
+        <v>1.020530368572792</v>
       </c>
       <c r="F114" t="n">
-        <v>-2.94378946848739</v>
+        <v>-3.062684346706512</v>
       </c>
       <c r="G114" t="n">
-        <v>-38.78892359573226</v>
+        <v>-38.86390780781814</v>
       </c>
       <c r="H114" t="n">
-        <v>-65.48312317087421</v>
+        <v>-65.52540670785376</v>
       </c>
       <c r="I114" t="n">
-        <v>35.30738174329389</v>
+        <v>35.24593531685518</v>
       </c>
       <c r="J114" t="n">
         <v>40.22919263312446</v>
       </c>
       <c r="K114" t="n">
-        <v>0.3338180019543226</v>
+        <v>0.3318148056178002</v>
       </c>
       <c r="L114" t="n">
-        <v>0.2952553840945915</v>
+        <v>0.295226812182371</v>
       </c>
       <c r="M114" t="n">
-        <v>0.4246822695263598</v>
+        <v>0.4246705046213279</v>
       </c>
       <c r="N114" t="n">
-        <v>0.5393885910192036</v>
+        <v>0.5393856058940462</v>
       </c>
       <c r="O114" t="n">
-        <v>0.01457182661862066</v>
+        <v>0.01455268099538912</v>
       </c>
       <c r="P114" t="n">
-        <v>13.14928894410395</v>
+        <v>12.76318196794313</v>
       </c>
       <c r="Q114" t="n">
-        <v>-86.85071105589604</v>
+        <v>-87.23681803205687</v>
       </c>
       <c r="R114" t="n">
-        <v>-17.31949942349831</v>
+        <v>-17.37609666265417</v>
       </c>
       <c r="S114" t="n">
-        <v>-37.25098010498182</v>
+        <v>-37.32784831401174</v>
       </c>
       <c r="T114" t="inlineStr">
         <is>
@@ -21997,52 +21997,52 @@
         </is>
       </c>
       <c r="D116" t="n">
-        <v>1.269999980926514</v>
+        <v>1.274999976158142</v>
       </c>
       <c r="E116" t="n">
-        <v>2.037536023351483</v>
+        <v>2.439258229041319</v>
       </c>
       <c r="F116" t="n">
-        <v>0.6101564814476435</v>
+        <v>1.006259087916694</v>
       </c>
       <c r="G116" t="n">
-        <v>-40.65004371499583</v>
+        <v>-40.41638268910677</v>
       </c>
       <c r="H116" t="n">
-        <v>-71.75229380177693</v>
+        <v>-71.6410824644409</v>
       </c>
       <c r="I116" t="n">
-        <v>35.316982553975</v>
+        <v>35.51284228660265</v>
       </c>
       <c r="J116" t="n">
         <v>26.05081721968851</v>
       </c>
       <c r="K116" t="n">
-        <v>0.3604430717943172</v>
+        <v>0.3658438471609581</v>
       </c>
       <c r="L116" t="n">
-        <v>1.516041285527757</v>
+        <v>1.516517475549817</v>
       </c>
       <c r="M116" t="n">
-        <v>2.404628382659237</v>
+        <v>2.404824460903614</v>
       </c>
       <c r="N116" t="n">
-        <v>5.609546708089879</v>
+        <v>5.609596459286213</v>
       </c>
       <c r="O116" t="n">
-        <v>0.07741920880592407</v>
+        <v>0.07773829682070599</v>
       </c>
       <c r="P116" t="n">
-        <v>20.34976070118206</v>
+        <v>21.18693730646416</v>
       </c>
       <c r="Q116" t="n">
-        <v>-79.65023929881794</v>
+        <v>-78.81306269353584</v>
       </c>
       <c r="R116" t="n">
-        <v>-17.85597427842953</v>
+        <v>-17.66994034680465</v>
       </c>
       <c r="S116" t="n">
-        <v>-38.5334950049203</v>
+        <v>-38.29150111791564</v>
       </c>
       <c r="T116" t="inlineStr">
         <is>
@@ -22072,7 +22072,7 @@
       </c>
       <c r="Z116" t="inlineStr">
         <is>
-          <t>EMA e SMA allineate al ribasso — struttura bearish solida; trend in sviluppo (ADX 26); RSI scarico (35) — zona di interesse long; candela di inversione bullish (engulfing)</t>
+          <t>EMA e SMA allineate al ribasso — struttura bearish solida; trend in sviluppo (ADX 26); RSI scarico (36) — zona di interesse long; candela di inversione bullish (engulfing)</t>
         </is>
       </c>
     </row>
@@ -27737,66 +27737,66 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>XLV</t>
+          <t>USDJPY</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>USD/JPY</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Settoriali</t>
+          <t>FX/Macro</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>149.8899993896484</v>
+        <v>158.8699951171875</v>
       </c>
       <c r="E61" t="n">
-        <v>2.671411569107041</v>
+        <v>-0.82031324792321</v>
       </c>
       <c r="F61" t="n">
-        <v>-3.171836928496508</v>
+        <v>1.57084182301237</v>
       </c>
       <c r="G61" t="n">
-        <v>-4.650125763679602</v>
+        <v>9.64869610492789</v>
       </c>
       <c r="H61" t="n">
-        <v>28.39643835231478</v>
+        <v>44.0279177531836</v>
       </c>
       <c r="I61" t="n">
-        <v>54.0276924129715</v>
+        <v>59.9651498619826</v>
       </c>
       <c r="J61" t="n">
-        <v>27.39184541707561</v>
+        <v>20.2697483957454</v>
       </c>
       <c r="K61" t="n">
-        <v>0.6450712695305483</v>
+        <v>0.8116156674265609</v>
       </c>
       <c r="L61" t="n">
-        <v>146.240990662911</v>
+        <v>152.9059987033013</v>
       </c>
       <c r="M61" t="n">
-        <v>138.3316249810972</v>
+        <v>144.7234797231319</v>
       </c>
       <c r="N61" t="n">
-        <v>114.368931294505</v>
+        <v>131.0044180674282</v>
       </c>
       <c r="O61" t="n">
-        <v>0.2031153142987767</v>
+        <v>0.5506131007248407</v>
       </c>
       <c r="P61" t="n">
-        <v>67.80987474158408</v>
+        <v>91.19653557256028</v>
       </c>
       <c r="Q61" t="n">
-        <v>-32.19012525841592</v>
+        <v>-8.803464427439721</v>
       </c>
       <c r="R61" t="n">
-        <v>30.26995588985354</v>
+        <v>88.06232718544621</v>
       </c>
       <c r="S61" t="n">
-        <v>-2.681473034831583</v>
+        <v>11.26674031226747</v>
       </c>
       <c r="T61" t="inlineStr">
         <is>
@@ -27810,10 +27810,10 @@
         </is>
       </c>
       <c r="W61" t="n">
-        <v>72.90000000000001</v>
+        <v>73</v>
       </c>
       <c r="X61" t="n">
-        <v>78.5</v>
+        <v>75.09999999999999</v>
       </c>
       <c r="Y61" t="inlineStr">
         <is>
@@ -27822,73 +27822,73 @@
       </c>
       <c r="Z61" t="inlineStr">
         <is>
-          <t>EMA e SMA allineate al rialzo — struttura bullish solida; trend in sviluppo (ADX 27); pattern: Double Top</t>
+          <t>EMA e SMA allineate al rialzo — struttura bullish solida; trend in sviluppo (ADX 20); pattern: Double Top; vicino alla resistenza dei 20g (160.70)</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>USDJPY</t>
+          <t>XLV</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>USD/JPY</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>FX/Macro</t>
+          <t>Settoriali</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>158.8950042724609</v>
+        <v>149.8899993896484</v>
       </c>
       <c r="E62" t="n">
-        <v>-0.8047004811189806</v>
+        <v>2.671411569107041</v>
       </c>
       <c r="F62" t="n">
-        <v>1.586831003049349</v>
+        <v>-3.171836928496508</v>
       </c>
       <c r="G62" t="n">
-        <v>9.66595689268328</v>
+        <v>-4.650125763679602</v>
       </c>
       <c r="H62" t="n">
-        <v>44.05059048352607</v>
+        <v>28.39643835231478</v>
       </c>
       <c r="I62" t="n">
-        <v>60.00078455776788</v>
+        <v>54.0276924129715</v>
       </c>
       <c r="J62" t="n">
-        <v>20.2697483957454</v>
+        <v>27.39184541707561</v>
       </c>
       <c r="K62" t="n">
-        <v>0.8126358937882379</v>
+        <v>0.6450712695305483</v>
       </c>
       <c r="L62" t="n">
-        <v>152.908380527613</v>
+        <v>146.240990662911</v>
       </c>
       <c r="M62" t="n">
-        <v>144.7244604743191</v>
+        <v>138.3316249810972</v>
       </c>
       <c r="N62" t="n">
-        <v>131.0047805189539</v>
+        <v>114.368931294505</v>
       </c>
       <c r="O62" t="n">
-        <v>0.5522091265884548</v>
+        <v>0.2031153142987767</v>
       </c>
       <c r="P62" t="n">
-        <v>91.31671413194272</v>
+        <v>67.80987474158408</v>
       </c>
       <c r="Q62" t="n">
-        <v>-8.683285868057286</v>
+        <v>-32.19012525841592</v>
       </c>
       <c r="R62" t="n">
-        <v>88.17474475766802</v>
+        <v>30.26995588985354</v>
       </c>
       <c r="S62" t="n">
-        <v>11.28425581091896</v>
+        <v>-2.681473034831583</v>
       </c>
       <c r="T62" t="inlineStr">
         <is>
@@ -27902,10 +27902,10 @@
         </is>
       </c>
       <c r="W62" t="n">
-        <v>72.7</v>
+        <v>72.90000000000001</v>
       </c>
       <c r="X62" t="n">
-        <v>75.09999999999999</v>
+        <v>78.5</v>
       </c>
       <c r="Y62" t="inlineStr">
         <is>
@@ -27914,7 +27914,7 @@
       </c>
       <c r="Z62" t="inlineStr">
         <is>
-          <t>EMA e SMA allineate al rialzo — struttura bullish solida; trend in sviluppo (ADX 20); RSI in forza (60) — momentum positivo; pattern: Double Top; vicino alla resistenza dei 20g (160.70)</t>
+          <t>EMA e SMA allineate al rialzo — struttura bullish solida; trend in sviluppo (ADX 27); pattern: Double Top</t>
         </is>
       </c>
     </row>
@@ -29407,52 +29407,52 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>1.350894927978516</v>
+        <v>1.350566625595093</v>
       </c>
       <c r="E79" t="n">
-        <v>0.150887468067995</v>
+        <v>0.1265482138619767</v>
       </c>
       <c r="F79" t="n">
-        <v>0.3100263571973905</v>
+        <v>0.2856484281281269</v>
       </c>
       <c r="G79" t="n">
-        <v>2.603168348602014</v>
+        <v>2.578233126759111</v>
       </c>
       <c r="H79" t="n">
-        <v>-1.729146838774576</v>
+        <v>-1.753029196051692</v>
       </c>
       <c r="I79" t="n">
-        <v>55.45318337127343</v>
+        <v>55.40814945772713</v>
       </c>
       <c r="J79" t="n">
         <v>23.83028542371799</v>
       </c>
       <c r="K79" t="n">
-        <v>0.6828863114468039</v>
+        <v>0.6809902891045472</v>
       </c>
       <c r="L79" t="n">
-        <v>1.32611903230066</v>
+        <v>1.326087765407</v>
       </c>
       <c r="M79" t="n">
-        <v>1.306032675596496</v>
+        <v>1.306019800993224</v>
       </c>
       <c r="N79" t="n">
-        <v>1.341609903293911</v>
+        <v>1.341605145288354</v>
       </c>
       <c r="O79" t="n">
-        <v>-3.076365077849322e-05</v>
+        <v>-5.17151419142832e-05</v>
       </c>
       <c r="P79" t="n">
-        <v>69.94364951333671</v>
+        <v>69.6515560816207</v>
       </c>
       <c r="Q79" t="n">
-        <v>-30.05635048666329</v>
+        <v>-30.3484439183793</v>
       </c>
       <c r="R79" t="n">
-        <v>55.22876401991392</v>
+        <v>55.04226008028867</v>
       </c>
       <c r="S79" t="n">
-        <v>0.9388669392780935</v>
+        <v>0.9143361856940535</v>
       </c>
       <c r="T79" t="inlineStr">
         <is>
@@ -29469,7 +29469,7 @@
         <v>59.6</v>
       </c>
       <c r="X79" t="n">
-        <v>67.3</v>
+        <v>67.2</v>
       </c>
       <c r="Y79" t="inlineStr">
         <is>
@@ -29577,83 +29577,83 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>EURUSD</t>
+          <t>XRP</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>EUR/USD</t>
+          <t>XRP</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>FX/Macro</t>
+          <t>Crypto</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>1.164686679840088</v>
+        <v>1.354699969291687</v>
       </c>
       <c r="E81" t="n">
-        <v>-0.3237862453742135</v>
+        <v>-0.9309436436792606</v>
       </c>
       <c r="F81" t="n">
-        <v>-0.8548819540785235</v>
+        <v>-26.37392020064773</v>
       </c>
       <c r="G81" t="n">
-        <v>5.11181383371353</v>
+        <v>139.213986171788</v>
       </c>
       <c r="H81" t="n">
-        <v>-0.6545547132576157</v>
+        <v>136.0643270553444</v>
       </c>
       <c r="I81" t="n">
-        <v>56.37064729976593</v>
+        <v>45.19711114308426</v>
       </c>
       <c r="J81" t="n">
-        <v>41.82770114805145</v>
+        <v>45.48102698280077</v>
       </c>
       <c r="K81" t="n">
-        <v>0.6580899121841214</v>
+        <v>0.2368726141490748</v>
       </c>
       <c r="L81" t="n">
-        <v>1.142772183562191</v>
+        <v>1.718164585505744</v>
       </c>
       <c r="M81" t="n">
-        <v>1.122062054858426</v>
+        <v>1.350795886610891</v>
       </c>
       <c r="N81" t="n">
-        <v>1.136432611356771</v>
+        <v>1.028834358201207</v>
       </c>
       <c r="O81" t="n">
-        <v>0.0014224996347682</v>
+        <v>-0.180545891312973</v>
       </c>
       <c r="P81" t="n">
-        <v>69.71841783481484</v>
+        <v>8.790699784975654</v>
       </c>
       <c r="Q81" t="n">
-        <v>-30.28158216518516</v>
+        <v>-91.20930021502434</v>
       </c>
       <c r="R81" t="n">
-        <v>52.24325987634691</v>
+        <v>-47.18197333971845</v>
       </c>
       <c r="S81" t="n">
-        <v>4.270900925514831</v>
+        <v>121.5401048022284</v>
       </c>
       <c r="T81" t="inlineStr">
         <is>
-          <t>Range</t>
-        </is>
-      </c>
-      <c r="U81" t="inlineStr"/>
-      <c r="V81" t="inlineStr">
-        <is>
-          <t>Double Bottom, Inside Bar</t>
-        </is>
-      </c>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="U81" t="inlineStr">
+        <is>
+          <t>Doji, Bearish Harami</t>
+        </is>
+      </c>
+      <c r="V81" t="inlineStr"/>
       <c r="W81" t="n">
-        <v>58.4</v>
+        <v>58.5</v>
       </c>
       <c r="X81" t="n">
-        <v>64.7</v>
+        <v>67.2</v>
       </c>
       <c r="Y81" t="inlineStr">
         <is>
@@ -29662,90 +29662,90 @@
       </c>
       <c r="Z81" t="inlineStr">
         <is>
-          <t>trend molto direzionale (ADX 42); pattern: Double Bottom; in zona Fib Fib 23.6 — livello strutturale</t>
+          <t>trend molto direzionale (ADX 45); doji — indecisione del mercato</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>XRP</t>
+          <t>EURUSD</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>XRP</t>
+          <t>EUR/USD</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Crypto</t>
+          <t>FX/Macro</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>1.353500008583069</v>
+        <v>1.164279937744141</v>
       </c>
       <c r="E82" t="n">
-        <v>-1.018696635310035</v>
+        <v>-0.3585960468430516</v>
       </c>
       <c r="F82" t="n">
-        <v>-26.43913641448953</v>
+        <v>-0.8895062816465793</v>
       </c>
       <c r="G82" t="n">
-        <v>139.0020961659823</v>
+        <v>5.075105764318066</v>
       </c>
       <c r="H82" t="n">
-        <v>135.8552269419659</v>
+        <v>-0.6892490008614582</v>
       </c>
       <c r="I82" t="n">
-        <v>45.1791473268999</v>
+        <v>56.28272325487121</v>
       </c>
       <c r="J82" t="n">
-        <v>45.48102698280077</v>
+        <v>41.82770114805145</v>
       </c>
       <c r="K82" t="n">
-        <v>0.2364573959916733</v>
+        <v>0.6562995380571306</v>
       </c>
       <c r="L82" t="n">
-        <v>1.718050303533494</v>
+        <v>1.14273344621972</v>
       </c>
       <c r="M82" t="n">
-        <v>1.350747888182546</v>
+        <v>1.122046104187997</v>
       </c>
       <c r="N82" t="n">
-        <v>1.028809869207153</v>
+        <v>1.136426716543786</v>
       </c>
       <c r="O82" t="n">
-        <v>-0.1806224700020699</v>
+        <v>0.001396542304428636</v>
       </c>
       <c r="P82" t="n">
-        <v>8.74302080311754</v>
+        <v>69.39145134025597</v>
       </c>
       <c r="Q82" t="n">
-        <v>-91.25697919688245</v>
+        <v>-30.60854865974402</v>
       </c>
       <c r="R82" t="n">
-        <v>-47.20841509210625</v>
+        <v>52.06970894581277</v>
       </c>
       <c r="S82" t="n">
-        <v>121.3438698962183</v>
+        <v>4.234486527099479</v>
       </c>
       <c r="T82" t="inlineStr">
         <is>
-          <t>Bullish</t>
-        </is>
-      </c>
-      <c r="U82" t="inlineStr">
-        <is>
-          <t>Doji, Bearish Harami</t>
-        </is>
-      </c>
-      <c r="V82" t="inlineStr"/>
+          <t>Range</t>
+        </is>
+      </c>
+      <c r="U82" t="inlineStr"/>
+      <c r="V82" t="inlineStr">
+        <is>
+          <t>Double Bottom, Inside Bar</t>
+        </is>
+      </c>
       <c r="W82" t="n">
-        <v>57.9</v>
+        <v>58.4</v>
       </c>
       <c r="X82" t="n">
-        <v>66.7</v>
+        <v>64.7</v>
       </c>
       <c r="Y82" t="inlineStr">
         <is>
@@ -29754,7 +29754,7 @@
       </c>
       <c r="Z82" t="inlineStr">
         <is>
-          <t>trend molto direzionale (ADX 45); doji — indecisione del mercato</t>
+          <t>trend molto direzionale (ADX 42); pattern: Double Bottom; in zona Fib Fib 23.6 — livello strutturale</t>
         </is>
       </c>
     </row>
@@ -29775,52 +29775,52 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>77280.0390625</v>
+        <v>77285.0234375</v>
       </c>
       <c r="E83" t="n">
-        <v>1.278720190421723</v>
+        <v>1.28525242212183</v>
       </c>
       <c r="F83" t="n">
-        <v>-11.68886531983827</v>
+        <v>-11.68316946593782</v>
       </c>
       <c r="G83" t="n">
-        <v>31.04997822644417</v>
+        <v>31.05843063204783</v>
       </c>
       <c r="H83" t="n">
-        <v>31.16356247780232</v>
+        <v>31.17202220931457</v>
       </c>
       <c r="I83" t="n">
-        <v>49.1190652137216</v>
+        <v>49.12162884487427</v>
       </c>
       <c r="J83" t="n">
         <v>31.03302765789525</v>
       </c>
       <c r="K83" t="n">
-        <v>0.2732652757903316</v>
+        <v>0.2733377595944074</v>
       </c>
       <c r="L83" t="n">
-        <v>82387.59308946253</v>
+        <v>82388.0677918435</v>
       </c>
       <c r="M83" t="n">
-        <v>66974.85716823765</v>
+        <v>66975.05654323765</v>
       </c>
       <c r="N83" t="n">
-        <v>49416.1563367731</v>
+        <v>49416.25805871188</v>
       </c>
       <c r="O83" t="n">
-        <v>-5353.431344097797</v>
+        <v>-5353.113252929705</v>
       </c>
       <c r="P83" t="n">
-        <v>26.02061353839355</v>
+        <v>26.02815147471217</v>
       </c>
       <c r="Q83" t="n">
-        <v>-73.97938646160644</v>
+        <v>-73.97184852528783</v>
       </c>
       <c r="R83" t="n">
-        <v>-35.78319332003179</v>
+        <v>-35.77915925383775</v>
       </c>
       <c r="S83" t="n">
-        <v>22.02850024475165</v>
+        <v>22.03637078691605</v>
       </c>
       <c r="T83" t="inlineStr">
         <is>
@@ -31249,52 +31249,52 @@
         </is>
       </c>
       <c r="D99" t="n">
-        <v>2114.89990234375</v>
+        <v>2110.68994140625</v>
       </c>
       <c r="E99" t="n">
-        <v>-6.264874986541836</v>
+        <v>-6.451465952072177</v>
       </c>
       <c r="F99" t="n">
-        <v>-28.72015157427155</v>
+        <v>-28.86204262886504</v>
       </c>
       <c r="G99" t="n">
-        <v>-15.85481338698987</v>
+        <v>-16.0223144343571</v>
       </c>
       <c r="H99" t="n">
-        <v>10.24508594278846</v>
+        <v>10.02562992746778</v>
       </c>
       <c r="I99" t="n">
-        <v>44.33932040315945</v>
+        <v>44.30447300811836</v>
       </c>
       <c r="J99" t="n">
         <v>14.47629393105002</v>
       </c>
       <c r="K99" t="n">
-        <v>0.2765368439606921</v>
+        <v>0.27534679589133</v>
       </c>
       <c r="L99" t="n">
-        <v>2693.148071618368</v>
+        <v>2692.747122957654</v>
       </c>
       <c r="M99" t="n">
-        <v>2484.742920642468</v>
+        <v>2484.574522204968</v>
       </c>
       <c r="N99" t="n">
-        <v>2000.001133808427</v>
+        <v>1999.915216238274</v>
       </c>
       <c r="O99" t="n">
-        <v>-162.8299649263068</v>
+        <v>-163.0986347981017</v>
       </c>
       <c r="P99" t="n">
-        <v>20.41250746056169</v>
+        <v>20.29448000569467</v>
       </c>
       <c r="Q99" t="n">
-        <v>-79.58749253943832</v>
+        <v>-79.70551999430533</v>
       </c>
       <c r="R99" t="n">
-        <v>-73.66017898700912</v>
+        <v>-73.79749367957039</v>
       </c>
       <c r="S99" t="n">
-        <v>-18.75340280965978</v>
+        <v>-18.91513386846643</v>
       </c>
       <c r="T99" t="inlineStr">
         <is>
@@ -31308,7 +31308,7 @@
       </c>
       <c r="V99" t="inlineStr"/>
       <c r="W99" t="n">
-        <v>41.2</v>
+        <v>41.1</v>
       </c>
       <c r="X99" t="n">
         <v>68.59999999999999</v>
@@ -31521,52 +31521,52 @@
         </is>
       </c>
       <c r="D102" t="n">
-        <v>85.47000122070312</v>
+        <v>85.45999908447266</v>
       </c>
       <c r="E102" t="n">
-        <v>2.94643767879148</v>
+        <v>2.934390360675199</v>
       </c>
       <c r="F102" t="n">
-        <v>-31.34083023563736</v>
+        <v>-31.34886508248006</v>
       </c>
       <c r="G102" t="n">
-        <v>-36.863916323551</v>
+        <v>-36.87130483064087</v>
       </c>
       <c r="H102" t="n">
-        <v>339.0906527200441</v>
+        <v>339.0392680884388</v>
       </c>
       <c r="I102" t="n">
-        <v>42.302713467815</v>
+        <v>42.30071721794506</v>
       </c>
       <c r="J102" t="n">
         <v>29.49738868005443</v>
       </c>
       <c r="K102" t="n">
-        <v>0.1621458091610761</v>
+        <v>0.1621020282624433</v>
       </c>
       <c r="L102" t="n">
-        <v>127.6891410765633</v>
+        <v>127.6881884921604</v>
       </c>
       <c r="M102" t="n">
-        <v>120.8995017381257</v>
+        <v>120.898975309903</v>
       </c>
       <c r="N102" t="n">
-        <v>95.96541847646438</v>
+        <v>95.96514444533477</v>
       </c>
       <c r="O102" t="n">
-        <v>-14.27559203839011</v>
+        <v>-14.27623035135753</v>
       </c>
       <c r="P102" t="n">
-        <v>9.092974971339855</v>
+        <v>9.08755429053708</v>
       </c>
       <c r="Q102" t="n">
-        <v>-90.90702502866014</v>
+        <v>-90.91244570946292</v>
       </c>
       <c r="R102" t="n">
-        <v>-88.16250759283028</v>
+        <v>-88.16644636380137</v>
       </c>
       <c r="S102" t="n">
-        <v>-64.04952667948332</v>
+        <v>-64.05373378755125</v>
       </c>
       <c r="T102" t="inlineStr">
         <is>
@@ -31709,52 +31709,52 @@
         </is>
       </c>
       <c r="D104" t="n">
-        <v>0.2449000030755997</v>
+        <v>0.2445999979972839</v>
       </c>
       <c r="E104" t="n">
-        <v>-0.5199426664229345</v>
+        <v>-0.6418067824556339</v>
       </c>
       <c r="F104" t="n">
-        <v>-26.41889422221968</v>
+        <v>-26.5090318503299</v>
       </c>
       <c r="G104" t="n">
-        <v>-29.08684261168147</v>
+        <v>-29.1737119749674</v>
       </c>
       <c r="H104" t="n">
-        <v>-79.47646107464027</v>
+        <v>-79.50160262558063</v>
       </c>
       <c r="I104" t="n">
-        <v>39.46836317351504</v>
+        <v>39.45885746681632</v>
       </c>
       <c r="J104" t="n">
         <v>29.35481237847949</v>
       </c>
       <c r="K104" t="n">
-        <v>0.18192593769646</v>
+        <v>0.1816746665159332</v>
       </c>
       <c r="L104" t="n">
-        <v>0.4638923498235749</v>
+        <v>0.4638637779113544</v>
       </c>
       <c r="M104" t="n">
-        <v>0.5191923782946398</v>
+        <v>0.5191803780915072</v>
       </c>
       <c r="N104" t="n">
-        <v>0.4832887574659289</v>
+        <v>0.4832826349133102</v>
       </c>
       <c r="O104" t="n">
-        <v>-0.05145215950060671</v>
+        <v>-0.05147130512383827</v>
       </c>
       <c r="P104" t="n">
-        <v>2.361603607116411</v>
+        <v>2.323639141351004</v>
       </c>
       <c r="Q104" t="n">
-        <v>-97.63839639288359</v>
+        <v>-97.67636085864899</v>
       </c>
       <c r="R104" t="n">
-        <v>-93.13043518745593</v>
+        <v>-93.15469516509968</v>
       </c>
       <c r="S104" t="n">
-        <v>-34.38081131461959</v>
+        <v>-34.46119551059077</v>
       </c>
       <c r="T104" t="inlineStr">
         <is>
@@ -31989,52 +31989,52 @@
         </is>
       </c>
       <c r="D107" t="n">
-        <v>9.522000312805176</v>
+        <v>9.510000228881836</v>
       </c>
       <c r="E107" t="n">
-        <v>4.58721660248862</v>
+        <v>4.455410749169042</v>
       </c>
       <c r="F107" t="n">
-        <v>-21.87402509207121</v>
+        <v>-21.97248321270655</v>
       </c>
       <c r="G107" t="n">
-        <v>-13.62931509958734</v>
+        <v>-13.73816360129632</v>
       </c>
       <c r="H107" t="n">
-        <v>-67.55832572860332</v>
+        <v>-67.59921029078369</v>
       </c>
       <c r="I107" t="n">
-        <v>43.33029148375309</v>
+        <v>43.30817055137159</v>
       </c>
       <c r="J107" t="n">
         <v>20.59975096251946</v>
       </c>
       <c r="K107" t="n">
-        <v>0.2318996396189867</v>
+        <v>0.231356072336629</v>
       </c>
       <c r="L107" t="n">
-        <v>13.07984807937861</v>
+        <v>13.07870521424305</v>
       </c>
       <c r="M107" t="n">
-        <v>13.0534943421771</v>
+        <v>13.05301433882017</v>
       </c>
       <c r="N107" t="n">
-        <v>11.01278071666322</v>
+        <v>11.01253581699132</v>
       </c>
       <c r="O107" t="n">
-        <v>-1.047401408744292</v>
+        <v>-1.048167226065896</v>
       </c>
       <c r="P107" t="n">
-        <v>10.78762425593816</v>
+        <v>10.72884531543803</v>
       </c>
       <c r="Q107" t="n">
-        <v>-89.21237574406183</v>
+        <v>-89.27115468456198</v>
       </c>
       <c r="R107" t="n">
-        <v>-87.61985275922098</v>
+        <v>-87.67916729697477</v>
       </c>
       <c r="S107" t="n">
-        <v>-19.64944947886832</v>
+        <v>-19.75071111695538</v>
       </c>
       <c r="T107" t="inlineStr">
         <is>
@@ -32048,7 +32048,7 @@
       </c>
       <c r="V107" t="inlineStr"/>
       <c r="W107" t="n">
-        <v>34</v>
+        <v>33.9</v>
       </c>
       <c r="X107" t="n">
         <v>72.40000000000001</v>
@@ -32725,52 +32725,52 @@
         </is>
       </c>
       <c r="D115" t="n">
-        <v>1.269999980926514</v>
+        <v>1.274999976158142</v>
       </c>
       <c r="E115" t="n">
-        <v>5.532298819103709</v>
+        <v>5.947779920523377</v>
       </c>
       <c r="F115" t="n">
-        <v>-29.01851696018273</v>
+        <v>-28.7390625648574</v>
       </c>
       <c r="G115" t="n">
-        <v>-70.17718007839933</v>
+        <v>-70.05976751175274</v>
       </c>
       <c r="H115" t="n">
-        <v>-96.57007164029457</v>
+        <v>-96.55656799801039</v>
       </c>
       <c r="I115" t="n">
-        <v>35.61591898777293</v>
+        <v>35.64629111726357</v>
       </c>
       <c r="J115" t="n">
         <v>27.37097468108967</v>
       </c>
       <c r="K115" t="n">
-        <v>0.2164274905644594</v>
+        <v>0.2169723299704548</v>
       </c>
       <c r="L115" t="n">
-        <v>3.217244074585384</v>
+        <v>3.217720264607444</v>
       </c>
       <c r="M115" t="n">
-        <v>4.711733946345683</v>
+        <v>4.712011723858551</v>
       </c>
       <c r="N115" t="n">
-        <v>6.653257679810903</v>
+        <v>6.653402607208921</v>
       </c>
       <c r="O115" t="n">
-        <v>-0.07990825982799898</v>
+        <v>-0.07958917181321712</v>
       </c>
       <c r="P115" t="n">
-        <v>3.297511455477438</v>
+        <v>3.415550293499998</v>
       </c>
       <c r="Q115" t="n">
-        <v>-96.70248854452257</v>
+        <v>-96.5844497065</v>
       </c>
       <c r="R115" t="n">
-        <v>-77.97623812689596</v>
+        <v>-77.9281665786247</v>
       </c>
       <c r="S115" t="n">
-        <v>-80.85888486805202</v>
+        <v>-80.78352621779601</v>
       </c>
       <c r="T115" t="inlineStr">
         <is>
@@ -33238,7 +33238,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>25/05/2026 19:41:12</t>
+          <t>25/05/2026 21:07:48</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -33451,10 +33451,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>76.77885939877726</v>
+        <v>76.77884174568915</v>
       </c>
       <c r="C2" t="n">
-        <v>0.173569170076488</v>
+        <v>0.1735684639529637</v>
       </c>
       <c r="D2" t="n">
         <v>68.10344827586206</v>
@@ -33603,7 +33603,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.962</v>
+        <v>0.961</v>
       </c>
       <c r="D6" t="n">
         <v>0.954</v>
@@ -33657,43 +33657,43 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ADA</t>
+          <t>RUSSELL</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>AVAX</t>
+          <t>MSCIWORLD</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.907</v>
+        <v>0.9330000000000001</v>
       </c>
       <c r="D9" t="n">
         <v>0.9340000000000001</v>
       </c>
       <c r="E9" t="n">
-        <v>0.9350000000000001</v>
+        <v>0.925</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>RUSSELL</t>
+          <t>ADA</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>MSCIWORLD</t>
+          <t>AVAX</t>
         </is>
       </c>
       <c r="C10" t="n">
+        <v>0.906</v>
+      </c>
+      <c r="D10" t="n">
         <v>0.9330000000000001</v>
       </c>
-      <c r="D10" t="n">
-        <v>0.9340000000000001</v>
-      </c>
       <c r="E10" t="n">
-        <v>0.925</v>
+        <v>0.9350000000000001</v>
       </c>
     </row>
     <row r="11">
@@ -33792,7 +33792,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.893</v>
+        <v>0.894</v>
       </c>
       <c r="D15" t="n">
         <v>0.923</v>

</xml_diff>

<commit_message>
📊 Dashboard aggiornata 03/07/2026 21:08
</commit_message>
<xml_diff>
--- a/docs/sarada_dati.xlsx
+++ b/docs/sarada_dati.xlsx
@@ -1089,7 +1089,7 @@
         <v>75.3</v>
       </c>
       <c r="X7" t="n">
-        <v>68.59999999999999</v>
+        <v>68.5</v>
       </c>
       <c r="Y7" t="inlineStr">
         <is>
@@ -3593,66 +3593,66 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>MSCIWORLD</t>
+          <t>USDJPY</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>MSCI World ETF</t>
+          <t>USD/JPY</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Indici</t>
+          <t>FX/Macro</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>156.1699981689453</v>
+        <v>161.3370056152344</v>
       </c>
       <c r="E35" t="n">
-        <v>0.03202860192268453</v>
+        <v>-0.7395122639961338</v>
       </c>
       <c r="F35" t="n">
-        <v>0.8524326854383757</v>
+        <v>-0.2892290607401815</v>
       </c>
       <c r="G35" t="n">
-        <v>-1.995612056961293</v>
+        <v>0.8734545157581319</v>
       </c>
       <c r="H35" t="n">
-        <v>12.05424671044277</v>
+        <v>1.651378651693602</v>
       </c>
       <c r="I35" t="n">
-        <v>52.16795734087916</v>
+        <v>55.98624080733547</v>
       </c>
       <c r="J35" t="n">
-        <v>23.66507112143193</v>
+        <v>51.34634873082719</v>
       </c>
       <c r="K35" t="n">
-        <v>0.5538400296627888</v>
+        <v>0.5648774089171957</v>
       </c>
       <c r="L35" t="n">
-        <v>155.8037604548409</v>
+        <v>161.187718709663</v>
       </c>
       <c r="M35" t="n">
-        <v>153.8972543060498</v>
+        <v>160.1064602219826</v>
       </c>
       <c r="N35" t="n">
-        <v>144.9799985099418</v>
+        <v>156.7091873106595</v>
       </c>
       <c r="O35" t="n">
-        <v>-0.153957316628815</v>
+        <v>0.01652384429840703</v>
       </c>
       <c r="P35" t="n">
-        <v>48.98994050616003</v>
+        <v>46.04056926600718</v>
       </c>
       <c r="Q35" t="n">
-        <v>-51.01005949383998</v>
+        <v>-53.95943073399282</v>
       </c>
       <c r="R35" t="n">
-        <v>20.27515186218173</v>
+        <v>0.9822531698327827</v>
       </c>
       <c r="S35" t="n">
-        <v>-1.126938153648815</v>
+        <v>0.8419276678679033</v>
       </c>
       <c r="T35" t="inlineStr">
         <is>
@@ -3661,19 +3661,19 @@
       </c>
       <c r="U35" t="inlineStr">
         <is>
-          <t>Evening Star</t>
+          <t>Hammer</t>
         </is>
       </c>
       <c r="V35" t="inlineStr">
         <is>
-          <t>Double Top, Double Bottom, Outside Bar, Volatility Squeeze</t>
+          <t>Double Top, Double Bottom, Bull Flag / Consolidation, Volatility Squeeze</t>
         </is>
       </c>
       <c r="W35" t="n">
-        <v>66.40000000000001</v>
+        <v>66.5</v>
       </c>
       <c r="X35" t="n">
-        <v>70</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="Y35" t="inlineStr">
         <is>
@@ -3682,84 +3682,94 @@
       </c>
       <c r="Z35" t="inlineStr">
         <is>
-          <t>EMA e SMA allineate al rialzo — struttura bullish solida; trend in sviluppo (ADX 24); pattern: Double Bottom; evening star — inversione ribassista a 3 candele</t>
+          <t>EMA e SMA allineate al rialzo — struttura bullish solida; trend molto direzionale (ADX 51); pattern: Double Bottom; hammer — segnale di rimbalzo da supporto; sul supporto dei 20g (159.89); vicino alla resistenza dei 20g (162.84); in zona Fib Fib 23.6 — livello strutturale</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>USDJPY</t>
+          <t>MSCIWORLD</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>USD/JPY</t>
+          <t>MSCI World ETF</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>FX/Macro</t>
+          <t>Indici</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>162.5390014648438</v>
+        <v>156.1699981689453</v>
       </c>
       <c r="E36" t="n">
-        <v>-0.05472889866934283</v>
+        <v>0.03202860192268453</v>
       </c>
       <c r="F36" t="n">
-        <v>0.4797147519643774</v>
+        <v>0.8524326854383757</v>
       </c>
       <c r="G36" t="n">
-        <v>1.607195881821077</v>
+        <v>-1.995612056961293</v>
       </c>
       <c r="H36" t="n">
-        <v>1.788545325196367</v>
+        <v>12.05424671044277</v>
       </c>
       <c r="I36" t="n">
-        <v>78.30385849751123</v>
+        <v>52.16795734087916</v>
       </c>
       <c r="J36" t="n">
-        <v>51.34634873082719</v>
+        <v>23.66507112143193</v>
       </c>
       <c r="K36" t="n">
-        <v>0.9278053096179374</v>
+        <v>0.5538400296627888</v>
       </c>
       <c r="L36" t="n">
-        <v>161.1720042985502</v>
+        <v>155.8037604548409</v>
       </c>
       <c r="M36" t="n">
-        <v>160.0562338794009</v>
+        <v>153.8972543060498</v>
       </c>
       <c r="N36" t="n">
-        <v>156.6626765739301</v>
+        <v>144.9799985099418</v>
       </c>
       <c r="O36" t="n">
-        <v>0.1048596616097186</v>
-      </c>
-      <c r="P36" t="inlineStr"/>
-      <c r="Q36" t="inlineStr"/>
-      <c r="R36" t="inlineStr"/>
+        <v>-0.153957316628815</v>
+      </c>
+      <c r="P36" t="n">
+        <v>48.98994050616003</v>
+      </c>
+      <c r="Q36" t="n">
+        <v>-51.01005949383998</v>
+      </c>
+      <c r="R36" t="n">
+        <v>20.27515186218173</v>
+      </c>
       <c r="S36" t="n">
-        <v>1.624983733753305</v>
+        <v>-1.126938153648815</v>
       </c>
       <c r="T36" t="inlineStr">
         <is>
           <t>Trend Bullish</t>
         </is>
       </c>
-      <c r="U36" t="inlineStr"/>
+      <c r="U36" t="inlineStr">
+        <is>
+          <t>Evening Star</t>
+        </is>
+      </c>
       <c r="V36" t="inlineStr">
         <is>
-          <t>Double Top, Double Bottom</t>
+          <t>Double Top, Double Bottom, Outside Bar, Volatility Squeeze</t>
         </is>
       </c>
       <c r="W36" t="n">
-        <v>66.3</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="X36" t="n">
-        <v>64.3</v>
+        <v>70</v>
       </c>
       <c r="Y36" t="inlineStr">
         <is>
@@ -3768,7 +3778,7 @@
       </c>
       <c r="Z36" t="inlineStr">
         <is>
-          <t>EMA e SMA allineate al rialzo — struttura bullish solida; trend molto direzionale (ADX 51); RSI ipercomprato (78) — attenzione estensione; pattern: Double Bottom; vicino alla resistenza dei 20g (162.84); in zona Fib Fib 23.6 — livello strutturale</t>
+          <t>EMA e SMA allineate al rialzo — struttura bullish solida; trend in sviluppo (ADX 24); pattern: Double Bottom; evening star — inversione ribassista a 3 candele</t>
         </is>
       </c>
     </row>
@@ -4799,52 +4809,52 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>82.19000244140625</v>
+        <v>82.76000213623047</v>
       </c>
       <c r="E48" t="n">
-        <v>1.917093465307262</v>
+        <v>2.623903423294682</v>
       </c>
       <c r="F48" t="n">
-        <v>15.25257485452753</v>
+        <v>16.05186832749732</v>
       </c>
       <c r="G48" t="n">
-        <v>23.13242681045211</v>
+        <v>23.98636820989373</v>
       </c>
       <c r="H48" t="n">
-        <v>-2.475905062906114</v>
+        <v>-1.799561192594379</v>
       </c>
       <c r="I48" t="n">
-        <v>65.61314610942259</v>
+        <v>66.28160320729185</v>
       </c>
       <c r="J48" t="n">
-        <v>19.1381050228664</v>
+        <v>19.18628673119542</v>
       </c>
       <c r="K48" t="n">
-        <v>1.125693225559595</v>
+        <v>1.148414066395675</v>
       </c>
       <c r="L48" t="n">
-        <v>73.8573379788607</v>
+        <v>73.91162366408204</v>
       </c>
       <c r="M48" t="n">
-        <v>75.70067373861689</v>
+        <v>75.72302666782568</v>
       </c>
       <c r="N48" t="n">
-        <v>96.8473341421401</v>
+        <v>96.85300578089458</v>
       </c>
       <c r="O48" t="n">
-        <v>1.639001831675933</v>
+        <v>1.6753778805764</v>
       </c>
       <c r="P48" t="n">
-        <v>97.75221817537843</v>
+        <v>99.086038124678</v>
       </c>
       <c r="Q48" t="n">
-        <v>-2.247781824621568</v>
+        <v>-0.913961875321999</v>
       </c>
       <c r="R48" t="n">
-        <v>214.4834328801499</v>
+        <v>222.2465830321673</v>
       </c>
       <c r="S48" t="n">
-        <v>19.33596047719284</v>
+        <v>20.16357282702879</v>
       </c>
       <c r="T48" t="inlineStr">
         <is>
@@ -4854,14 +4864,14 @@
       <c r="U48" t="inlineStr"/>
       <c r="V48" t="inlineStr">
         <is>
-          <t>Inside Bar</t>
+          <t>Breakout 20d</t>
         </is>
       </c>
       <c r="W48" t="n">
-        <v>58.6</v>
+        <v>59.3</v>
       </c>
       <c r="X48" t="n">
-        <v>63.5</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="Y48" t="inlineStr">
         <is>
@@ -4870,7 +4880,7 @@
       </c>
       <c r="Z48" t="inlineStr">
         <is>
-          <t>RSI in forza (66) — momentum positivo; vicino alla resistenza dei 20g (82.60)</t>
+          <t>RSI in forza (66) — momentum positivo; breakout massimi 20g — momentum di breve; vicino alla resistenza dei 20g (82.93); in zona Fib Fib 38.2 — livello strutturale</t>
         </is>
       </c>
     </row>
@@ -7107,66 +7117,70 @@
         </is>
       </c>
       <c r="D73" t="n">
-        <v>1.33552360534668</v>
+        <v>1.334988713264465</v>
       </c>
       <c r="E73" t="n">
-        <v>0.5716050346918244</v>
+        <v>0.5313249864670855</v>
       </c>
       <c r="F73" t="n">
-        <v>1.268753801018629</v>
+        <v>1.228194536946448</v>
       </c>
       <c r="G73" t="n">
-        <v>-0.5355437761158766</v>
+        <v>-0.5753803989077988</v>
       </c>
       <c r="H73" t="n">
-        <v>-0.3472356574381497</v>
+        <v>-0.3871476997294399</v>
       </c>
       <c r="I73" t="n">
-        <v>53.44604511167641</v>
+        <v>52.9812659969456</v>
       </c>
       <c r="J73" t="n">
         <v>34.79252082454199</v>
       </c>
       <c r="K73" t="n">
-        <v>0.6581396890618093</v>
+        <v>0.6443909969799766</v>
       </c>
       <c r="L73" t="n">
-        <v>1.329965885929094</v>
+        <v>1.329914943826026</v>
       </c>
       <c r="M73" t="n">
-        <v>1.336473015716562</v>
+        <v>1.336452039556475</v>
       </c>
       <c r="N73" t="n">
-        <v>1.338412322962132</v>
+        <v>1.338407000652856</v>
       </c>
       <c r="O73" t="n">
-        <v>0.001050636427556501</v>
+        <v>0.001016500864475073</v>
       </c>
       <c r="P73" t="n">
-        <v>71.16507027839519</v>
+        <v>69.37133217135457</v>
       </c>
       <c r="Q73" t="n">
-        <v>-28.83492972160481</v>
+        <v>-30.62866782864544</v>
       </c>
       <c r="R73" t="n">
-        <v>42.3195952542145</v>
+        <v>41.08927004577082</v>
       </c>
       <c r="S73" t="n">
-        <v>-0.5344752518426032</v>
+        <v>-0.5743123025904073</v>
       </c>
       <c r="T73" t="inlineStr">
         <is>
           <t>Bearish</t>
         </is>
       </c>
-      <c r="U73" t="inlineStr"/>
+      <c r="U73" t="inlineStr">
+        <is>
+          <t>Doji</t>
+        </is>
+      </c>
       <c r="V73" t="inlineStr">
         <is>
           <t>Double Top, Double Bottom, Inside Bar</t>
         </is>
       </c>
       <c r="W73" t="n">
-        <v>46.2</v>
+        <v>46.1</v>
       </c>
       <c r="X73" t="n">
         <v>56.4</v>
@@ -7178,7 +7192,7 @@
       </c>
       <c r="Z73" t="inlineStr">
         <is>
-          <t>trend molto direzionale (ADX 35); pattern: Double Bottom; vicino alla resistenza dei 20g (1.3461); in zona Fib Fib 61.8 — livello strutturale</t>
+          <t>trend molto direzionale (ADX 35); pattern: Double Bottom; doji — indecisione del mercato; vicino alla resistenza dei 20g (1.3461); in zona Fib Fib 61.8 — livello strutturale</t>
         </is>
       </c>
     </row>
@@ -7369,79 +7383,83 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>AVAX</t>
+          <t>COTTON</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Avalanche</t>
+          <t>Cotton</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Crypto</t>
+          <t>Commodities</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>6.909999847412109</v>
+        <v>72.56999969482422</v>
       </c>
       <c r="E76" t="n">
-        <v>1.723555302599666</v>
+        <v>-0.9688852296668493</v>
       </c>
       <c r="F76" t="n">
-        <v>7.2521374647327</v>
+        <v>-1.130792661853075</v>
       </c>
       <c r="G76" t="n">
-        <v>5.257477085340923</v>
+        <v>-5.802182200911943</v>
       </c>
       <c r="H76" t="n">
-        <v>-24.73356863766768</v>
+        <v>2.326567355442233</v>
       </c>
       <c r="I76" t="n">
-        <v>51.67755511342694</v>
+        <v>43.1498933780203</v>
       </c>
       <c r="J76" t="n">
-        <v>36.97876607456516</v>
+        <v>14.64486009625032</v>
       </c>
       <c r="K76" t="n">
-        <v>0.859439642414791</v>
+        <v>0.3719258006802371</v>
       </c>
       <c r="L76" t="n">
-        <v>6.687766796962074</v>
+        <v>73.9394938126256</v>
       </c>
       <c r="M76" t="n">
-        <v>7.365478550225608</v>
+        <v>74.79148975701614</v>
       </c>
       <c r="N76" t="n">
-        <v>10.42381850983205</v>
+        <v>70.44261985394238</v>
       </c>
       <c r="O76" t="n">
-        <v>0.1425425837437522</v>
+        <v>0.01847026383485018</v>
       </c>
       <c r="P76" t="n">
-        <v>100.3564351617813</v>
+        <v>26.16434562224022</v>
       </c>
       <c r="Q76" t="n">
-        <v>0.3564351617812837</v>
+        <v>-73.83565437775978</v>
       </c>
       <c r="R76" t="n">
-        <v>58.57887739433393</v>
+        <v>-20.67858884527496</v>
       </c>
       <c r="S76" t="n">
-        <v>2.896898036971352</v>
+        <v>-5.42161277220049</v>
       </c>
       <c r="T76" t="inlineStr">
         <is>
-          <t>Bearish</t>
-        </is>
-      </c>
-      <c r="U76" t="inlineStr"/>
+          <t>Range</t>
+        </is>
+      </c>
+      <c r="U76" t="inlineStr">
+        <is>
+          <t>Doji</t>
+        </is>
+      </c>
       <c r="V76" t="inlineStr"/>
       <c r="W76" t="n">
-        <v>45.5</v>
+        <v>45.4</v>
       </c>
       <c r="X76" t="n">
-        <v>56.1</v>
+        <v>61.9</v>
       </c>
       <c r="Y76" t="inlineStr">
         <is>
@@ -7450,77 +7468,77 @@
       </c>
       <c r="Z76" t="inlineStr">
         <is>
-          <t>trend molto direzionale (ADX 37); in zona Fib Fib 78.6 — livello strutturale</t>
+          <t>mercato laterale — ATR basso (ADX 15); doji — indecisione del mercato; in zona Fib Fib 61.8 — livello strutturale</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>COTTON</t>
+          <t>CPR</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Cotton</t>
+          <t>Campari</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Commodities</t>
+          <t>Azioni IT</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>72.56999969482422</v>
+        <v>5.513999938964844</v>
       </c>
       <c r="E77" t="n">
-        <v>-0.9688852296668493</v>
+        <v>2.988416971911323</v>
       </c>
       <c r="F77" t="n">
-        <v>-1.130792661853075</v>
+        <v>-0.1810323783124401</v>
       </c>
       <c r="G77" t="n">
-        <v>-5.802182200911943</v>
+        <v>2.528824133529306</v>
       </c>
       <c r="H77" t="n">
-        <v>2.326567355442233</v>
+        <v>-11.71949881557952</v>
       </c>
       <c r="I77" t="n">
-        <v>43.1498933780203</v>
+        <v>49.93210808971318</v>
       </c>
       <c r="J77" t="n">
-        <v>14.64486009625032</v>
+        <v>9.660583359844347</v>
       </c>
       <c r="K77" t="n">
-        <v>0.3719258006802371</v>
+        <v>0.7267940500573961</v>
       </c>
       <c r="L77" t="n">
-        <v>73.9394938126256</v>
+        <v>5.483130379921562</v>
       </c>
       <c r="M77" t="n">
-        <v>74.79148975701614</v>
+        <v>5.638946845876156</v>
       </c>
       <c r="N77" t="n">
-        <v>70.44261985394238</v>
+        <v>5.914717133435826</v>
       </c>
       <c r="O77" t="n">
-        <v>0.01847026383485018</v>
+        <v>0.01521546702563684</v>
       </c>
       <c r="P77" t="n">
-        <v>26.16434562224022</v>
+        <v>54.63914611740272</v>
       </c>
       <c r="Q77" t="n">
-        <v>-73.83565437775978</v>
+        <v>-45.36085388259729</v>
       </c>
       <c r="R77" t="n">
-        <v>-20.67858884527496</v>
+        <v>48.25729487085574</v>
       </c>
       <c r="S77" t="n">
-        <v>-5.42161277220049</v>
+        <v>1.771866256775656</v>
       </c>
       <c r="T77" t="inlineStr">
         <is>
-          <t>Range</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="U77" t="inlineStr">
@@ -7528,12 +7546,16 @@
           <t>Doji</t>
         </is>
       </c>
-      <c r="V77" t="inlineStr"/>
+      <c r="V77" t="inlineStr">
+        <is>
+          <t>Double Top, Double Bottom</t>
+        </is>
+      </c>
       <c r="W77" t="n">
-        <v>45.4</v>
+        <v>45.2</v>
       </c>
       <c r="X77" t="n">
-        <v>61.9</v>
+        <v>57</v>
       </c>
       <c r="Y77" t="inlineStr">
         <is>
@@ -7542,94 +7564,86 @@
       </c>
       <c r="Z77" t="inlineStr">
         <is>
-          <t>mercato laterale — ATR basso (ADX 15); doji — indecisione del mercato; in zona Fib Fib 61.8 — livello strutturale</t>
+          <t>mercato laterale — ATR basso (ADX 10); pattern: Double Bottom; doji — indecisione del mercato</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>CPR</t>
+          <t>AVAX</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Campari</t>
+          <t>Avalanche</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Azioni IT</t>
+          <t>Crypto</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>5.513999938964844</v>
+        <v>6.980000019073486</v>
       </c>
       <c r="E78" t="n">
-        <v>2.988416971911323</v>
+        <v>2.754042493689002</v>
       </c>
       <c r="F78" t="n">
-        <v>-0.1810323783124401</v>
+        <v>8.338630691847971</v>
       </c>
       <c r="G78" t="n">
-        <v>2.528824133529306</v>
+        <v>6.323763862087639</v>
       </c>
       <c r="H78" t="n">
-        <v>-11.71949881557952</v>
+        <v>-23.97109928426014</v>
       </c>
       <c r="I78" t="n">
-        <v>49.93210808971318</v>
+        <v>53.02111416353829</v>
       </c>
       <c r="J78" t="n">
-        <v>9.660583359844347</v>
+        <v>37.14692377733794</v>
       </c>
       <c r="K78" t="n">
-        <v>0.7267940500573961</v>
+        <v>0.9106523592144119</v>
       </c>
       <c r="L78" t="n">
-        <v>5.483130379921562</v>
+        <v>6.694433479977443</v>
       </c>
       <c r="M78" t="n">
-        <v>5.638946845876156</v>
+        <v>7.368223654996642</v>
       </c>
       <c r="N78" t="n">
-        <v>5.914717133435826</v>
+        <v>10.42451502895305</v>
       </c>
       <c r="O78" t="n">
-        <v>0.01521546702563684</v>
+        <v>0.1470098311660166</v>
       </c>
       <c r="P78" t="n">
-        <v>54.63914611740272</v>
+        <v>99.68823676370866</v>
       </c>
       <c r="Q78" t="n">
-        <v>-45.36085388259729</v>
+        <v>-0.3117632362913401</v>
       </c>
       <c r="R78" t="n">
-        <v>48.25729487085574</v>
+        <v>65.45808773311462</v>
       </c>
       <c r="S78" t="n">
-        <v>1.771866256775656</v>
+        <v>3.939271508037145</v>
       </c>
       <c r="T78" t="inlineStr">
         <is>
           <t>Bearish</t>
         </is>
       </c>
-      <c r="U78" t="inlineStr">
-        <is>
-          <t>Doji</t>
-        </is>
-      </c>
-      <c r="V78" t="inlineStr">
-        <is>
-          <t>Double Top, Double Bottom</t>
-        </is>
-      </c>
+      <c r="U78" t="inlineStr"/>
+      <c r="V78" t="inlineStr"/>
       <c r="W78" t="n">
-        <v>45.2</v>
+        <v>44.9</v>
       </c>
       <c r="X78" t="n">
-        <v>57</v>
+        <v>56.5</v>
       </c>
       <c r="Y78" t="inlineStr">
         <is>
@@ -7638,7 +7652,7 @@
       </c>
       <c r="Z78" t="inlineStr">
         <is>
-          <t>mercato laterale — ATR basso (ADX 10); pattern: Double Bottom; doji — indecisione del mercato</t>
+          <t>trend molto direzionale (ADX 37); vicino alla resistenza dei 20g (7.0609)</t>
         </is>
       </c>
     </row>
@@ -8109,66 +8123,66 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>ETH</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Microsoft</t>
+          <t>Ethereum</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Azioni USA</t>
+          <t>Crypto</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>390.489990234375</v>
+        <v>1764.400024414062</v>
       </c>
       <c r="E84" t="n">
-        <v>1.616006941502235</v>
+        <v>3.900116767509587</v>
       </c>
       <c r="F84" t="n">
-        <v>10.67369699156677</v>
+        <v>12.35631761732514</v>
       </c>
       <c r="G84" t="n">
-        <v>-11.51571630041562</v>
+        <v>5.961837664517433</v>
       </c>
       <c r="H84" t="n">
-        <v>4.560059757122703</v>
+        <v>-23.82455319677302</v>
       </c>
       <c r="I84" t="n">
-        <v>49.80110187594683</v>
+        <v>55.81156908631785</v>
       </c>
       <c r="J84" t="n">
-        <v>45.34042955827164</v>
+        <v>20.70025469109621</v>
       </c>
       <c r="K84" t="n">
-        <v>0.5465301148068399</v>
+        <v>0.7856915835980655</v>
       </c>
       <c r="L84" t="n">
-        <v>386.6018465676733</v>
+        <v>1674.44437466409</v>
       </c>
       <c r="M84" t="n">
-        <v>398.6495915414451</v>
+        <v>1808.036562341718</v>
       </c>
       <c r="N84" t="n">
-        <v>427.8201890951816</v>
+        <v>2270.12606745985</v>
       </c>
       <c r="O84" t="n">
-        <v>1.082789350491073</v>
+        <v>22.29034938941281</v>
       </c>
       <c r="P84" t="n">
-        <v>78.57276426022005</v>
+        <v>95.33199342727954</v>
       </c>
       <c r="Q84" t="n">
-        <v>-21.42723573977995</v>
+        <v>-4.66800657272046</v>
       </c>
       <c r="R84" t="n">
-        <v>3.539648516898157</v>
+        <v>86.73405657287813</v>
       </c>
       <c r="S84" t="n">
-        <v>-8.623111906047509</v>
+        <v>5.010397173328895</v>
       </c>
       <c r="T84" t="inlineStr">
         <is>
@@ -8176,12 +8190,16 @@
         </is>
       </c>
       <c r="U84" t="inlineStr"/>
-      <c r="V84" t="inlineStr"/>
+      <c r="V84" t="inlineStr">
+        <is>
+          <t>Double Bottom</t>
+        </is>
+      </c>
       <c r="W84" t="n">
-        <v>43.5</v>
+        <v>44</v>
       </c>
       <c r="X84" t="n">
-        <v>59.2</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="Y84" t="inlineStr">
         <is>
@@ -8190,73 +8208,73 @@
       </c>
       <c r="Z84" t="inlineStr">
         <is>
-          <t>trend molto direzionale (ADX 45); in zona Fib Fib 61.8 — livello strutturale</t>
+          <t>trend in sviluppo (ADX 21); pattern: Double Bottom; in zona Fib Fib 78.6 — livello strutturale</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>ETH</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Ethereum</t>
+          <t>Microsoft</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Crypto</t>
+          <t>Azioni USA</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>1744.18994140625</v>
+        <v>390.489990234375</v>
       </c>
       <c r="E85" t="n">
-        <v>2.710006840431056</v>
+        <v>1.616006941502235</v>
       </c>
       <c r="F85" t="n">
-        <v>11.06934727382134</v>
+        <v>10.67369699156677</v>
       </c>
       <c r="G85" t="n">
-        <v>4.748112032445184</v>
+        <v>-11.51571630041562</v>
       </c>
       <c r="H85" t="n">
-        <v>-24.69709461694314</v>
+        <v>4.560059757122703</v>
       </c>
       <c r="I85" t="n">
-        <v>54.15421101017839</v>
+        <v>49.80110187594683</v>
       </c>
       <c r="J85" t="n">
-        <v>20.44441239659244</v>
+        <v>45.34042955827164</v>
       </c>
       <c r="K85" t="n">
-        <v>0.7285309396920854</v>
+        <v>0.5465301148068399</v>
       </c>
       <c r="L85" t="n">
-        <v>1672.519604853822</v>
+        <v>386.6018465676733</v>
       </c>
       <c r="M85" t="n">
-        <v>1807.244010066902</v>
+        <v>398.6495915414451</v>
       </c>
       <c r="N85" t="n">
-        <v>2269.924972106538</v>
+        <v>427.8201890951816</v>
       </c>
       <c r="O85" t="n">
-        <v>21.00058910629328</v>
+        <v>1.082789350491073</v>
       </c>
       <c r="P85" t="n">
-        <v>87.74352639744791</v>
+        <v>78.57276426022005</v>
       </c>
       <c r="Q85" t="n">
-        <v>-12.25647360255209</v>
+        <v>-21.42723573977995</v>
       </c>
       <c r="R85" t="n">
-        <v>71.83130038425395</v>
+        <v>3.539648516898157</v>
       </c>
       <c r="S85" t="n">
-        <v>3.807569688523627</v>
+        <v>-8.623111906047509</v>
       </c>
       <c r="T85" t="inlineStr">
         <is>
@@ -8264,16 +8282,12 @@
         </is>
       </c>
       <c r="U85" t="inlineStr"/>
-      <c r="V85" t="inlineStr">
-        <is>
-          <t>Double Bottom</t>
-        </is>
-      </c>
+      <c r="V85" t="inlineStr"/>
       <c r="W85" t="n">
-        <v>43.4</v>
+        <v>43.5</v>
       </c>
       <c r="X85" t="n">
-        <v>68.8</v>
+        <v>59.2</v>
       </c>
       <c r="Y85" t="inlineStr">
         <is>
@@ -8282,7 +8296,7 @@
       </c>
       <c r="Z85" t="inlineStr">
         <is>
-          <t>trend in sviluppo (ADX 20); pattern: Double Bottom; in zona Fib Fib 78.6 — livello strutturale</t>
+          <t>trend molto direzionale (ADX 45); in zona Fib Fib 61.8 — livello strutturale</t>
         </is>
       </c>
     </row>
@@ -8649,66 +8663,66 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>BC</t>
+          <t>BTC</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Brunello Cucinelli</t>
+          <t>Bitcoin</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Azioni IT</t>
+          <t>Crypto</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>82.33999633789062</v>
+        <v>62698.01171875</v>
       </c>
       <c r="E90" t="n">
-        <v>-1.223613561651382</v>
+        <v>1.972359120132694</v>
       </c>
       <c r="F90" t="n">
-        <v>1.478921564294811</v>
+        <v>5.317566692840736</v>
       </c>
       <c r="G90" t="n">
-        <v>1.579075768379634</v>
+        <v>-1.330099067077828</v>
       </c>
       <c r="H90" t="n">
-        <v>7.213532638012077</v>
+        <v>-20.28959604009802</v>
       </c>
       <c r="I90" t="n">
-        <v>45.8851808697758</v>
+        <v>48.39434138306207</v>
       </c>
       <c r="J90" t="n">
-        <v>31.51892426920546</v>
+        <v>27.69677535557079</v>
       </c>
       <c r="K90" t="n">
-        <v>0.2724760646027921</v>
+        <v>0.5444593542232661</v>
       </c>
       <c r="L90" t="n">
-        <v>83.44553913114018</v>
+        <v>62141.98333455706</v>
       </c>
       <c r="M90" t="n">
-        <v>83.20928345388599</v>
+        <v>66005.51660402081</v>
       </c>
       <c r="N90" t="n">
-        <v>86.61875784929082</v>
+        <v>75895.14235070042</v>
       </c>
       <c r="O90" t="n">
-        <v>-0.3183206989983882</v>
+        <v>396.3779778982425</v>
       </c>
       <c r="P90" t="n">
-        <v>22.79905760623027</v>
+        <v>63.49534731310589</v>
       </c>
       <c r="Q90" t="n">
-        <v>-77.20094239376974</v>
+        <v>-36.50465268689411</v>
       </c>
       <c r="R90" t="n">
-        <v>-57.19999918572849</v>
+        <v>-2.061225582050607</v>
       </c>
       <c r="S90" t="n">
-        <v>-0.9145633576240653</v>
+        <v>-2.675065315559633</v>
       </c>
       <c r="T90" t="inlineStr">
         <is>
@@ -8716,16 +8730,12 @@
         </is>
       </c>
       <c r="U90" t="inlineStr"/>
-      <c r="V90" t="inlineStr">
-        <is>
-          <t>Double Bottom, Inside Bar</t>
-        </is>
-      </c>
+      <c r="V90" t="inlineStr"/>
       <c r="W90" t="n">
-        <v>41.7</v>
+        <v>42</v>
       </c>
       <c r="X90" t="n">
-        <v>63.9</v>
+        <v>63.2</v>
       </c>
       <c r="Y90" t="inlineStr">
         <is>
@@ -8734,73 +8744,73 @@
       </c>
       <c r="Z90" t="inlineStr">
         <is>
-          <t>trend molto direzionale (ADX 32); pattern: Double Bottom; in zona Fib Fib 38.2 — livello strutturale</t>
+          <t>trend in sviluppo (ADX 28); in zona Fib Fib 78.6 — livello strutturale</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>ADA</t>
+          <t>BC</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Cardano</t>
+          <t>Brunello Cucinelli</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Crypto</t>
+          <t>Azioni IT</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>0.1821999996900558</v>
+        <v>82.33999633789062</v>
       </c>
       <c r="E91" t="n">
-        <v>12.96212464858801</v>
+        <v>-1.223613561651382</v>
       </c>
       <c r="F91" t="n">
-        <v>26.81929080679977</v>
+        <v>1.478921564294811</v>
       </c>
       <c r="G91" t="n">
-        <v>7.277441751977953</v>
+        <v>1.579075768379634</v>
       </c>
       <c r="H91" t="n">
-        <v>-27.14389290221047</v>
+        <v>7.213532638012077</v>
       </c>
       <c r="I91" t="n">
-        <v>59.73830029790061</v>
+        <v>45.8851808697758</v>
       </c>
       <c r="J91" t="n">
-        <v>38.18681898929582</v>
+        <v>31.51892426920546</v>
       </c>
       <c r="K91" t="n">
-        <v>0.9583160521575457</v>
+        <v>0.2724760646027921</v>
       </c>
       <c r="L91" t="n">
-        <v>0.1613835235165188</v>
+        <v>83.44553913114018</v>
       </c>
       <c r="M91" t="n">
-        <v>0.1859171884166575</v>
+        <v>83.20928345388599</v>
       </c>
       <c r="N91" t="n">
-        <v>0.2929863611985647</v>
+        <v>86.61875784929082</v>
       </c>
       <c r="O91" t="n">
-        <v>0.004898882676287518</v>
+        <v>-0.3183206989983882</v>
       </c>
       <c r="P91" t="n">
-        <v>99.95689581386112</v>
+        <v>22.79905760623027</v>
       </c>
       <c r="Q91" t="n">
-        <v>-0.04310418613887149</v>
+        <v>-77.20094239376974</v>
       </c>
       <c r="R91" t="n">
-        <v>75.73660974138078</v>
+        <v>-57.19999918572849</v>
       </c>
       <c r="S91" t="n">
-        <v>6.08380259786232</v>
+        <v>-0.9145633576240653</v>
       </c>
       <c r="T91" t="inlineStr">
         <is>
@@ -8808,12 +8818,16 @@
         </is>
       </c>
       <c r="U91" t="inlineStr"/>
-      <c r="V91" t="inlineStr"/>
+      <c r="V91" t="inlineStr">
+        <is>
+          <t>Double Bottom, Inside Bar</t>
+        </is>
+      </c>
       <c r="W91" t="n">
-        <v>41.3</v>
+        <v>41.7</v>
       </c>
       <c r="X91" t="n">
-        <v>63.7</v>
+        <v>63.9</v>
       </c>
       <c r="Y91" t="inlineStr">
         <is>
@@ -8822,90 +8836,86 @@
       </c>
       <c r="Z91" t="inlineStr">
         <is>
-          <t>trend molto direzionale (ADX 38)</t>
+          <t>trend molto direzionale (ADX 32); pattern: Double Bottom; in zona Fib Fib 38.2 — livello strutturale</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>ENI</t>
+          <t>LINK</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Eni</t>
+          <t>Chainlink</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Azioni IT</t>
+          <t>Crypto</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>20.44499969482422</v>
+        <v>8.003000259399414</v>
       </c>
       <c r="E92" t="n">
-        <v>1.817727950722015</v>
+        <v>3.377832972274364</v>
       </c>
       <c r="F92" t="n">
-        <v>-0.170897696261807</v>
+        <v>10.23463049134337</v>
       </c>
       <c r="G92" t="n">
-        <v>-12.8330856477199</v>
+        <v>1.875167454931481</v>
       </c>
       <c r="H92" t="n">
-        <v>-17.17642237330426</v>
+        <v>-12.7676662088706</v>
       </c>
       <c r="I92" t="n">
-        <v>35.36943537656649</v>
+        <v>54.10236676207693</v>
       </c>
       <c r="J92" t="n">
-        <v>49.89199583755958</v>
+        <v>23.42564059683689</v>
       </c>
       <c r="K92" t="n">
-        <v>0.2357528920674938</v>
+        <v>0.6960021632551494</v>
       </c>
       <c r="L92" t="n">
-        <v>21.44480031734003</v>
+        <v>7.69331488071971</v>
       </c>
       <c r="M92" t="n">
-        <v>22.09834073766282</v>
+        <v>8.192324367286872</v>
       </c>
       <c r="N92" t="n">
-        <v>19.75335525708702</v>
+        <v>10.1765501817318</v>
       </c>
       <c r="O92" t="n">
-        <v>-0.1333154045249789</v>
+        <v>0.07724331408102098</v>
       </c>
       <c r="P92" t="n">
-        <v>15.43339562124327</v>
+        <v>88.00588343791685</v>
       </c>
       <c r="Q92" t="n">
-        <v>-84.56660437875674</v>
+        <v>-11.99411656208315</v>
       </c>
       <c r="R92" t="n">
-        <v>-84.6928807933466</v>
+        <v>52.55236837141192</v>
       </c>
       <c r="S92" t="n">
-        <v>-12.68418152712353</v>
+        <v>0.3206601465092884</v>
       </c>
       <c r="T92" t="inlineStr">
         <is>
-          <t>Range</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="U92" t="inlineStr"/>
-      <c r="V92" t="inlineStr">
-        <is>
-          <t>Double Top, Inside Bar</t>
-        </is>
-      </c>
+      <c r="V92" t="inlineStr"/>
       <c r="W92" t="n">
-        <v>41.2</v>
+        <v>41.4</v>
       </c>
       <c r="X92" t="n">
-        <v>64.3</v>
+        <v>59.6</v>
       </c>
       <c r="Y92" t="inlineStr">
         <is>
@@ -8914,19 +8924,19 @@
       </c>
       <c r="Z92" t="inlineStr">
         <is>
-          <t>trend molto direzionale (ADX 50); RSI scarico (35) — zona di interesse long; pattern: Double Top</t>
+          <t>trend in sviluppo (ADX 23); in zona Fib Fib 78.6 — livello strutturale</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>TEN</t>
+          <t>ENI</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Tenaris</t>
+          <t>Eni</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -8935,52 +8945,52 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>23.68000030517578</v>
+        <v>20.44499969482422</v>
       </c>
       <c r="E93" t="n">
-        <v>-0.837516175123687</v>
+        <v>1.817727950722015</v>
       </c>
       <c r="F93" t="n">
-        <v>-5.619768189864582</v>
+        <v>-0.170897696261807</v>
       </c>
       <c r="G93" t="n">
-        <v>-14.48176291636287</v>
+        <v>-12.8330856477199</v>
       </c>
       <c r="H93" t="n">
-        <v>-6.329115261120021</v>
+        <v>-17.17642237330426</v>
       </c>
       <c r="I93" t="n">
-        <v>31.31686685186551</v>
+        <v>35.36943537656649</v>
       </c>
       <c r="J93" t="n">
-        <v>46.90604926204401</v>
+        <v>49.89199583755958</v>
       </c>
       <c r="K93" t="n">
-        <v>0.08482012712002281</v>
+        <v>0.2357528920674938</v>
       </c>
       <c r="L93" t="n">
-        <v>25.22706973010341</v>
+        <v>21.44480031734003</v>
       </c>
       <c r="M93" t="n">
-        <v>25.50369548459471</v>
+        <v>22.09834073766282</v>
       </c>
       <c r="N93" t="n">
-        <v>22.12538715960772</v>
+        <v>19.75335525708702</v>
       </c>
       <c r="O93" t="n">
-        <v>-0.2220522757085613</v>
+        <v>-0.1333154045249789</v>
       </c>
       <c r="P93" t="n">
-        <v>2.089544080839735</v>
+        <v>15.43339562124327</v>
       </c>
       <c r="Q93" t="n">
-        <v>-97.91045591916027</v>
+        <v>-84.56660437875674</v>
       </c>
       <c r="R93" t="n">
-        <v>-131.3620125677935</v>
+        <v>-84.6928807933466</v>
       </c>
       <c r="S93" t="n">
-        <v>-13.51350974799381</v>
+        <v>-12.68418152712353</v>
       </c>
       <c r="T93" t="inlineStr">
         <is>
@@ -8990,14 +9000,14 @@
       <c r="U93" t="inlineStr"/>
       <c r="V93" t="inlineStr">
         <is>
-          <t>Breakdown 20d, Breakdown 50d, Double Top</t>
+          <t>Double Top, Inside Bar</t>
         </is>
       </c>
       <c r="W93" t="n">
-        <v>41</v>
+        <v>41.2</v>
       </c>
       <c r="X93" t="n">
-        <v>67.8</v>
+        <v>64.3</v>
       </c>
       <c r="Y93" t="inlineStr">
         <is>
@@ -9006,90 +9016,86 @@
       </c>
       <c r="Z93" t="inlineStr">
         <is>
-          <t>trend molto direzionale (ADX 47); RSI scarico (31) — zona di interesse long; pattern: Double Top; breakdown minimi 50g — rottura supporto importante; sul supporto dei 20g (23.61); in zona Fib Fib 78.6 — livello strutturale</t>
+          <t>trend molto direzionale (ADX 50); RSI scarico (35) — zona di interesse long; pattern: Double Top</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>NVDA</t>
+          <t>ADA</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Nvidia</t>
+          <t>Cardano</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Azioni USA</t>
+          <t>Crypto</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>194.8300018310547</v>
+        <v>0.1817999929189682</v>
       </c>
       <c r="E94" t="n">
-        <v>-1.391841266582972</v>
+        <v>12.71412456728864</v>
       </c>
       <c r="F94" t="n">
-        <v>-0.4649042794377389</v>
+        <v>26.54086833087468</v>
       </c>
       <c r="G94" t="n">
-        <v>-12.56171105516419</v>
+        <v>7.041921976134091</v>
       </c>
       <c r="H94" t="n">
-        <v>9.831446249175624</v>
+        <v>-27.30384315579872</v>
       </c>
       <c r="I94" t="n">
-        <v>41.15855680536166</v>
+        <v>59.54583000729774</v>
       </c>
       <c r="J94" t="n">
-        <v>25.99327297142875</v>
+        <v>38.20070968919521</v>
       </c>
       <c r="K94" t="n">
-        <v>0.1815789893158984</v>
+        <v>0.9523051444134021</v>
       </c>
       <c r="L94" t="n">
-        <v>202.75171786607</v>
+        <v>0.1613454276335581</v>
       </c>
       <c r="M94" t="n">
-        <v>204.1884814568574</v>
+        <v>0.1859015018766148</v>
       </c>
       <c r="N94" t="n">
-        <v>188.9462997597143</v>
+        <v>0.2929823810316882</v>
       </c>
       <c r="O94" t="n">
-        <v>-1.000431665214234</v>
+        <v>0.004873355178645476</v>
       </c>
       <c r="P94" t="n">
-        <v>20.79370926679602</v>
+        <v>98.6759191320066</v>
       </c>
       <c r="Q94" t="n">
-        <v>-79.20629073320399</v>
+        <v>-1.324080867993408</v>
       </c>
       <c r="R94" t="n">
-        <v>-57.88591258461099</v>
+        <v>75.41412588923626</v>
       </c>
       <c r="S94" t="n">
-        <v>-9.275901359229477</v>
+        <v>5.850903369464633</v>
       </c>
       <c r="T94" t="inlineStr">
         <is>
-          <t>Range</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="U94" t="inlineStr"/>
-      <c r="V94" t="inlineStr">
-        <is>
-          <t>Outside Bar</t>
-        </is>
-      </c>
+      <c r="V94" t="inlineStr"/>
       <c r="W94" t="n">
-        <v>41</v>
+        <v>41.2</v>
       </c>
       <c r="X94" t="n">
-        <v>59.7</v>
+        <v>63.7</v>
       </c>
       <c r="Y94" t="inlineStr">
         <is>
@@ -9098,86 +9104,90 @@
       </c>
       <c r="Z94" t="inlineStr">
         <is>
-          <t>trend in sviluppo (ADX 26); in zona Fib Fib 61.8 — livello strutturale</t>
+          <t>trend molto direzionale (ADX 38)</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>LINK</t>
+          <t>TEN</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Chainlink</t>
+          <t>Tenaris</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Crypto</t>
+          <t>Azioni IT</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>7.941999912261963</v>
+        <v>23.68000030517578</v>
       </c>
       <c r="E95" t="n">
-        <v>2.58986802247696</v>
+        <v>-0.837516175123687</v>
       </c>
       <c r="F95" t="n">
-        <v>9.394401763543069</v>
+        <v>-5.619768189864582</v>
       </c>
       <c r="G95" t="n">
-        <v>1.098656099438511</v>
+        <v>-14.48176291636287</v>
       </c>
       <c r="H95" t="n">
-        <v>-13.43256717980574</v>
+        <v>-6.329115261120021</v>
       </c>
       <c r="I95" t="n">
-        <v>52.91208799379964</v>
+        <v>31.31686685186551</v>
       </c>
       <c r="J95" t="n">
-        <v>23.38371168862766</v>
+        <v>46.90604926204401</v>
       </c>
       <c r="K95" t="n">
-        <v>0.6583378098447404</v>
+        <v>0.08482012712002281</v>
       </c>
       <c r="L95" t="n">
-        <v>7.687505323849476</v>
+        <v>25.22706973010341</v>
       </c>
       <c r="M95" t="n">
-        <v>8.189932196810894</v>
+        <v>25.50369548459471</v>
       </c>
       <c r="N95" t="n">
-        <v>10.17594321310356</v>
+        <v>22.12538715960772</v>
       </c>
       <c r="O95" t="n">
-        <v>0.07335041443464219</v>
+        <v>-0.2220522757085613</v>
       </c>
       <c r="P95" t="n">
-        <v>82.53126485784188</v>
+        <v>2.089544080839735</v>
       </c>
       <c r="Q95" t="n">
-        <v>-17.46873514215812</v>
+        <v>-97.91045591916027</v>
       </c>
       <c r="R95" t="n">
-        <v>41.66116915245308</v>
+        <v>-131.3620125677935</v>
       </c>
       <c r="S95" t="n">
-        <v>-0.4440024669659537</v>
+        <v>-13.51350974799381</v>
       </c>
       <c r="T95" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Range</t>
         </is>
       </c>
       <c r="U95" t="inlineStr"/>
-      <c r="V95" t="inlineStr"/>
+      <c r="V95" t="inlineStr">
+        <is>
+          <t>Breakdown 20d, Breakdown 50d, Double Top</t>
+        </is>
+      </c>
       <c r="W95" t="n">
         <v>41</v>
       </c>
       <c r="X95" t="n">
-        <v>59.7</v>
+        <v>67.8</v>
       </c>
       <c r="Y95" t="inlineStr">
         <is>
@@ -9186,86 +9196,90 @@
       </c>
       <c r="Z95" t="inlineStr">
         <is>
-          <t>trend in sviluppo (ADX 23); in zona Fib Fib 78.6 — livello strutturale</t>
+          <t>trend molto direzionale (ADX 47); RSI scarico (31) — zona di interesse long; pattern: Double Top; breakdown minimi 50g — rottura supporto importante; sul supporto dei 20g (23.61); in zona Fib Fib 78.6 — livello strutturale</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>XRP</t>
+          <t>NVDA</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>XRP</t>
+          <t>Nvidia</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Crypto</t>
+          <t>Azioni USA</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>1.137699961662292</v>
+        <v>194.8300018310547</v>
       </c>
       <c r="E96" t="n">
-        <v>4.712761607203886</v>
+        <v>-1.391841266582972</v>
       </c>
       <c r="F96" t="n">
-        <v>8.603100423045662</v>
+        <v>-0.4649042794377389</v>
       </c>
       <c r="G96" t="n">
-        <v>0.4982941428640419</v>
+        <v>-12.56171105516419</v>
       </c>
       <c r="H96" t="n">
-        <v>-18.33626460924583</v>
+        <v>9.831446249175624</v>
       </c>
       <c r="I96" t="n">
-        <v>51.92229010703826</v>
+        <v>41.15855680536166</v>
       </c>
       <c r="J96" t="n">
-        <v>21.34413613892223</v>
+        <v>25.99327297142875</v>
       </c>
       <c r="K96" t="n">
-        <v>0.6021630511366372</v>
+        <v>0.1815789893158984</v>
       </c>
       <c r="L96" t="n">
-        <v>1.105973995425375</v>
+        <v>202.75171786607</v>
       </c>
       <c r="M96" t="n">
-        <v>1.18680673959604</v>
+        <v>204.1884814568574</v>
       </c>
       <c r="N96" t="n">
-        <v>1.506304605452055</v>
+        <v>188.9462997597143</v>
       </c>
       <c r="O96" t="n">
-        <v>0.008861550458650613</v>
+        <v>-1.000431665214234</v>
       </c>
       <c r="P96" t="n">
-        <v>83.98833409499245</v>
+        <v>20.79370926679602</v>
       </c>
       <c r="Q96" t="n">
-        <v>-16.01166590500754</v>
+        <v>-79.20629073320399</v>
       </c>
       <c r="R96" t="n">
-        <v>10.29947933087513</v>
+        <v>-57.88591258461099</v>
       </c>
       <c r="S96" t="n">
-        <v>-1.073442796345536</v>
+        <v>-9.275901359229477</v>
       </c>
       <c r="T96" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Range</t>
         </is>
       </c>
       <c r="U96" t="inlineStr"/>
-      <c r="V96" t="inlineStr"/>
+      <c r="V96" t="inlineStr">
+        <is>
+          <t>Outside Bar</t>
+        </is>
+      </c>
       <c r="W96" t="n">
-        <v>40.2</v>
+        <v>41</v>
       </c>
       <c r="X96" t="n">
-        <v>60.4</v>
+        <v>59.7</v>
       </c>
       <c r="Y96" t="inlineStr">
         <is>
@@ -9274,182 +9288,178 @@
       </c>
       <c r="Z96" t="inlineStr">
         <is>
-          <t>trend in sviluppo (ADX 21); in zona Fib Fib 78.6 — livello strutturale</t>
+          <t>trend in sviluppo (ADX 26); in zona Fib Fib 61.8 — livello strutturale</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>AVGO</t>
+          <t>XRP</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Broadcom</t>
+          <t>XRP</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Azioni USA</t>
+          <t>Crypto</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>360.4500122070312</v>
+        <v>1.136399984359741</v>
       </c>
       <c r="E97" t="n">
-        <v>-2.406991990850182</v>
+        <v>4.593113002155214</v>
       </c>
       <c r="F97" t="n">
-        <v>-4.871867007116471</v>
+        <v>8.479006575551473</v>
       </c>
       <c r="G97" t="n">
-        <v>-25.15106698404559</v>
+        <v>0.3834611414284428</v>
       </c>
       <c r="H97" t="n">
-        <v>14.59228300599176</v>
+        <v>-18.42957655969577</v>
       </c>
       <c r="I97" t="n">
-        <v>39.62802974353724</v>
+        <v>51.72834257013492</v>
       </c>
       <c r="J97" t="n">
-        <v>30.17285108714634</v>
+        <v>21.27718461741929</v>
       </c>
       <c r="K97" t="n">
-        <v>0.08801324705436597</v>
+        <v>0.5972432581753909</v>
       </c>
       <c r="L97" t="n">
-        <v>386.498095764574</v>
+        <v>1.105850188063227</v>
       </c>
       <c r="M97" t="n">
-        <v>392.3199534757471</v>
+        <v>1.186755760093979</v>
       </c>
       <c r="N97" t="n">
-        <v>355.0082245455592</v>
+        <v>1.506291670354517</v>
       </c>
       <c r="O97" t="n">
-        <v>-2.45503104873473</v>
+        <v>0.008778588944185844</v>
       </c>
       <c r="P97" t="n">
-        <v>6.906060838008919</v>
+        <v>83.13498895072587</v>
       </c>
       <c r="Q97" t="n">
-        <v>-93.09393916199109</v>
+        <v>-16.86501104927413</v>
       </c>
       <c r="R97" t="n">
-        <v>-52.75529600430337</v>
+        <v>11.11621030352144</v>
       </c>
       <c r="S97" t="n">
-        <v>-24.78559273339948</v>
+        <v>-1.186479874061874</v>
       </c>
       <c r="T97" t="inlineStr">
         <is>
-          <t>Range</t>
+          <t>Bearish</t>
         </is>
       </c>
       <c r="U97" t="inlineStr"/>
-      <c r="V97" t="inlineStr">
-        <is>
-          <t>Breakdown 20d, Breakdown 50d, Outside Bar</t>
-        </is>
-      </c>
+      <c r="V97" t="inlineStr"/>
       <c r="W97" t="n">
-        <v>39.7</v>
+        <v>40.2</v>
       </c>
       <c r="X97" t="n">
-        <v>69.2</v>
+        <v>60.5</v>
       </c>
       <c r="Y97" t="inlineStr">
         <is>
-          <t>SELL</t>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="Z97" t="inlineStr">
         <is>
-          <t>trend molto direzionale (ADX 30); breakdown minimi 50g — rottura supporto importante; sul supporto dei 20g (356.43); in zona Fib Fib 61.8 — livello strutturale</t>
+          <t>trend in sviluppo (ADX 21); in zona Fib Fib 78.6 — livello strutturale</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>BTC</t>
+          <t>AVGO</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Bitcoin</t>
+          <t>Broadcom</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Crypto</t>
+          <t>Azioni USA</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>62185.109375</v>
+        <v>360.4500122070312</v>
       </c>
       <c r="E98" t="n">
-        <v>1.138172188893982</v>
+        <v>-2.406991990850182</v>
       </c>
       <c r="F98" t="n">
-        <v>4.456014223886573</v>
+        <v>-4.871867007116471</v>
       </c>
       <c r="G98" t="n">
-        <v>-2.137270172807515</v>
+        <v>-25.15106698404559</v>
       </c>
       <c r="H98" t="n">
-        <v>-20.94166860016082</v>
+        <v>14.59228300599176</v>
       </c>
       <c r="I98" t="n">
-        <v>46.51349577400001</v>
+        <v>39.62802974353724</v>
       </c>
       <c r="J98" t="n">
-        <v>28.05262053307027</v>
+        <v>30.17285108714634</v>
       </c>
       <c r="K98" t="n">
-        <v>0.4923568117219368</v>
+        <v>0.08801324705436597</v>
       </c>
       <c r="L98" t="n">
-        <v>62093.13549229515</v>
+        <v>386.498095764574</v>
       </c>
       <c r="M98" t="n">
-        <v>65985.40278661886</v>
+        <v>392.3199534757471</v>
       </c>
       <c r="N98" t="n">
-        <v>75890.03884479246</v>
+        <v>355.0082245455592</v>
       </c>
       <c r="O98" t="n">
-        <v>363.6457485535152</v>
+        <v>-2.45503104873473</v>
       </c>
       <c r="P98" t="n">
-        <v>56.91650015331922</v>
+        <v>6.906060838008919</v>
       </c>
       <c r="Q98" t="n">
-        <v>-43.08349984668079</v>
+        <v>-93.09393916199109</v>
       </c>
       <c r="R98" t="n">
-        <v>-14.23601452760458</v>
+        <v>-52.75529600430337</v>
       </c>
       <c r="S98" t="n">
-        <v>-3.471233897888648</v>
+        <v>-24.78559273339948</v>
       </c>
       <c r="T98" t="inlineStr">
         <is>
-          <t>Bearish</t>
+          <t>Range</t>
         </is>
       </c>
       <c r="U98" t="inlineStr"/>
       <c r="V98" t="inlineStr">
         <is>
-          <t>Bear Flag / Consolidation</t>
+          <t>Breakdown 20d, Breakdown 50d, Outside Bar</t>
         </is>
       </c>
       <c r="W98" t="n">
-        <v>39.3</v>
+        <v>39.7</v>
       </c>
       <c r="X98" t="n">
-        <v>69.40000000000001</v>
+        <v>69.2</v>
       </c>
       <c r="Y98" t="inlineStr">
         <is>
@@ -9458,7 +9468,7 @@
       </c>
       <c r="Z98" t="inlineStr">
         <is>
-          <t>trend in sviluppo (ADX 28); pattern: Bear Flag / Consolidation</t>
+          <t>trend molto direzionale (ADX 30); breakdown minimi 50g — rottura supporto importante; sul supporto dei 20g (356.43); in zona Fib Fib 61.8 — livello strutturale</t>
         </is>
       </c>
     </row>
@@ -10399,66 +10409,70 @@
         </is>
       </c>
       <c r="D109" t="n">
-        <v>1.144295692443848</v>
+        <v>1.144033789634705</v>
       </c>
       <c r="E109" t="n">
-        <v>0.5710066102658784</v>
+        <v>0.5479882337015907</v>
       </c>
       <c r="F109" t="n">
-        <v>0.7151907420130277</v>
+        <v>0.6921393650368701</v>
       </c>
       <c r="G109" t="n">
-        <v>-1.433797862359387</v>
+        <v>-1.456357385563811</v>
       </c>
       <c r="H109" t="n">
-        <v>-2.084910798157502</v>
+        <v>-2.107321296675324</v>
       </c>
       <c r="I109" t="n">
-        <v>43.23530794052655</v>
+        <v>42.87896660623295</v>
       </c>
       <c r="J109" t="n">
         <v>45.77819595267555</v>
       </c>
       <c r="K109" t="n">
-        <v>0.4058234016718369</v>
+        <v>0.3985569314885554</v>
       </c>
       <c r="L109" t="n">
-        <v>1.146906324225985</v>
+        <v>1.146881381101304</v>
       </c>
       <c r="M109" t="n">
-        <v>1.155256984870591</v>
+        <v>1.155246714172193</v>
       </c>
       <c r="N109" t="n">
-        <v>1.159072212002603</v>
+        <v>1.159069606004502</v>
       </c>
       <c r="O109" t="n">
-        <v>-5.104572813746655e-08</v>
+        <v>-1.676507115493803e-05</v>
       </c>
       <c r="P109" t="n">
-        <v>40.11236000764796</v>
+        <v>39.21860571075231</v>
       </c>
       <c r="Q109" t="n">
-        <v>-59.88763999235204</v>
+        <v>-60.78139428924769</v>
       </c>
       <c r="R109" t="n">
-        <v>-23.3258052016601</v>
+        <v>-23.9167743004216</v>
       </c>
       <c r="S109" t="n">
-        <v>-1.461269000870102</v>
+        <v>-1.483822236566501</v>
       </c>
       <c r="T109" t="inlineStr">
         <is>
           <t>Trend Bearish</t>
         </is>
       </c>
-      <c r="U109" t="inlineStr"/>
+      <c r="U109" t="inlineStr">
+        <is>
+          <t>Doji</t>
+        </is>
+      </c>
       <c r="V109" t="inlineStr">
         <is>
           <t>Double Top, Inside Bar</t>
         </is>
       </c>
       <c r="W109" t="n">
-        <v>34.5</v>
+        <v>34.4</v>
       </c>
       <c r="X109" t="n">
         <v>68</v>
@@ -10470,7 +10484,7 @@
       </c>
       <c r="Z109" t="inlineStr">
         <is>
-          <t>EMA e SMA allineate al ribasso — struttura bearish solida; trend molto direzionale (ADX 46); pattern: Double Top; sul supporto dei 20g (1.1325); in zona Fib Fib 78.6 — livello strutturale</t>
+          <t>EMA e SMA allineate al ribasso — struttura bearish solida; trend molto direzionale (ADX 46); pattern: Double Top; doji — indecisione del mercato; sul supporto dei 20g (1.1325); in zona Fib Fib 78.6 — livello strutturale</t>
         </is>
       </c>
     </row>
@@ -11061,7 +11075,7 @@
         <v>42.10328459094667</v>
       </c>
       <c r="J116" t="n">
-        <v>41.92978016425015</v>
+        <v>41.82325251481323</v>
       </c>
       <c r="K116" t="n">
         <v>0.4309656950866962</v>
@@ -11085,7 +11099,7 @@
         <v>-51.48469630029851</v>
       </c>
       <c r="R116" t="n">
-        <v>-36.32692057529458</v>
+        <v>-35.52136878030612</v>
       </c>
       <c r="S116" t="n">
         <v>-9.687706273537843</v>
@@ -13179,7 +13193,7 @@
         <v>76.8</v>
       </c>
       <c r="X21" t="n">
-        <v>79</v>
+        <v>78.90000000000001</v>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
@@ -15403,83 +15417,87 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>USDJPY</t>
+          <t>XLU</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>USD/JPY</t>
+          <t>Utilities</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>FX/Macro</t>
+          <t>Settoriali</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>162.5390014648438</v>
+        <v>45.7599983215332</v>
       </c>
       <c r="E46" t="n">
-        <v>0.4536379112437317</v>
+        <v>-0.9523862210825129</v>
       </c>
       <c r="F46" t="n">
-        <v>2.052487665405334</v>
+        <v>3.01665963040203</v>
       </c>
       <c r="G46" t="n">
-        <v>3.670658363273338</v>
+        <v>5.559400074375609</v>
       </c>
       <c r="H46" t="n">
-        <v>13.75989751079645</v>
+        <v>17.01828118450424</v>
       </c>
       <c r="I46" t="n">
-        <v>65.45319266692401</v>
+        <v>53.89785577945819</v>
       </c>
       <c r="J46" t="n">
-        <v>9.945181945279062</v>
+        <v>26.55932112184005</v>
       </c>
       <c r="K46" t="n">
-        <v>0.9788170950808129</v>
+        <v>0.5122357292179918</v>
       </c>
       <c r="L46" t="n">
-        <v>159.0005133284217</v>
+        <v>45.16994268429265</v>
       </c>
       <c r="M46" t="n">
-        <v>155.9758671175692</v>
+        <v>44.07865702561099</v>
       </c>
       <c r="N46" t="n">
-        <v>146.2743544108127</v>
+        <v>38.99714510207828</v>
       </c>
       <c r="O46" t="n">
-        <v>0.1672610832034351</v>
+        <v>-0.09362646135646041</v>
       </c>
       <c r="P46" t="n">
-        <v>96.18696861654195</v>
+        <v>57.97411596023506</v>
       </c>
       <c r="Q46" t="n">
-        <v>-3.813031383458057</v>
+        <v>-42.02588403976493</v>
       </c>
       <c r="R46" t="n">
-        <v>110.0274831366821</v>
+        <v>-4.14939351047682</v>
       </c>
       <c r="S46" t="n">
-        <v>6.359075240754697</v>
+        <v>-1.591401459068376</v>
       </c>
       <c r="T46" t="inlineStr">
         <is>
           <t>Trend Bullish</t>
         </is>
       </c>
-      <c r="U46" t="inlineStr"/>
+      <c r="U46" t="inlineStr">
+        <is>
+          <t>Hammer</t>
+        </is>
+      </c>
       <c r="V46" t="inlineStr">
         <is>
-          <t>Breakout 20d, Breakout 50d, Outside Bar</t>
+          <t>Bear Flag / Consolidation</t>
         </is>
       </c>
       <c r="W46" t="n">
-        <v>68.40000000000001</v>
+        <v>68.2</v>
       </c>
       <c r="X46" t="n">
-        <v>73.59999999999999</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="Y46" t="inlineStr">
         <is>
@@ -15488,94 +15506,86 @@
       </c>
       <c r="Z46" t="inlineStr">
         <is>
-          <t>EMA e SMA allineate al rialzo — struttura bullish solida; mercato laterale — ATR basso (ADX 10); RSI in forza (65) — momentum positivo; breakout massimi 50g — rottura resistenza rilevante; vicino alla resistenza dei 20g (162.84)</t>
+          <t>EMA e SMA allineate al rialzo — struttura bullish solida; trend in sviluppo (ADX 27); pattern: Bear Flag / Consolidation; hammer — segnale di rimbalzo da supporto; in zona Fib Fib 23.6 — livello strutturale</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>XLU</t>
+          <t>RTX</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Utilities</t>
+          <t>RTX Corp</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Settoriali</t>
+          <t>Azioni USA</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>45.7599983215332</v>
+        <v>199.25</v>
       </c>
       <c r="E47" t="n">
-        <v>-0.9523862210825129</v>
+        <v>5.989677205071087</v>
       </c>
       <c r="F47" t="n">
-        <v>3.01665963040203</v>
+        <v>10.90392738426855</v>
       </c>
       <c r="G47" t="n">
-        <v>5.559400074375609</v>
+        <v>0.2969879829933575</v>
       </c>
       <c r="H47" t="n">
-        <v>17.01828118450424</v>
+        <v>59.11994733877801</v>
       </c>
       <c r="I47" t="n">
-        <v>53.89785577945819</v>
+        <v>61.00399934266526</v>
       </c>
       <c r="J47" t="n">
-        <v>26.55932112184005</v>
+        <v>25.90933183830862</v>
       </c>
       <c r="K47" t="n">
-        <v>0.5122357292179918</v>
+        <v>0.6965404128151647</v>
       </c>
       <c r="L47" t="n">
-        <v>45.16994268429265</v>
+        <v>186.3324815388961</v>
       </c>
       <c r="M47" t="n">
-        <v>44.07865702561099</v>
+        <v>176.8514671638395</v>
       </c>
       <c r="N47" t="n">
-        <v>38.99714510207828</v>
+        <v>134.8966729737741</v>
       </c>
       <c r="O47" t="n">
-        <v>-0.09362646135646041</v>
+        <v>-0.04224641687515485</v>
       </c>
       <c r="P47" t="n">
-        <v>57.97411596023506</v>
+        <v>82.33082623823213</v>
       </c>
       <c r="Q47" t="n">
-        <v>-42.02588403976493</v>
+        <v>-17.66917376176787</v>
       </c>
       <c r="R47" t="n">
-        <v>-4.14939351047682</v>
+        <v>31.07253660631657</v>
       </c>
       <c r="S47" t="n">
-        <v>-1.591401459068376</v>
+        <v>-0.4048773210429069</v>
       </c>
       <c r="T47" t="inlineStr">
         <is>
           <t>Trend Bullish</t>
         </is>
       </c>
-      <c r="U47" t="inlineStr">
-        <is>
-          <t>Hammer</t>
-        </is>
-      </c>
-      <c r="V47" t="inlineStr">
-        <is>
-          <t>Bear Flag / Consolidation</t>
-        </is>
-      </c>
+      <c r="U47" t="inlineStr"/>
+      <c r="V47" t="inlineStr"/>
       <c r="W47" t="n">
-        <v>68.2</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="X47" t="n">
-        <v>72.40000000000001</v>
+        <v>66.8</v>
       </c>
       <c r="Y47" t="inlineStr">
         <is>
@@ -15584,73 +15594,73 @@
       </c>
       <c r="Z47" t="inlineStr">
         <is>
-          <t>EMA e SMA allineate al rialzo — struttura bullish solida; trend in sviluppo (ADX 27); pattern: Bear Flag / Consolidation; hammer — segnale di rimbalzo da supporto; in zona Fib Fib 23.6 — livello strutturale</t>
+          <t>EMA e SMA allineate al rialzo — struttura bullish solida; trend in sviluppo (ADX 26); RSI in forza (61) — momentum positivo</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>RTX</t>
+          <t>XLB</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>RTX Corp</t>
+          <t>Materials</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Azioni USA</t>
+          <t>Settoriali</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>199.25</v>
+        <v>52.0099983215332</v>
       </c>
       <c r="E48" t="n">
-        <v>5.989677205071087</v>
+        <v>0.7945733711944403</v>
       </c>
       <c r="F48" t="n">
-        <v>10.90392738426855</v>
+        <v>1.681323108503108</v>
       </c>
       <c r="G48" t="n">
-        <v>0.2969879829933575</v>
+        <v>0.9706853354545242</v>
       </c>
       <c r="H48" t="n">
-        <v>59.11994733877801</v>
+        <v>25.90171046365608</v>
       </c>
       <c r="I48" t="n">
-        <v>61.00399934266526</v>
+        <v>58.74856606186125</v>
       </c>
       <c r="J48" t="n">
-        <v>25.90933183830862</v>
+        <v>18.48568976186834</v>
       </c>
       <c r="K48" t="n">
-        <v>0.6965404128151647</v>
+        <v>0.665200043353758</v>
       </c>
       <c r="L48" t="n">
-        <v>186.3324815388961</v>
+        <v>50.69319614821309</v>
       </c>
       <c r="M48" t="n">
-        <v>176.8514671638395</v>
+        <v>48.63919074658908</v>
       </c>
       <c r="N48" t="n">
-        <v>134.8966729737741</v>
+        <v>44.16581083382468</v>
       </c>
       <c r="O48" t="n">
-        <v>-0.04224641687515485</v>
+        <v>-0.1124608706984098</v>
       </c>
       <c r="P48" t="n">
-        <v>82.33082623823213</v>
+        <v>70.58817944949283</v>
       </c>
       <c r="Q48" t="n">
-        <v>-17.66917376176787</v>
+        <v>-29.41182055050717</v>
       </c>
       <c r="R48" t="n">
-        <v>31.07253660631657</v>
+        <v>14.35640206828334</v>
       </c>
       <c r="S48" t="n">
-        <v>-0.4048773210429069</v>
+        <v>-2.438572534738537</v>
       </c>
       <c r="T48" t="inlineStr">
         <is>
@@ -15658,12 +15668,16 @@
         </is>
       </c>
       <c r="U48" t="inlineStr"/>
-      <c r="V48" t="inlineStr"/>
+      <c r="V48" t="inlineStr">
+        <is>
+          <t>Double Top</t>
+        </is>
+      </c>
       <c r="W48" t="n">
-        <v>67.59999999999999</v>
+        <v>67.5</v>
       </c>
       <c r="X48" t="n">
-        <v>66.8</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="Y48" t="inlineStr">
         <is>
@@ -15672,90 +15686,90 @@
       </c>
       <c r="Z48" t="inlineStr">
         <is>
-          <t>EMA e SMA allineate al rialzo — struttura bullish solida; trend in sviluppo (ADX 26); RSI in forza (61) — momentum positivo</t>
+          <t>EMA e SMA allineate al rialzo — struttura bullish solida; pattern: Double Top; favorito dal quadrante macro (Surriscaldamento)</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>XLB</t>
+          <t>UNH</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Materials</t>
+          <t>UnitedHealth</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Settoriali</t>
+          <t>Azioni USA</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>52.0099983215332</v>
+        <v>425.3599853515625</v>
       </c>
       <c r="E49" t="n">
-        <v>0.7945733711944403</v>
+        <v>-0.5912802847137577</v>
       </c>
       <c r="F49" t="n">
-        <v>1.681323108503108</v>
+        <v>11.84559650868184</v>
       </c>
       <c r="G49" t="n">
-        <v>0.9706853354545242</v>
+        <v>53.75383869002424</v>
       </c>
       <c r="H49" t="n">
-        <v>25.90171046365608</v>
+        <v>1.605190729024852</v>
       </c>
       <c r="I49" t="n">
-        <v>58.74856606186125</v>
+        <v>68.45871892016839</v>
       </c>
       <c r="J49" t="n">
-        <v>18.48568976186834</v>
+        <v>46.29858167286974</v>
       </c>
       <c r="K49" t="n">
-        <v>0.665200043353758</v>
+        <v>0.8448360151512742</v>
       </c>
       <c r="L49" t="n">
-        <v>50.69319614821309</v>
+        <v>367.7965184471579</v>
       </c>
       <c r="M49" t="n">
-        <v>48.63919074658908</v>
+        <v>358.869380319478</v>
       </c>
       <c r="N49" t="n">
-        <v>44.16581083382468</v>
+        <v>413.4087611238132</v>
       </c>
       <c r="O49" t="n">
-        <v>-0.1124608706984098</v>
+        <v>10.24943012717425</v>
       </c>
       <c r="P49" t="n">
-        <v>70.58817944949283</v>
+        <v>97.21084141674864</v>
       </c>
       <c r="Q49" t="n">
-        <v>-29.41182055050717</v>
+        <v>-2.789158583251366</v>
       </c>
       <c r="R49" t="n">
-        <v>14.35640206828334</v>
+        <v>102.1131625874269</v>
       </c>
       <c r="S49" t="n">
-        <v>-2.438572534738537</v>
+        <v>45.07997605974654</v>
       </c>
       <c r="T49" t="inlineStr">
         <is>
-          <t>Trend Bullish</t>
-        </is>
-      </c>
-      <c r="U49" t="inlineStr"/>
-      <c r="V49" t="inlineStr">
-        <is>
-          <t>Double Top</t>
-        </is>
-      </c>
+          <t>Range</t>
+        </is>
+      </c>
+      <c r="U49" t="inlineStr">
+        <is>
+          <t>Doji, Bearish Harami</t>
+        </is>
+      </c>
+      <c r="V49" t="inlineStr"/>
       <c r="W49" t="n">
-        <v>67.5</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="X49" t="n">
-        <v>78.59999999999999</v>
+        <v>73.90000000000001</v>
       </c>
       <c r="Y49" t="inlineStr">
         <is>
@@ -15764,90 +15778,90 @@
       </c>
       <c r="Z49" t="inlineStr">
         <is>
-          <t>EMA e SMA allineate al rialzo — struttura bullish solida; pattern: Double Top; favorito dal quadrante macro (Surriscaldamento)</t>
+          <t>trend molto direzionale (ADX 46); RSI in forza (68) — momentum positivo; doji — indecisione del mercato; vicino alla resistenza dei 20g (430.20); in zona Fib Fib 50.0 — livello strutturale</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>UNH</t>
+          <t>USDJPY</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>UnitedHealth</t>
+          <t>USD/JPY</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Azioni USA</t>
+          <t>FX/Macro</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>425.3599853515625</v>
+        <v>161.3370056152344</v>
       </c>
       <c r="E50" t="n">
-        <v>-0.5912802847137577</v>
+        <v>-0.2892290607401815</v>
       </c>
       <c r="F50" t="n">
-        <v>11.84559650868184</v>
+        <v>1.297797003406531</v>
       </c>
       <c r="G50" t="n">
-        <v>53.75383869002424</v>
+        <v>2.904001130511391</v>
       </c>
       <c r="H50" t="n">
-        <v>1.605190729024852</v>
+        <v>12.91862911719468</v>
       </c>
       <c r="I50" t="n">
-        <v>68.45871892016839</v>
+        <v>61.71018241587444</v>
       </c>
       <c r="J50" t="n">
-        <v>46.29858167286974</v>
+        <v>9.945181945279062</v>
       </c>
       <c r="K50" t="n">
-        <v>0.8448360151512742</v>
+        <v>0.845492167440176</v>
       </c>
       <c r="L50" t="n">
-        <v>367.7965184471579</v>
+        <v>158.8860375332208</v>
       </c>
       <c r="M50" t="n">
-        <v>358.869380319478</v>
+        <v>155.9287300254277</v>
       </c>
       <c r="N50" t="n">
-        <v>413.4087611238132</v>
+        <v>146.2623942531051</v>
       </c>
       <c r="O50" t="n">
-        <v>10.24943012717425</v>
+        <v>0.09055251616285731</v>
       </c>
       <c r="P50" t="n">
-        <v>97.21084141674864</v>
+        <v>80.75500528934685</v>
       </c>
       <c r="Q50" t="n">
-        <v>-2.789158583251366</v>
+        <v>-19.24499471065313</v>
       </c>
       <c r="R50" t="n">
-        <v>102.1131625874269</v>
+        <v>97.79504397761916</v>
       </c>
       <c r="S50" t="n">
-        <v>45.07997605974654</v>
+        <v>5.572536835476449</v>
       </c>
       <c r="T50" t="inlineStr">
         <is>
-          <t>Range</t>
-        </is>
-      </c>
-      <c r="U50" t="inlineStr">
-        <is>
-          <t>Doji, Bearish Harami</t>
-        </is>
-      </c>
-      <c r="V50" t="inlineStr"/>
+          <t>Trend Bullish</t>
+        </is>
+      </c>
+      <c r="U50" t="inlineStr"/>
+      <c r="V50" t="inlineStr">
+        <is>
+          <t>Outside Bar</t>
+        </is>
+      </c>
       <c r="W50" t="n">
         <v>67.40000000000001</v>
       </c>
       <c r="X50" t="n">
-        <v>73.90000000000001</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="Y50" t="inlineStr">
         <is>
@@ -15856,7 +15870,7 @@
       </c>
       <c r="Z50" t="inlineStr">
         <is>
-          <t>trend molto direzionale (ADX 46); RSI in forza (68) — momentum positivo; doji — indecisione del mercato; vicino alla resistenza dei 20g (430.20); in zona Fib Fib 50.0 — livello strutturale</t>
+          <t>EMA e SMA allineate al rialzo — struttura bullish solida; mercato laterale — ATR basso (ADX 10); RSI in forza (62) — momentum positivo; vicino alla resistenza dei 20g (162.84)</t>
         </is>
       </c>
     </row>
@@ -18265,52 +18279,52 @@
         </is>
       </c>
       <c r="D77" t="n">
-        <v>1.33552360534668</v>
+        <v>1.334988713264465</v>
       </c>
       <c r="E77" t="n">
-        <v>1.268753801018629</v>
+        <v>1.228194536946448</v>
       </c>
       <c r="F77" t="n">
-        <v>-0.6637587744611317</v>
+        <v>-0.7035440457178632</v>
       </c>
       <c r="G77" t="n">
-        <v>-1.224677502061344</v>
+        <v>-1.26423811911881</v>
       </c>
       <c r="H77" t="n">
-        <v>0.2176878853985764</v>
+        <v>0.1775495849348996</v>
       </c>
       <c r="I77" t="n">
-        <v>48.37516140821143</v>
+        <v>48.1656696929986</v>
       </c>
       <c r="J77" t="n">
         <v>8.445603970678251</v>
       </c>
       <c r="K77" t="n">
-        <v>0.3871741041073808</v>
+        <v>0.3756807699251772</v>
       </c>
       <c r="L77" t="n">
-        <v>1.33915811988631</v>
+        <v>1.339107177783242</v>
       </c>
       <c r="M77" t="n">
-        <v>1.335778697764153</v>
+        <v>1.335757721604066</v>
       </c>
       <c r="N77" t="n">
-        <v>1.306191940274505</v>
+        <v>1.30618661796523</v>
       </c>
       <c r="O77" t="n">
-        <v>-0.002481013949176832</v>
+        <v>-0.002515149512258438</v>
       </c>
       <c r="P77" t="n">
-        <v>41.22084730378082</v>
+        <v>40.18186280866199</v>
       </c>
       <c r="Q77" t="n">
-        <v>-58.77915269621918</v>
+        <v>-59.81813719133801</v>
       </c>
       <c r="R77" t="n">
-        <v>-74.36476467415059</v>
+        <v>-75.64335678897294</v>
       </c>
       <c r="S77" t="n">
-        <v>-1.945856586858108</v>
+        <v>-1.985128363657873</v>
       </c>
       <c r="T77" t="inlineStr">
         <is>
@@ -18328,7 +18342,7 @@
         </is>
       </c>
       <c r="W77" t="n">
-        <v>49.2</v>
+        <v>49.1</v>
       </c>
       <c r="X77" t="n">
         <v>59</v>
@@ -18361,52 +18375,52 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>1.144295692443848</v>
+        <v>1.144033789634705</v>
       </c>
       <c r="E78" t="n">
-        <v>0.7151907420130277</v>
+        <v>0.6921393650368701</v>
       </c>
       <c r="F78" t="n">
-        <v>-1.801115465822423</v>
+        <v>-1.823590918525819</v>
       </c>
       <c r="G78" t="n">
-        <v>-2.843574889172495</v>
+        <v>-2.865811747032609</v>
       </c>
       <c r="H78" t="n">
-        <v>0.6247846442251737</v>
+        <v>0.6017539591131493</v>
       </c>
       <c r="I78" t="n">
-        <v>41.66360970463042</v>
+        <v>41.51846349056211</v>
       </c>
       <c r="J78" t="n">
         <v>16.14987160359328</v>
       </c>
       <c r="K78" t="n">
-        <v>0.1323338664952269</v>
+        <v>0.1277493789869589</v>
       </c>
       <c r="L78" t="n">
-        <v>1.159674693165957</v>
+        <v>1.159649750041276</v>
       </c>
       <c r="M78" t="n">
-        <v>1.155849568041267</v>
+        <v>1.155839297342869</v>
       </c>
       <c r="N78" t="n">
-        <v>1.123232149170123</v>
+        <v>1.123229543172022</v>
       </c>
       <c r="O78" t="n">
-        <v>-0.003425579577398078</v>
+        <v>-0.003442293602824878</v>
       </c>
       <c r="P78" t="n">
-        <v>22.35794295043309</v>
+        <v>21.85977960183212</v>
       </c>
       <c r="Q78" t="n">
-        <v>-77.64205704956692</v>
+        <v>-78.14022039816788</v>
       </c>
       <c r="R78" t="n">
-        <v>-128.9925082517503</v>
+        <v>-129.4882190153232</v>
       </c>
       <c r="S78" t="n">
-        <v>-3.585072564952696</v>
+        <v>-3.607139711150398</v>
       </c>
       <c r="T78" t="inlineStr">
         <is>
@@ -20761,52 +20775,52 @@
         </is>
       </c>
       <c r="D104" t="n">
-        <v>62185.109375</v>
+        <v>62698.01171875</v>
       </c>
       <c r="E104" t="n">
-        <v>4.456014223886573</v>
+        <v>5.317566692840736</v>
       </c>
       <c r="F104" t="n">
-        <v>-15.48603767174195</v>
+        <v>-14.7889671062411</v>
       </c>
       <c r="G104" t="n">
-        <v>-11.49882392314333</v>
+        <v>-10.76886684675199</v>
       </c>
       <c r="H104" t="n">
-        <v>-33.6726435800817</v>
+        <v>-33.12557601190606</v>
       </c>
       <c r="I104" t="n">
-        <v>36.51220069319579</v>
+        <v>37.15867609873862</v>
       </c>
       <c r="J104" t="n">
         <v>26.69989001937627</v>
       </c>
       <c r="K104" t="n">
-        <v>0.1930743704751001</v>
+        <v>0.2106601213417184</v>
       </c>
       <c r="L104" t="n">
-        <v>71772.30535502026</v>
+        <v>71821.15319728217</v>
       </c>
       <c r="M104" t="n">
-        <v>80724.72043081961</v>
+        <v>80744.83424822157</v>
       </c>
       <c r="N104" t="n">
-        <v>68716.60459259992</v>
+        <v>68721.70809850788</v>
       </c>
       <c r="O104" t="n">
-        <v>-430.3895383852268</v>
+        <v>-397.6573090405054</v>
       </c>
       <c r="P104" t="n">
-        <v>17.71787593868276</v>
+        <v>19.76584440973532</v>
       </c>
       <c r="Q104" t="n">
-        <v>-82.28212406131723</v>
+        <v>-80.23415559026468</v>
       </c>
       <c r="R104" t="n">
-        <v>-70.15854316776078</v>
+        <v>-67.94597034898517</v>
       </c>
       <c r="S104" t="n">
-        <v>-9.599145383791363</v>
+        <v>-8.85351977219926</v>
       </c>
       <c r="T104" t="inlineStr">
         <is>
@@ -20820,10 +20834,10 @@
       </c>
       <c r="V104" t="inlineStr"/>
       <c r="W104" t="n">
-        <v>32.9</v>
+        <v>33.2</v>
       </c>
       <c r="X104" t="n">
-        <v>76</v>
+        <v>75.8</v>
       </c>
       <c r="Y104" t="inlineStr">
         <is>
@@ -20853,52 +20867,52 @@
         </is>
       </c>
       <c r="D105" t="n">
-        <v>1.137699961662292</v>
+        <v>1.136399984359741</v>
       </c>
       <c r="E105" t="n">
-        <v>8.603100423045662</v>
+        <v>8.479006575551473</v>
       </c>
       <c r="F105" t="n">
-        <v>-14.54352776208303</v>
+        <v>-14.64117343142373</v>
       </c>
       <c r="G105" t="n">
-        <v>-20.56194423873603</v>
+        <v>-20.65271304679467</v>
       </c>
       <c r="H105" t="n">
-        <v>-49.57533510353211</v>
+        <v>-49.63295215729239</v>
       </c>
       <c r="I105" t="n">
-        <v>34.41627093345076</v>
+        <v>34.34171722695334</v>
       </c>
       <c r="J105" t="n">
         <v>26.18980210004506</v>
       </c>
       <c r="K105" t="n">
-        <v>0.1276460089856344</v>
+        <v>0.1253839427965282</v>
       </c>
       <c r="L105" t="n">
-        <v>1.367798822056294</v>
+        <v>1.367675014694147</v>
       </c>
       <c r="M105" t="n">
-        <v>1.677431877356326</v>
+        <v>1.677380897854265</v>
       </c>
       <c r="N105" t="n">
-        <v>1.402683725491625</v>
+        <v>1.402670790394087</v>
       </c>
       <c r="O105" t="n">
-        <v>0.00633629539991909</v>
+        <v>0.006253333885454126</v>
       </c>
       <c r="P105" t="n">
-        <v>23.79872954829073</v>
+        <v>23.55692774904588</v>
       </c>
       <c r="Q105" t="n">
-        <v>-76.20127045170926</v>
+        <v>-76.44307225095413</v>
       </c>
       <c r="R105" t="n">
-        <v>-49.37638176788406</v>
+        <v>-49.253050687848</v>
       </c>
       <c r="S105" t="n">
-        <v>-22.8603191546199</v>
+        <v>-22.94846175601239</v>
       </c>
       <c r="T105" t="inlineStr">
         <is>
@@ -21141,52 +21155,52 @@
         </is>
       </c>
       <c r="D108" t="n">
-        <v>82.19000244140625</v>
+        <v>82.76000213623047</v>
       </c>
       <c r="E108" t="n">
-        <v>15.25257485452753</v>
+        <v>16.05186832749732</v>
       </c>
       <c r="F108" t="n">
-        <v>-0.131593548272857</v>
+        <v>0.5610084654653402</v>
       </c>
       <c r="G108" t="n">
-        <v>-5.576601722580632</v>
+        <v>-4.92176163736755</v>
       </c>
       <c r="H108" t="n">
-        <v>-44.5583055999837</v>
+        <v>-44.17380933584164</v>
       </c>
       <c r="I108" t="n">
-        <v>42.73060598087816</v>
+        <v>43.08363708821363</v>
       </c>
       <c r="J108" t="n">
-        <v>36.41395833640571</v>
+        <v>36.3706862521602</v>
       </c>
       <c r="K108" t="n">
-        <v>0.5099045572523577</v>
+        <v>0.5289891301356819</v>
       </c>
       <c r="L108" t="n">
-        <v>87.3097853428178</v>
+        <v>87.36407102803915</v>
       </c>
       <c r="M108" t="n">
-        <v>113.5564705849316</v>
+        <v>113.5788235141404</v>
       </c>
       <c r="N108" t="n">
-        <v>113.8762520988705</v>
+        <v>113.881923737625</v>
       </c>
       <c r="O108" t="n">
-        <v>2.165141293934727</v>
+        <v>2.201517342835194</v>
       </c>
       <c r="P108" t="n">
-        <v>57.52749463248983</v>
+        <v>59.03336039595818</v>
       </c>
       <c r="Q108" t="n">
-        <v>-42.47250536751017</v>
+        <v>-40.96663960404182</v>
       </c>
       <c r="R108" t="n">
-        <v>-11.48866578273564</v>
+        <v>-10.62427310283685</v>
       </c>
       <c r="S108" t="n">
-        <v>-4.435892932228381</v>
+        <v>-3.773141864619978</v>
       </c>
       <c r="T108" t="inlineStr">
         <is>
@@ -21194,16 +21208,12 @@
         </is>
       </c>
       <c r="U108" t="inlineStr"/>
-      <c r="V108" t="inlineStr">
-        <is>
-          <t>Bear Flag / Consolidation</t>
-        </is>
-      </c>
+      <c r="V108" t="inlineStr"/>
       <c r="W108" t="n">
-        <v>30.4</v>
+        <v>30.9</v>
       </c>
       <c r="X108" t="n">
-        <v>72.09999999999999</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="Y108" t="inlineStr">
         <is>
@@ -21212,7 +21222,7 @@
       </c>
       <c r="Z108" t="inlineStr">
         <is>
-          <t>EMA allineate al ribasso (EMA20&lt;EMA50&lt;EMA200); trend molto direzionale (ADX 36); pattern: Bear Flag / Consolidation</t>
+          <t>EMA allineate al ribasso (EMA20&lt;EMA50&lt;EMA200); trend molto direzionale (ADX 36)</t>
         </is>
       </c>
     </row>
@@ -21329,52 +21339,52 @@
         </is>
       </c>
       <c r="D110" t="n">
-        <v>7.941999912261963</v>
+        <v>8.003000259399414</v>
       </c>
       <c r="E110" t="n">
-        <v>9.394401763543069</v>
+        <v>10.23463049134337</v>
       </c>
       <c r="F110" t="n">
-        <v>-12.98053653321117</v>
+        <v>-12.31216363748836</v>
       </c>
       <c r="G110" t="n">
-        <v>-10.08142867014775</v>
+        <v>-9.390788513282978</v>
       </c>
       <c r="H110" t="n">
-        <v>-45.5601584207865</v>
+        <v>-45.14202076388315</v>
       </c>
       <c r="I110" t="n">
-        <v>38.82459066275896</v>
+        <v>39.21677800075066</v>
       </c>
       <c r="J110" t="n">
         <v>33.87766288270218</v>
       </c>
       <c r="K110" t="n">
-        <v>0.2315483507451034</v>
+        <v>0.2490921795993415</v>
       </c>
       <c r="L110" t="n">
-        <v>9.23058057424179</v>
+        <v>9.236390131112023</v>
       </c>
       <c r="M110" t="n">
-        <v>11.66232766525144</v>
+        <v>11.66471983572741</v>
       </c>
       <c r="N110" t="n">
-        <v>13.18343420274407</v>
+        <v>13.18404117137231</v>
       </c>
       <c r="O110" t="n">
-        <v>0.1081229332336178</v>
+        <v>0.1120158328799961</v>
       </c>
       <c r="P110" t="n">
-        <v>23.99992533203909</v>
+        <v>25.59193337128955</v>
       </c>
       <c r="Q110" t="n">
-        <v>-76.00007466796092</v>
+        <v>-74.40806662871046</v>
       </c>
       <c r="R110" t="n">
-        <v>-45.01541943496667</v>
+        <v>-43.34252854319253</v>
       </c>
       <c r="S110" t="n">
-        <v>-9.563690298235572</v>
+        <v>-8.869073533367523</v>
       </c>
       <c r="T110" t="inlineStr">
         <is>
@@ -21392,10 +21402,10 @@
         </is>
       </c>
       <c r="W110" t="n">
-        <v>26.1</v>
+        <v>26.3</v>
       </c>
       <c r="X110" t="n">
-        <v>74.40000000000001</v>
+        <v>74.3</v>
       </c>
       <c r="Y110" t="inlineStr">
         <is>
@@ -21517,52 +21527,52 @@
         </is>
       </c>
       <c r="D112" t="n">
-        <v>1744.18994140625</v>
+        <v>1764.400024414062</v>
       </c>
       <c r="E112" t="n">
-        <v>11.06934727382134</v>
+        <v>12.35631761732514</v>
       </c>
       <c r="F112" t="n">
-        <v>-12.97940518038053</v>
+        <v>-11.97108985706443</v>
       </c>
       <c r="G112" t="n">
-        <v>-16.49651052010192</v>
+        <v>-15.5289482072095</v>
       </c>
       <c r="H112" t="n">
-        <v>-2.714931079208693</v>
+        <v>-1.587680387277313</v>
       </c>
       <c r="I112" t="n">
-        <v>36.6743814927552</v>
+        <v>37.34068155257297</v>
       </c>
       <c r="J112" t="n">
         <v>28.69207376073257</v>
       </c>
       <c r="K112" t="n">
-        <v>0.2131361118332369</v>
+        <v>0.2320177061029869</v>
       </c>
       <c r="L112" t="n">
-        <v>2080.362592396723</v>
+        <v>2082.287362206991</v>
       </c>
       <c r="M112" t="n">
-        <v>2493.835740900546</v>
+        <v>2494.628293175362</v>
       </c>
       <c r="N112" t="n">
-        <v>2504.569311112561</v>
+        <v>2504.770406465872</v>
       </c>
       <c r="O112" t="n">
-        <v>-10.86346668649276</v>
+        <v>-9.573706403373251</v>
       </c>
       <c r="P112" t="n">
-        <v>24.80326961912234</v>
+        <v>26.91227025617528</v>
       </c>
       <c r="Q112" t="n">
-        <v>-75.19673038087765</v>
+        <v>-73.08772974382472</v>
       </c>
       <c r="R112" t="n">
-        <v>-54.13814587912968</v>
+        <v>-52.23476423891217</v>
       </c>
       <c r="S112" t="n">
-        <v>-11.28424102982871</v>
+        <v>-10.25628368967648</v>
       </c>
       <c r="T112" t="inlineStr">
         <is>
@@ -21580,10 +21590,10 @@
         </is>
       </c>
       <c r="W112" t="n">
-        <v>24.4</v>
+        <v>24.7</v>
       </c>
       <c r="X112" t="n">
-        <v>78.59999999999999</v>
+        <v>78.3</v>
       </c>
       <c r="Y112" t="inlineStr">
         <is>
@@ -21655,7 +21665,7 @@
         <v>-86.41186684705525</v>
       </c>
       <c r="R113" t="n">
-        <v>-61.51845920248106</v>
+        <v>-61.38706640133118</v>
       </c>
       <c r="S113" t="n">
         <v>-34.77236939700853</v>
@@ -21885,52 +21895,52 @@
         </is>
       </c>
       <c r="D116" t="n">
-        <v>6.909999847412109</v>
+        <v>6.980000019073486</v>
       </c>
       <c r="E116" t="n">
-        <v>7.2521374647327</v>
+        <v>8.338630691847971</v>
       </c>
       <c r="F116" t="n">
-        <v>-22.87876859096326</v>
+        <v>-22.0975096102715</v>
       </c>
       <c r="G116" t="n">
-        <v>-23.97811818442498</v>
+        <v>-23.20799591313374</v>
       </c>
       <c r="H116" t="n">
-        <v>-68.24447241189071</v>
+        <v>-67.92278030893101</v>
       </c>
       <c r="I116" t="n">
-        <v>34.5078055763031</v>
+        <v>34.93588890719694</v>
       </c>
       <c r="J116" t="n">
-        <v>39.9463597661663</v>
+        <v>39.80619071900788</v>
       </c>
       <c r="K116" t="n">
-        <v>0.1641669434128665</v>
+        <v>0.1766774438436565</v>
       </c>
       <c r="L116" t="n">
-        <v>8.920053469751149</v>
+        <v>8.926720152766519</v>
       </c>
       <c r="M116" t="n">
-        <v>13.31697812218337</v>
+        <v>13.3197232269544</v>
       </c>
       <c r="N116" t="n">
-        <v>21.52542311784752</v>
+        <v>21.52611963696853</v>
       </c>
       <c r="O116" t="n">
-        <v>0.1261100314748882</v>
+        <v>0.130577278897154</v>
       </c>
       <c r="P116" t="n">
-        <v>25.44304846587029</v>
+        <v>26.90717866724965</v>
       </c>
       <c r="Q116" t="n">
-        <v>-74.55695153412971</v>
+        <v>-73.09282133275035</v>
       </c>
       <c r="R116" t="n">
-        <v>-57.04378685423205</v>
+        <v>-55.68633479871686</v>
       </c>
       <c r="S116" t="n">
-        <v>-25.58639664537676</v>
+        <v>-24.83256667087741</v>
       </c>
       <c r="T116" t="inlineStr">
         <is>
@@ -21973,52 +21983,52 @@
         </is>
       </c>
       <c r="D117" t="n">
-        <v>0.1821999996900558</v>
+        <v>0.1817999929189682</v>
       </c>
       <c r="E117" t="n">
-        <v>26.81929080679977</v>
+        <v>26.54086833087468</v>
       </c>
       <c r="F117" t="n">
-        <v>-22.56265625947009</v>
+        <v>-22.73266428298242</v>
       </c>
       <c r="G117" t="n">
-        <v>-32.5841832422288</v>
+        <v>-32.73218973634179</v>
       </c>
       <c r="H117" t="n">
-        <v>-74.11839993781932</v>
+        <v>-74.17522109747389</v>
       </c>
       <c r="I117" t="n">
-        <v>35.46758846501636</v>
+        <v>35.39594934724062</v>
       </c>
       <c r="J117" t="n">
-        <v>37.03940095404671</v>
+        <v>37.03199990200294</v>
       </c>
       <c r="K117" t="n">
-        <v>0.2029452460801919</v>
+        <v>0.2008306792699845</v>
       </c>
       <c r="L117" t="n">
-        <v>0.2438165182632546</v>
+        <v>0.2437784223802939</v>
       </c>
       <c r="M117" t="n">
-        <v>0.3774812121957179</v>
+        <v>0.3774655256556752</v>
       </c>
       <c r="N117" t="n">
-        <v>0.521972399722639</v>
+        <v>0.5219684195557626</v>
       </c>
       <c r="O117" t="n">
-        <v>0.004576000362527408</v>
+        <v>0.004550472864885372</v>
       </c>
       <c r="P117" t="n">
-        <v>29.09857894348664</v>
+        <v>28.83103201513348</v>
       </c>
       <c r="Q117" t="n">
-        <v>-70.90142105651336</v>
+        <v>-71.16896798486651</v>
       </c>
       <c r="R117" t="n">
-        <v>-55.27942496097625</v>
+        <v>-55.34046220607726</v>
       </c>
       <c r="S117" t="n">
-        <v>-35.339627802019</v>
+        <v>-35.48158491916631</v>
       </c>
       <c r="T117" t="inlineStr">
         <is>
@@ -26569,87 +26579,79 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>USDJPY</t>
+          <t>CAC40</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>USD/JPY</t>
+          <t>CAC 40</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>FX/Macro</t>
+          <t>Indici</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>162.5390014648438</v>
+        <v>8508.0703125</v>
       </c>
       <c r="E49" t="n">
-        <v>0.3804260658856196</v>
+        <v>1.23846024593508</v>
       </c>
       <c r="F49" t="n">
-        <v>4.285930367741542</v>
+        <v>-0.8470085656848148</v>
       </c>
       <c r="G49" t="n">
-        <v>6.093187536683131</v>
+        <v>15.75022994563811</v>
       </c>
       <c r="H49" t="n">
-        <v>47.88776410497768</v>
+        <v>31.96596980688293</v>
       </c>
       <c r="I49" t="n">
-        <v>63.65245627563166</v>
+        <v>61.02375772956118</v>
       </c>
       <c r="J49" t="n">
-        <v>27.3767733214772</v>
+        <v>20.25340740770403</v>
       </c>
       <c r="K49" t="n">
-        <v>0.8767279602492908</v>
+        <v>0.9190424072220069</v>
       </c>
       <c r="L49" t="n">
-        <v>154.6315885454979</v>
+        <v>8017.549061549589</v>
       </c>
       <c r="M49" t="n">
-        <v>146.0859737153522</v>
+        <v>7516.814290505398</v>
       </c>
       <c r="N49" t="n">
-        <v>131.9592172792647</v>
+        <v>6414.561488370104</v>
       </c>
       <c r="O49" t="n">
-        <v>0.7122027117553245</v>
+        <v>20.4095634821403</v>
       </c>
       <c r="P49" t="n">
-        <v>98.54505877621682</v>
+        <v>88.2001035003296</v>
       </c>
       <c r="Q49" t="n">
-        <v>-1.454941223783176</v>
+        <v>-11.79989649967039</v>
       </c>
       <c r="R49" t="n">
-        <v>122.5933705657518</v>
+        <v>116.1129330983738</v>
       </c>
       <c r="S49" t="n">
-        <v>7.517830973584338</v>
+        <v>17.59421036132602</v>
       </c>
       <c r="T49" t="inlineStr">
         <is>
           <t>Trend Bullish</t>
         </is>
       </c>
-      <c r="U49" t="inlineStr">
-        <is>
-          <t>Doji</t>
-        </is>
-      </c>
-      <c r="V49" t="inlineStr">
-        <is>
-          <t>Double Top</t>
-        </is>
-      </c>
+      <c r="U49" t="inlineStr"/>
+      <c r="V49" t="inlineStr"/>
       <c r="W49" t="n">
-        <v>76</v>
+        <v>75.8</v>
       </c>
       <c r="X49" t="n">
-        <v>74.3</v>
+        <v>71.8</v>
       </c>
       <c r="Y49" t="inlineStr">
         <is>
@@ -26658,73 +26660,73 @@
       </c>
       <c r="Z49" t="inlineStr">
         <is>
-          <t>EMA e SMA allineate al rialzo — struttura bullish solida; trend in sviluppo (ADX 27); RSI in forza (64) — momentum positivo; pattern: Double Top; doji — indecisione del mercato; vicino alla resistenza dei 20g (162.84)</t>
+          <t>EMA e SMA allineate al rialzo — struttura bullish solida; trend in sviluppo (ADX 20); RSI in forza (61) — momentum positivo</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>CAC40</t>
+          <t>JPM</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>CAC 40</t>
+          <t>JPMorgan Chase</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Indici</t>
+          <t>Azioni USA</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>8508.0703125</v>
+        <v>334.4700012207031</v>
       </c>
       <c r="E50" t="n">
-        <v>1.23846024593508</v>
+        <v>2.181289506411033</v>
       </c>
       <c r="F50" t="n">
-        <v>-0.8470085656848148</v>
+        <v>11.37862631259636</v>
       </c>
       <c r="G50" t="n">
-        <v>15.75022994563811</v>
+        <v>50.71647619881227</v>
       </c>
       <c r="H50" t="n">
-        <v>31.96596980688293</v>
+        <v>103.647095734312</v>
       </c>
       <c r="I50" t="n">
-        <v>61.02375772956118</v>
+        <v>69.45571405011987</v>
       </c>
       <c r="J50" t="n">
-        <v>20.25340740770403</v>
+        <v>42.19688223662929</v>
       </c>
       <c r="K50" t="n">
-        <v>0.9190424072220069</v>
+        <v>0.8674561455249195</v>
       </c>
       <c r="L50" t="n">
-        <v>8017.549061549589</v>
+        <v>288.7435547467752</v>
       </c>
       <c r="M50" t="n">
-        <v>7516.814290505398</v>
+        <v>235.7457515951549</v>
       </c>
       <c r="N50" t="n">
-        <v>6414.561488370104</v>
+        <v>163.1935900089675</v>
       </c>
       <c r="O50" t="n">
-        <v>20.4095634821403</v>
+        <v>-1.406551709366589</v>
       </c>
       <c r="P50" t="n">
-        <v>88.2001035003296</v>
+        <v>89.19893023317276</v>
       </c>
       <c r="Q50" t="n">
-        <v>-11.79989649967039</v>
+        <v>-10.80106976682724</v>
       </c>
       <c r="R50" t="n">
-        <v>116.1129330983738</v>
+        <v>56.90722939838383</v>
       </c>
       <c r="S50" t="n">
-        <v>17.59421036132602</v>
+        <v>33.93801040594171</v>
       </c>
       <c r="T50" t="inlineStr">
         <is>
@@ -26732,12 +26734,16 @@
         </is>
       </c>
       <c r="U50" t="inlineStr"/>
-      <c r="V50" t="inlineStr"/>
+      <c r="V50" t="inlineStr">
+        <is>
+          <t>Inside Bar</t>
+        </is>
+      </c>
       <c r="W50" t="n">
-        <v>75.8</v>
+        <v>75.09999999999999</v>
       </c>
       <c r="X50" t="n">
-        <v>71.8</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="Y50" t="inlineStr">
         <is>
@@ -26746,73 +26752,73 @@
       </c>
       <c r="Z50" t="inlineStr">
         <is>
-          <t>EMA e SMA allineate al rialzo — struttura bullish solida; trend in sviluppo (ADX 20); RSI in forza (61) — momentum positivo</t>
+          <t>EMA e SMA allineate al rialzo — struttura bullish solida; trend molto direzionale (ADX 42); RSI in forza (69) — momentum positivo</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>JPM</t>
+          <t>USDJPY</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>JPMorgan Chase</t>
+          <t>USD/JPY</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Azioni USA</t>
+          <t>FX/Macro</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>334.4700012207031</v>
+        <v>161.3370056152344</v>
       </c>
       <c r="E51" t="n">
-        <v>2.181289506411033</v>
+        <v>-0.361899495523188</v>
       </c>
       <c r="F51" t="n">
-        <v>11.37862631259636</v>
+        <v>3.514723123049635</v>
       </c>
       <c r="G51" t="n">
-        <v>50.71647619881227</v>
+        <v>5.308615403584938</v>
       </c>
       <c r="H51" t="n">
-        <v>103.647095734312</v>
+        <v>46.79411595247169</v>
       </c>
       <c r="I51" t="n">
-        <v>69.45571405011987</v>
+        <v>62.12245903796074</v>
       </c>
       <c r="J51" t="n">
-        <v>42.19688223662929</v>
+        <v>27.3767733214772</v>
       </c>
       <c r="K51" t="n">
-        <v>0.8674561455249195</v>
+        <v>0.8352508240058203</v>
       </c>
       <c r="L51" t="n">
-        <v>288.7435547467752</v>
+        <v>154.517112750297</v>
       </c>
       <c r="M51" t="n">
-        <v>235.7457515951549</v>
+        <v>146.0388366232106</v>
       </c>
       <c r="N51" t="n">
-        <v>163.1935900089675</v>
+        <v>131.9417970495603</v>
       </c>
       <c r="O51" t="n">
-        <v>-1.406551709366589</v>
+        <v>0.6354941447147469</v>
       </c>
       <c r="P51" t="n">
-        <v>89.19893023317276</v>
+        <v>92.65667304038165</v>
       </c>
       <c r="Q51" t="n">
-        <v>-10.80106976682724</v>
+        <v>-7.343326959618355</v>
       </c>
       <c r="R51" t="n">
-        <v>56.90722939838383</v>
+        <v>117.8389047708363</v>
       </c>
       <c r="S51" t="n">
-        <v>33.93801040594171</v>
+        <v>6.722723427552046</v>
       </c>
       <c r="T51" t="inlineStr">
         <is>
@@ -26822,14 +26828,14 @@
       <c r="U51" t="inlineStr"/>
       <c r="V51" t="inlineStr">
         <is>
-          <t>Inside Bar</t>
+          <t>Double Top</t>
         </is>
       </c>
       <c r="W51" t="n">
-        <v>75.09999999999999</v>
+        <v>74.90000000000001</v>
       </c>
       <c r="X51" t="n">
-        <v>68.09999999999999</v>
+        <v>73.3</v>
       </c>
       <c r="Y51" t="inlineStr">
         <is>
@@ -26838,7 +26844,7 @@
       </c>
       <c r="Z51" t="inlineStr">
         <is>
-          <t>EMA e SMA allineate al rialzo — struttura bullish solida; trend molto direzionale (ADX 42); RSI in forza (69) — momentum positivo</t>
+          <t>EMA e SMA allineate al rialzo — struttura bullish solida; trend in sviluppo (ADX 27); RSI in forza (62) — momentum positivo; pattern: Double Top; vicino alla resistenza dei 20g (162.84)</t>
         </is>
       </c>
     </row>
@@ -26925,7 +26931,7 @@
         <v>74.8</v>
       </c>
       <c r="X52" t="n">
-        <v>75.2</v>
+        <v>75.09999999999999</v>
       </c>
       <c r="Y52" t="inlineStr">
         <is>
@@ -28799,52 +28805,52 @@
         </is>
       </c>
       <c r="D73" t="n">
-        <v>1.144295692443848</v>
+        <v>1.144033789634705</v>
       </c>
       <c r="E73" t="n">
-        <v>0.1830923221352032</v>
+        <v>0.1601627301765163</v>
       </c>
       <c r="F73" t="n">
-        <v>-3.05069133732615</v>
+        <v>-3.072880791023225</v>
       </c>
       <c r="G73" t="n">
-        <v>5.37590049069423</v>
+        <v>5.351782385088533</v>
       </c>
       <c r="H73" t="n">
-        <v>-6.128848976654078</v>
+        <v>-6.150333911284922</v>
       </c>
       <c r="I73" t="n">
-        <v>51.97781031781346</v>
+        <v>51.92693916380263</v>
       </c>
       <c r="J73" t="n">
         <v>41.53072495647007</v>
       </c>
       <c r="K73" t="n">
-        <v>0.5296523543221597</v>
+        <v>0.5283683150152734</v>
       </c>
       <c r="L73" t="n">
-        <v>1.142914807816191</v>
+        <v>1.142889864691511</v>
       </c>
       <c r="M73" t="n">
-        <v>1.123285802906454</v>
+        <v>1.123275532208056</v>
       </c>
       <c r="N73" t="n">
-        <v>1.121889090770169</v>
+        <v>1.121885295077283</v>
       </c>
       <c r="O73" t="n">
-        <v>-0.002672617964168154</v>
+        <v>-0.002689331989594954</v>
       </c>
       <c r="P73" t="n">
-        <v>16.83642020104055</v>
+        <v>16.46128338794474</v>
       </c>
       <c r="Q73" t="n">
-        <v>-83.16357979895945</v>
+        <v>-83.53871661205527</v>
       </c>
       <c r="R73" t="n">
-        <v>7.985410014807637</v>
+        <v>7.868568944549224</v>
       </c>
       <c r="S73" t="n">
-        <v>8.330468686342485</v>
+        <v>8.30567434843481</v>
       </c>
       <c r="T73" t="inlineStr">
         <is>
@@ -28858,7 +28864,7 @@
         </is>
       </c>
       <c r="W73" t="n">
-        <v>67.40000000000001</v>
+        <v>67.3</v>
       </c>
       <c r="X73" t="n">
         <v>68.90000000000001</v>
@@ -29163,73 +29169,69 @@
         </is>
       </c>
       <c r="D77" t="n">
-        <v>1.33552360534668</v>
+        <v>1.334988713264465</v>
       </c>
       <c r="E77" t="n">
-        <v>0.7639242474242192</v>
+        <v>0.7235671732122473</v>
       </c>
       <c r="F77" t="n">
-        <v>-1.009653145394662</v>
+        <v>-1.049299882102428</v>
       </c>
       <c r="G77" t="n">
-        <v>3.053006715030793</v>
+        <v>3.011732837789238</v>
       </c>
       <c r="H77" t="n">
-        <v>-5.818873913862211</v>
+        <v>-5.856594504075541</v>
       </c>
       <c r="I77" t="n">
-        <v>52.81686770498219</v>
+        <v>52.73535902336642</v>
       </c>
       <c r="J77" t="n">
         <v>21.76605133944494</v>
       </c>
       <c r="K77" t="n">
-        <v>0.5630040009443538</v>
+        <v>0.5596065079727398</v>
       </c>
       <c r="L77" t="n">
-        <v>1.326449916832296</v>
+        <v>1.326398974729228</v>
       </c>
       <c r="M77" t="n">
-        <v>1.307439479749056</v>
+        <v>1.307418503588969</v>
       </c>
       <c r="N77" t="n">
-        <v>1.332742713552793</v>
+        <v>1.332734961493631</v>
       </c>
       <c r="O77" t="n">
-        <v>-0.002599268211243403</v>
+        <v>-0.002633403774325006</v>
       </c>
       <c r="P77" t="n">
-        <v>41.13960732139747</v>
+        <v>40.49908496806667</v>
       </c>
       <c r="Q77" t="n">
-        <v>-58.86039267860253</v>
+        <v>-59.50091503193333</v>
       </c>
       <c r="R77" t="n">
-        <v>16.83256107768281</v>
+        <v>16.50526806402261</v>
       </c>
       <c r="S77" t="n">
-        <v>5.185840601612202</v>
+        <v>5.143712500638453</v>
       </c>
       <c r="T77" t="inlineStr">
         <is>
           <t>Range</t>
         </is>
       </c>
-      <c r="U77" t="inlineStr">
-        <is>
-          <t>Piercing Pattern</t>
-        </is>
-      </c>
+      <c r="U77" t="inlineStr"/>
       <c r="V77" t="inlineStr">
         <is>
           <t>Inside Bar</t>
         </is>
       </c>
       <c r="W77" t="n">
-        <v>56.8</v>
+        <v>56.5</v>
       </c>
       <c r="X77" t="n">
-        <v>63.5</v>
+        <v>57.5</v>
       </c>
       <c r="Y77" t="inlineStr">
         <is>
@@ -29238,7 +29240,7 @@
       </c>
       <c r="Z77" t="inlineStr">
         <is>
-          <t>trend in sviluppo (ADX 22); segnale candlestick: Piercing Pattern; in zona Fib Fib 23.6 — livello strutturale</t>
+          <t>trend in sviluppo (ADX 22); in zona Fib Fib 23.6 — livello strutturale</t>
         </is>
       </c>
     </row>
@@ -30453,52 +30455,52 @@
         </is>
       </c>
       <c r="D91" t="n">
-        <v>1.137699961662292</v>
+        <v>1.136399984359741</v>
       </c>
       <c r="E91" t="n">
-        <v>9.559622554609803</v>
+        <v>9.434435750182924</v>
       </c>
       <c r="F91" t="n">
-        <v>-17.392098041086</v>
+        <v>-17.48648883055308</v>
       </c>
       <c r="G91" t="n">
-        <v>123.412670497926</v>
+        <v>123.1573910652667</v>
       </c>
       <c r="H91" t="n">
-        <v>8.706033214406972</v>
+        <v>8.58182175216642</v>
       </c>
       <c r="I91" t="n">
-        <v>42.51769061805193</v>
+        <v>42.49271013357987</v>
       </c>
       <c r="J91" t="n">
         <v>38.94285314741881</v>
       </c>
       <c r="K91" t="n">
-        <v>0.1468364540557429</v>
+        <v>0.1463956946851216</v>
       </c>
       <c r="L91" t="n">
-        <v>1.602503007059469</v>
+        <v>1.602379199697321</v>
       </c>
       <c r="M91" t="n">
-        <v>1.326392972800765</v>
+        <v>1.326341993298704</v>
       </c>
       <c r="N91" t="n">
-        <v>1.069001828376019</v>
+        <v>1.068975566208291</v>
       </c>
       <c r="O91" t="n">
-        <v>-0.1900046625387358</v>
+        <v>-0.1900876240532008</v>
       </c>
       <c r="P91" t="n">
-        <v>4.845637591164653</v>
+        <v>4.796404547625306</v>
       </c>
       <c r="Q91" t="n">
-        <v>-95.15436240883535</v>
+        <v>-95.2035954523747</v>
       </c>
       <c r="R91" t="n">
-        <v>-65.87569600819012</v>
+        <v>-65.83751608109058</v>
       </c>
       <c r="S91" t="n">
-        <v>-41.47998196519858</v>
+        <v>-41.54684906351418</v>
       </c>
       <c r="T91" t="inlineStr">
         <is>
@@ -30519,7 +30521,7 @@
         <v>47</v>
       </c>
       <c r="X91" t="n">
-        <v>59.7</v>
+        <v>59.8</v>
       </c>
       <c r="Y91" t="inlineStr">
         <is>
@@ -31021,52 +31023,52 @@
         </is>
       </c>
       <c r="D97" t="n">
-        <v>62185.109375</v>
+        <v>62698.01171875</v>
       </c>
       <c r="E97" t="n">
-        <v>6.192487419842263</v>
+        <v>7.068362307475362</v>
       </c>
       <c r="F97" t="n">
-        <v>-7.180667648537053</v>
+        <v>-6.415094449633663</v>
       </c>
       <c r="G97" t="n">
-        <v>-11.43638351033386</v>
+        <v>-10.70591142585783</v>
       </c>
       <c r="H97" t="n">
-        <v>66.56938933335259</v>
+        <v>67.9432524823403</v>
       </c>
       <c r="I97" t="n">
-        <v>42.78939649109316</v>
+        <v>43.06916592609986</v>
       </c>
       <c r="J97" t="n">
         <v>30.22243585581547</v>
       </c>
       <c r="K97" t="n">
-        <v>0.1258709896313172</v>
+        <v>0.1318602066049668</v>
       </c>
       <c r="L97" t="n">
-        <v>78121.89513842379</v>
+        <v>78170.7429806857</v>
       </c>
       <c r="M97" t="n">
-        <v>65927.10927732389</v>
+        <v>65947.22309472585</v>
       </c>
       <c r="N97" t="n">
-        <v>49823.73779601275</v>
+        <v>49834.09945952285</v>
       </c>
       <c r="O97" t="n">
-        <v>-6158.88653482241</v>
+        <v>-6126.154305477688</v>
       </c>
       <c r="P97" t="n">
-        <v>6.482577061209667</v>
+        <v>7.231883212718533</v>
       </c>
       <c r="Q97" t="n">
-        <v>-93.51742293879033</v>
+        <v>-92.76811678728147</v>
       </c>
       <c r="R97" t="n">
-        <v>-77.34408143289298</v>
+        <v>-76.55609529156209</v>
       </c>
       <c r="S97" t="n">
-        <v>-35.52543404755701</v>
+        <v>-34.99364828209581</v>
       </c>
       <c r="T97" t="inlineStr">
         <is>
@@ -31080,10 +31082,10 @@
       </c>
       <c r="V97" t="inlineStr"/>
       <c r="W97" t="n">
-        <v>42.9</v>
+        <v>43</v>
       </c>
       <c r="X97" t="n">
-        <v>66.40000000000001</v>
+        <v>66.3</v>
       </c>
       <c r="Y97" t="inlineStr">
         <is>
@@ -31293,73 +31295,65 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>82.19000244140625</v>
+        <v>82.76000213623047</v>
       </c>
       <c r="E100" t="n">
-        <v>11.78768325366171</v>
+        <v>12.56294719631848</v>
       </c>
       <c r="F100" t="n">
-        <v>-2.579443525455316</v>
+        <v>-1.90381770953344</v>
       </c>
       <c r="G100" t="n">
-        <v>-51.20227630739282</v>
+        <v>-50.86385695240214</v>
       </c>
       <c r="H100" t="n">
-        <v>150.4552237921127</v>
+        <v>152.1921674213626</v>
       </c>
       <c r="I100" t="n">
-        <v>42.3298994151066</v>
+        <v>42.45386201414408</v>
       </c>
       <c r="J100" t="n">
-        <v>26.05158966061029</v>
+        <v>26.04985559407729</v>
       </c>
       <c r="K100" t="n">
-        <v>0.2113270022384859</v>
+        <v>0.2138918221319564</v>
       </c>
       <c r="L100" t="n">
-        <v>118.4412691095029</v>
+        <v>118.4955547947242</v>
       </c>
       <c r="M100" t="n">
-        <v>115.8234781836664</v>
+        <v>115.8527089372471</v>
       </c>
       <c r="N100" t="n">
-        <v>93.75345065545287</v>
+        <v>93.76865064731484</v>
       </c>
       <c r="O100" t="n">
-        <v>-12.41554161225741</v>
+        <v>-12.37916556335694</v>
       </c>
       <c r="P100" t="n">
-        <v>11.29451663134818</v>
+        <v>11.59016701589431</v>
       </c>
       <c r="Q100" t="n">
-        <v>-88.70548336865183</v>
+        <v>-88.40983298410569</v>
       </c>
       <c r="R100" t="n">
-        <v>-89.59679363329131</v>
+        <v>-89.22438440900396</v>
       </c>
       <c r="S100" t="n">
-        <v>-56.57399519189412</v>
+        <v>-56.2728294934784</v>
       </c>
       <c r="T100" t="inlineStr">
         <is>
           <t>Range</t>
         </is>
       </c>
-      <c r="U100" t="inlineStr">
-        <is>
-          <t>Bullish Harami</t>
-        </is>
-      </c>
-      <c r="V100" t="inlineStr">
-        <is>
-          <t>Inside Bar</t>
-        </is>
-      </c>
+      <c r="U100" t="inlineStr"/>
+      <c r="V100" t="inlineStr"/>
       <c r="W100" t="n">
-        <v>38.2</v>
+        <v>37.9</v>
       </c>
       <c r="X100" t="n">
-        <v>70.7</v>
+        <v>64.7</v>
       </c>
       <c r="Y100" t="inlineStr">
         <is>
@@ -31368,7 +31362,7 @@
       </c>
       <c r="Z100" t="inlineStr">
         <is>
-          <t>trend in sviluppo (ADX 26); segnale candlestick: Bullish Harami</t>
+          <t>trend in sviluppo (ADX 26)</t>
         </is>
       </c>
     </row>
@@ -31669,52 +31663,52 @@
         </is>
       </c>
       <c r="D104" t="n">
-        <v>0.1821999996900558</v>
+        <v>0.1817999929189682</v>
       </c>
       <c r="E104" t="n">
-        <v>26.38559444844348</v>
+        <v>26.10812412114758</v>
       </c>
       <c r="F104" t="n">
-        <v>-35.30173933224128</v>
+        <v>-35.44377963075237</v>
       </c>
       <c r="G104" t="n">
-        <v>-46.70099120214918</v>
+        <v>-46.81800527705406</v>
       </c>
       <c r="H104" t="n">
-        <v>-89.54542657841273</v>
+        <v>-89.56837882959047</v>
       </c>
       <c r="I104" t="n">
-        <v>38.21413802174465</v>
+        <v>38.19360571134847</v>
       </c>
       <c r="J104" t="n">
         <v>30.70524078487225</v>
       </c>
       <c r="K104" t="n">
-        <v>0.1711761778033555</v>
+        <v>0.1708398670396497</v>
       </c>
       <c r="L104" t="n">
-        <v>0.4087730401324859</v>
+        <v>0.4087349442495252</v>
       </c>
       <c r="M104" t="n">
-        <v>0.4950607792438936</v>
+        <v>0.4950450927038509</v>
       </c>
       <c r="N104" t="n">
-        <v>0.4935733238240342</v>
+        <v>0.4935652428791638</v>
       </c>
       <c r="O104" t="n">
-        <v>-0.04804490588325543</v>
+        <v>-0.04807043338089746</v>
       </c>
       <c r="P104" t="n">
-        <v>4.956315205493219</v>
+        <v>4.91074435779804</v>
       </c>
       <c r="Q104" t="n">
-        <v>-95.04368479450677</v>
+        <v>-95.08925564220196</v>
       </c>
       <c r="R104" t="n">
-        <v>-98.6930297432328</v>
+        <v>-98.71115876479834</v>
       </c>
       <c r="S104" t="n">
-        <v>-83.11308581840255</v>
+        <v>-83.1501598031825</v>
       </c>
       <c r="T104" t="inlineStr">
         <is>
@@ -31728,7 +31722,7 @@
         </is>
       </c>
       <c r="W104" t="n">
-        <v>34.8</v>
+        <v>34.7</v>
       </c>
       <c r="X104" t="n">
         <v>67.90000000000001</v>
@@ -31761,52 +31755,52 @@
         </is>
       </c>
       <c r="D105" t="n">
-        <v>1744.18994140625</v>
+        <v>1764.400024414062</v>
       </c>
       <c r="E105" t="n">
-        <v>11.12435488761849</v>
+        <v>12.4119626092051</v>
       </c>
       <c r="F105" t="n">
-        <v>-11.2394359092675</v>
+        <v>-10.21095940822332</v>
       </c>
       <c r="G105" t="n">
-        <v>-30.67054553867288</v>
+        <v>-29.86721902228436</v>
       </c>
       <c r="H105" t="n">
-        <v>-35.75598251000682</v>
+        <v>-35.01158140127132</v>
       </c>
       <c r="I105" t="n">
-        <v>41.95918237642785</v>
+        <v>42.18019856256061</v>
       </c>
       <c r="J105" t="n">
         <v>13.65760872685721</v>
       </c>
       <c r="K105" t="n">
-        <v>0.2257813616949586</v>
+        <v>0.2310347574141265</v>
       </c>
       <c r="L105" t="n">
-        <v>2497.349085003687</v>
+        <v>2499.273854813955</v>
       </c>
       <c r="M105" t="n">
-        <v>2412.217813695128</v>
+        <v>2413.010365969944</v>
       </c>
       <c r="N105" t="n">
-        <v>2011.519027523597</v>
+        <v>2011.927312028805</v>
       </c>
       <c r="O105" t="n">
-        <v>-191.6977309180085</v>
+        <v>-190.407970634889</v>
       </c>
       <c r="P105" t="n">
-        <v>6.894938806859921</v>
+        <v>7.481209510658493</v>
       </c>
       <c r="Q105" t="n">
-        <v>-93.10506119314007</v>
+        <v>-92.51879048934151</v>
       </c>
       <c r="R105" t="n">
-        <v>-103.4060933895197</v>
+        <v>-102.2407203766606</v>
       </c>
       <c r="S105" t="n">
-        <v>-52.9323087044635</v>
+        <v>-52.3869312054384</v>
       </c>
       <c r="T105" t="inlineStr">
         <is>
@@ -31857,52 +31851,52 @@
         </is>
       </c>
       <c r="D106" t="n">
-        <v>7.941999912261963</v>
+        <v>8.003000259399414</v>
       </c>
       <c r="E106" t="n">
-        <v>10.46732781592985</v>
+        <v>11.31579739771798</v>
       </c>
       <c r="F106" t="n">
-        <v>-10.19627374175646</v>
+        <v>-9.506515678736127</v>
       </c>
       <c r="G106" t="n">
-        <v>-30.46901698099864</v>
+        <v>-29.93496836001858</v>
       </c>
       <c r="H106" t="n">
-        <v>-75.24976580601368</v>
+        <v>-75.05966597042499</v>
       </c>
       <c r="I106" t="n">
-        <v>41.42164839750207</v>
+        <v>41.54577117058346</v>
       </c>
       <c r="J106" t="n">
         <v>21.04094275559561</v>
       </c>
       <c r="K106" t="n">
-        <v>0.2118689467678845</v>
+        <v>0.2144250374371305</v>
       </c>
       <c r="L106" t="n">
-        <v>12.05216035266497</v>
+        <v>12.0579699095352</v>
       </c>
       <c r="M106" t="n">
-        <v>12.59276218819566</v>
+        <v>12.59515435867164</v>
       </c>
       <c r="N106" t="n">
-        <v>10.85979563288956</v>
+        <v>10.86102796313476</v>
       </c>
       <c r="O106" t="n">
-        <v>-1.00399346567364</v>
+        <v>-1.000100566027261</v>
       </c>
       <c r="P106" t="n">
-        <v>4.439734487794018</v>
+        <v>4.734239278909761</v>
       </c>
       <c r="Q106" t="n">
-        <v>-95.56026551220599</v>
+        <v>-95.26576072109025</v>
       </c>
       <c r="R106" t="n">
-        <v>-100.9548791744951</v>
+        <v>-100.3329189411848</v>
       </c>
       <c r="S106" t="n">
-        <v>-58.24979573068355</v>
+        <v>-57.92912373601937</v>
       </c>
       <c r="T106" t="inlineStr">
         <is>
@@ -32107,7 +32101,7 @@
         <v>31.7</v>
       </c>
       <c r="X108" t="n">
-        <v>74.40000000000001</v>
+        <v>74.3</v>
       </c>
       <c r="Y108" t="inlineStr">
         <is>
@@ -32789,52 +32783,52 @@
         </is>
       </c>
       <c r="D116" t="n">
-        <v>6.909999847412109</v>
+        <v>6.980000019073486</v>
       </c>
       <c r="E116" t="n">
-        <v>5.874467552541174</v>
+        <v>6.947004609978347</v>
       </c>
       <c r="F116" t="n">
-        <v>-24.60077954339602</v>
+        <v>-23.83696500046619</v>
       </c>
       <c r="G116" t="n">
-        <v>-72.37892013969314</v>
+        <v>-72.09911111300869</v>
       </c>
       <c r="H116" t="n">
-        <v>-61.95210508307181</v>
+        <v>-61.56666959329586</v>
       </c>
       <c r="I116" t="n">
-        <v>39.12523736802475</v>
+        <v>39.20413232289025</v>
       </c>
       <c r="J116" t="n">
         <v>16.96239899989589</v>
       </c>
       <c r="K116" t="n">
-        <v>0.2005941954561051</v>
+        <v>0.2023200386775247</v>
       </c>
       <c r="L116" t="n">
-        <v>15.6740075702936</v>
+        <v>15.68067425330896</v>
       </c>
       <c r="M116" t="n">
-        <v>19.48648044217415</v>
+        <v>19.49026423523693</v>
       </c>
       <c r="N116" t="n">
-        <v>20.89342913179688</v>
+        <v>20.89540096761833</v>
       </c>
       <c r="O116" t="n">
-        <v>-1.13593119586194</v>
+        <v>-1.131463948439676</v>
       </c>
       <c r="P116" t="n">
-        <v>4.025704446241574</v>
+        <v>4.257365187267792</v>
       </c>
       <c r="Q116" t="n">
-        <v>-95.97429555375842</v>
+        <v>-95.74263481273221</v>
       </c>
       <c r="R116" t="n">
-        <v>-76.81782086509412</v>
+        <v>-76.53101202182465</v>
       </c>
       <c r="S116" t="n">
-        <v>-79.91141533187478</v>
+        <v>-79.70791252344425</v>
       </c>
       <c r="T116" t="inlineStr">
         <is>
@@ -32923,7 +32917,7 @@
         <v>-97.88563390090216</v>
       </c>
       <c r="R117" t="n">
-        <v>-73.14157403768723</v>
+        <v>-73.11694337034973</v>
       </c>
       <c r="S117" t="n">
         <v>-85.99322067411389</v>
@@ -33210,7 +33204,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>03/07/2026 19:23:31</t>
+          <t>03/07/2026 21:07:22</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -33423,10 +33417,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>64.8397735969493</v>
+        <v>64.83242238611403</v>
       </c>
       <c r="C2" t="n">
-        <v>0.1217081405461109</v>
+        <v>0.1214140921127003</v>
       </c>
       <c r="D2" t="n">
         <v>55.17241379310344</v>
@@ -33823,17 +33817,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>SOXX</t>
+          <t>XLK</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>0.9340000000000001</v>
+        <v>0.947</v>
       </c>
       <c r="D18" t="n">
         <v>0.909</v>
       </c>
       <c r="E18" t="n">
-        <v>0.877</v>
+        <v>0.888</v>
       </c>
     </row>
     <row r="19">
@@ -33844,17 +33838,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>XLK</t>
+          <t>SOXX</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>0.947</v>
+        <v>0.9340000000000001</v>
       </c>
       <c r="D19" t="n">
         <v>0.909</v>
       </c>
       <c r="E19" t="n">
-        <v>0.888</v>
+        <v>0.877</v>
       </c>
     </row>
     <row r="20">
@@ -33881,22 +33875,22 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>RUSSELL</t>
+          <t>XRP</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>MSCIWORLD</t>
+          <t>LINK</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>0.931</v>
+        <v>0.926</v>
       </c>
       <c r="D21" t="n">
-        <v>0.904</v>
+        <v>0.908</v>
       </c>
       <c r="E21" t="n">
-        <v>0.916</v>
+        <v>0.907</v>
       </c>
     </row>
   </sheetData>

</xml_diff>